<commit_message>
Pauta audiências: 2026-06-17 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30210"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -759,7 +759,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1232,12 +1232,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE714E1C-EF1E-4220-BC30-903B22BAFB26}">
   <dimension ref="A1:R32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="13.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="16.149999999999999" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1293,7 +1293,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A2" s="4">
         <v>104967</v>
       </c>
@@ -1349,7 +1349,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A3" s="4">
         <v>104484</v>
       </c>
@@ -1405,7 +1405,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A4" s="4">
         <v>100254</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A5" s="4">
         <v>102033</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A6" s="4">
         <v>102059</v>
       </c>
@@ -1573,7 +1573,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A7" s="4">
         <v>104861</v>
       </c>
@@ -1629,7 +1629,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A8" s="4">
         <v>104039</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A9" s="4">
         <v>104661</v>
       </c>
@@ -1741,7 +1741,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A10" s="4">
         <v>105186</v>
       </c>
@@ -1797,7 +1797,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A11" s="4">
         <v>99425</v>
       </c>
@@ -1853,7 +1853,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A12" s="4">
         <v>105064</v>
       </c>
@@ -1909,7 +1909,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A13" s="4">
         <v>102178</v>
       </c>
@@ -1965,7 +1965,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A14" s="4">
         <v>104641</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A15" s="4">
         <v>99426</v>
       </c>
@@ -2077,7 +2077,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A16" s="4">
         <v>103743</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A17" s="4">
         <v>94994</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A18" s="4">
         <v>105060</v>
       </c>
@@ -2245,7 +2245,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A19" s="4">
         <v>104740</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A20" s="4">
         <v>103894</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A21" s="4">
         <v>104554</v>
       </c>
@@ -2413,7 +2413,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A22" s="4">
         <v>104395</v>
       </c>
@@ -2469,7 +2469,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A23" s="4">
         <v>66615</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A24" s="4">
         <v>99056</v>
       </c>
@@ -2581,7 +2581,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A25" s="4">
         <v>102819</v>
       </c>
@@ -2637,7 +2637,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A26" s="4">
         <v>104638</v>
       </c>
@@ -2693,7 +2693,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A27" s="4">
         <v>103586</v>
       </c>
@@ -2749,7 +2749,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A28" s="4">
         <v>98536</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A29" s="4">
         <v>103976</v>
       </c>
@@ -2861,7 +2861,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A30" s="4">
         <v>104533</v>
       </c>
@@ -2917,7 +2917,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A31" s="4">
         <v>103526</v>
       </c>
@@ -2973,7 +2973,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" ht="18" customHeight="1" thickBot="1">
       <c r="A32" s="4">
         <v>104294</v>
       </c>

</xml_diff>

<commit_message>
Audiências: sync 2026-06-30 — 424 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -6875,7 +6875,7 @@
         <v>46199</v>
       </c>
       <c r="B95" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D95" t="s">
         <v>55</v>
@@ -6907,7 +6907,7 @@
         <v>46199</v>
       </c>
       <c r="B96" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D96" t="s">
         <v>55</v>
@@ -6939,7 +6939,7 @@
         <v>46199</v>
       </c>
       <c r="B97" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D97" t="s">
         <v>56</v>
@@ -6971,7 +6971,7 @@
         <v>46199</v>
       </c>
       <c r="B98" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C98" t="s">
         <v>43</v>
@@ -7006,7 +7006,7 @@
         <v>46199</v>
       </c>
       <c r="B99" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C99" t="s">
         <v>18</v>
@@ -7041,7 +7041,7 @@
         <v>46199</v>
       </c>
       <c r="B100" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C100" t="s">
         <v>39</v>
@@ -7076,7 +7076,7 @@
         <v>46199</v>
       </c>
       <c r="B101" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D101" t="s">
         <v>58</v>
@@ -7108,7 +7108,7 @@
         <v>46199</v>
       </c>
       <c r="B102" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C102" t="s">
         <v>24</v>
@@ -7143,7 +7143,7 @@
         <v>46199</v>
       </c>
       <c r="B103" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C103" t="s">
         <v>44</v>
@@ -7178,7 +7178,7 @@
         <v>46199</v>
       </c>
       <c r="B104" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D104" t="s">
         <v>61</v>
@@ -7210,7 +7210,7 @@
         <v>46199</v>
       </c>
       <c r="B105" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D105" t="s">
         <v>55</v>
@@ -7242,7 +7242,7 @@
         <v>46199</v>
       </c>
       <c r="B106" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D106" t="s">
         <v>58</v>
@@ -7274,7 +7274,7 @@
         <v>46199</v>
       </c>
       <c r="B107" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C107" t="s">
         <v>45</v>
@@ -7309,7 +7309,7 @@
         <v>46199</v>
       </c>
       <c r="B108" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D108" t="s">
         <v>57</v>
@@ -7341,7 +7341,7 @@
         <v>46199</v>
       </c>
       <c r="B109" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D109" t="s">
         <v>55</v>
@@ -7373,7 +7373,7 @@
         <v>46199</v>
       </c>
       <c r="B110" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D110" t="s">
         <v>55</v>
@@ -7405,7 +7405,7 @@
         <v>46199</v>
       </c>
       <c r="B111" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C111" t="s">
         <v>37</v>
@@ -7440,7 +7440,7 @@
         <v>46199</v>
       </c>
       <c r="B112" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C112" t="s">
         <v>37</v>
@@ -7475,7 +7475,7 @@
         <v>46199</v>
       </c>
       <c r="B113" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D113" t="s">
         <v>55</v>
@@ -7507,7 +7507,7 @@
         <v>46199</v>
       </c>
       <c r="B114" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C114" t="s">
         <v>37</v>
@@ -7542,7 +7542,7 @@
         <v>46199</v>
       </c>
       <c r="B115" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D115" t="s">
         <v>58</v>
@@ -7574,7 +7574,7 @@
         <v>46199</v>
       </c>
       <c r="B116" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D116" t="s">
         <v>56</v>
@@ -7606,7 +7606,7 @@
         <v>46199</v>
       </c>
       <c r="B117" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D117" t="s">
         <v>56</v>
@@ -7638,7 +7638,7 @@
         <v>46199</v>
       </c>
       <c r="B118" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D118" t="s">
         <v>56</v>
@@ -7670,7 +7670,7 @@
         <v>46199</v>
       </c>
       <c r="B119" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D119" t="s">
         <v>61</v>
@@ -7702,7 +7702,7 @@
         <v>46199</v>
       </c>
       <c r="B120" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D120" t="s">
         <v>62</v>
@@ -7734,7 +7734,7 @@
         <v>46199</v>
       </c>
       <c r="B121" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D121" t="s">
         <v>56</v>
@@ -7766,7 +7766,7 @@
         <v>46199</v>
       </c>
       <c r="B122" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D122" t="s">
         <v>56</v>
@@ -7798,7 +7798,7 @@
         <v>46199</v>
       </c>
       <c r="B123" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D123" t="s">
         <v>55</v>
@@ -7830,7 +7830,7 @@
         <v>46199</v>
       </c>
       <c r="B124" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D124" t="s">
         <v>56</v>
@@ -7862,7 +7862,7 @@
         <v>46199</v>
       </c>
       <c r="B125" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D125" t="s">
         <v>55</v>
@@ -7894,7 +7894,7 @@
         <v>46199</v>
       </c>
       <c r="B126" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D126" t="s">
         <v>55</v>
@@ -7926,7 +7926,7 @@
         <v>46199</v>
       </c>
       <c r="B127" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D127" t="s">
         <v>56</v>
@@ -7958,7 +7958,7 @@
         <v>46199</v>
       </c>
       <c r="B128" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D128" t="s">
         <v>57</v>
@@ -7990,7 +7990,7 @@
         <v>46199</v>
       </c>
       <c r="B129" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D129" t="s">
         <v>56</v>
@@ -8022,7 +8022,7 @@
         <v>46202</v>
       </c>
       <c r="B130" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C130" t="s">
         <v>46</v>
@@ -8057,7 +8057,7 @@
         <v>46202</v>
       </c>
       <c r="B131" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D131" t="s">
         <v>63</v>
@@ -8089,7 +8089,7 @@
         <v>46202</v>
       </c>
       <c r="B132" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D132" t="s">
         <v>56</v>
@@ -8121,7 +8121,7 @@
         <v>46202</v>
       </c>
       <c r="B133" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D133" t="s">
         <v>58</v>
@@ -8153,7 +8153,7 @@
         <v>46202</v>
       </c>
       <c r="B134" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C134" t="s">
         <v>29</v>
@@ -8188,7 +8188,7 @@
         <v>46202</v>
       </c>
       <c r="B135" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D135" t="s">
         <v>58</v>
@@ -8220,7 +8220,7 @@
         <v>46202</v>
       </c>
       <c r="B136" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C136" t="s">
         <v>47</v>
@@ -8255,7 +8255,7 @@
         <v>46202</v>
       </c>
       <c r="B137" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C137" t="s">
         <v>36</v>
@@ -8290,7 +8290,7 @@
         <v>46202</v>
       </c>
       <c r="B138" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C138" t="s">
         <v>48</v>
@@ -8325,7 +8325,7 @@
         <v>46202</v>
       </c>
       <c r="B139" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C139" t="s">
         <v>16</v>
@@ -8360,7 +8360,7 @@
         <v>46202</v>
       </c>
       <c r="B140" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C140" t="s">
         <v>27</v>
@@ -8395,7 +8395,7 @@
         <v>46202</v>
       </c>
       <c r="B141" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C141" t="s">
         <v>37</v>
@@ -8430,7 +8430,7 @@
         <v>46202</v>
       </c>
       <c r="B142" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C142" t="s">
         <v>33</v>
@@ -8465,7 +8465,7 @@
         <v>46202</v>
       </c>
       <c r="B143" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C143" t="s">
         <v>49</v>
@@ -8500,7 +8500,7 @@
         <v>46202</v>
       </c>
       <c r="B144" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C144" t="s">
         <v>18</v>
@@ -8535,7 +8535,7 @@
         <v>46202</v>
       </c>
       <c r="B145" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D145" t="s">
         <v>55</v>
@@ -8567,7 +8567,7 @@
         <v>46202</v>
       </c>
       <c r="B146" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C146" t="s">
         <v>32</v>
@@ -8602,7 +8602,7 @@
         <v>46202</v>
       </c>
       <c r="B147" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C147" t="s">
         <v>40</v>
@@ -8637,7 +8637,7 @@
         <v>46202</v>
       </c>
       <c r="B148" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C148" t="s">
         <v>25</v>
@@ -8672,7 +8672,7 @@
         <v>46202</v>
       </c>
       <c r="B149" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C149" t="s">
         <v>38</v>
@@ -8707,7 +8707,7 @@
         <v>46202</v>
       </c>
       <c r="B150" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D150" t="s">
         <v>55</v>
@@ -8739,7 +8739,7 @@
         <v>46202</v>
       </c>
       <c r="B151" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D151" t="s">
         <v>55</v>
@@ -8771,7 +8771,7 @@
         <v>46202</v>
       </c>
       <c r="B152" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C152" t="s">
         <v>26</v>
@@ -8806,7 +8806,7 @@
         <v>46202</v>
       </c>
       <c r="B153" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C153" t="s">
         <v>48</v>
@@ -8841,7 +8841,7 @@
         <v>46202</v>
       </c>
       <c r="B154" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D154" t="s">
         <v>56</v>
@@ -8873,7 +8873,7 @@
         <v>46202</v>
       </c>
       <c r="B155" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D155" t="s">
         <v>62</v>
@@ -8905,7 +8905,7 @@
         <v>46202</v>
       </c>
       <c r="B156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D156" t="s">
         <v>56</v>
@@ -8937,7 +8937,7 @@
         <v>46202</v>
       </c>
       <c r="B157" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D157" t="s">
         <v>57</v>
@@ -8969,7 +8969,7 @@
         <v>46202</v>
       </c>
       <c r="B158" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C158" t="s">
         <v>18</v>
@@ -9004,7 +9004,7 @@
         <v>46202</v>
       </c>
       <c r="B159" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D159" t="s">
         <v>55</v>
@@ -9036,7 +9036,7 @@
         <v>46202</v>
       </c>
       <c r="B160" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D160" t="s">
         <v>55</v>
@@ -9068,7 +9068,7 @@
         <v>46202</v>
       </c>
       <c r="B161" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D161" t="s">
         <v>56</v>
@@ -9100,7 +9100,7 @@
         <v>46202</v>
       </c>
       <c r="B162" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C162" t="s">
         <v>18</v>
@@ -9135,7 +9135,7 @@
         <v>46202</v>
       </c>
       <c r="B163" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D163" t="s">
         <v>58</v>
@@ -9167,7 +9167,7 @@
         <v>46203</v>
       </c>
       <c r="B164" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D164" t="s">
         <v>56</v>
@@ -9199,7 +9199,7 @@
         <v>46203</v>
       </c>
       <c r="B165" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D165" t="s">
         <v>56</v>
@@ -9231,7 +9231,7 @@
         <v>46203</v>
       </c>
       <c r="B166" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D166" t="s">
         <v>56</v>
@@ -9263,7 +9263,7 @@
         <v>46203</v>
       </c>
       <c r="B167" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D167" t="s">
         <v>56</v>
@@ -9295,7 +9295,7 @@
         <v>46203</v>
       </c>
       <c r="B168" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C168" t="s">
         <v>32</v>
@@ -9330,7 +9330,7 @@
         <v>46203</v>
       </c>
       <c r="B169" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C169" t="s">
         <v>29</v>
@@ -9365,7 +9365,7 @@
         <v>46203</v>
       </c>
       <c r="B170" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C170" t="s">
         <v>26</v>
@@ -9400,7 +9400,7 @@
         <v>46203</v>
       </c>
       <c r="B171" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D171" t="s">
         <v>55</v>
@@ -9432,7 +9432,7 @@
         <v>46203</v>
       </c>
       <c r="B172" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C172" t="s">
         <v>23</v>
@@ -9467,7 +9467,7 @@
         <v>46203</v>
       </c>
       <c r="B173" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C173" t="s">
         <v>38</v>
@@ -9502,7 +9502,7 @@
         <v>46203</v>
       </c>
       <c r="B174" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C174" t="s">
         <v>21</v>
@@ -9537,7 +9537,7 @@
         <v>46203</v>
       </c>
       <c r="B175" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D175" t="s">
         <v>56</v>
@@ -9569,7 +9569,7 @@
         <v>46203</v>
       </c>
       <c r="B176" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D176" t="s">
         <v>58</v>
@@ -9601,7 +9601,7 @@
         <v>46203</v>
       </c>
       <c r="B177" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D177" t="s">
         <v>58</v>
@@ -9633,7 +9633,7 @@
         <v>46203</v>
       </c>
       <c r="B178" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C178" t="s">
         <v>46</v>
@@ -9668,7 +9668,7 @@
         <v>46203</v>
       </c>
       <c r="B179" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D179" t="s">
         <v>55</v>
@@ -9700,7 +9700,7 @@
         <v>46203</v>
       </c>
       <c r="B180" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D180" t="s">
         <v>58</v>
@@ -9732,7 +9732,7 @@
         <v>46203</v>
       </c>
       <c r="B181" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D181" t="s">
         <v>56</v>
@@ -9764,7 +9764,7 @@
         <v>46203</v>
       </c>
       <c r="B182" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C182" t="s">
         <v>45</v>
@@ -9799,7 +9799,7 @@
         <v>46203</v>
       </c>
       <c r="B183" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D183" t="s">
         <v>55</v>
@@ -9831,7 +9831,7 @@
         <v>46203</v>
       </c>
       <c r="B184" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D184" t="s">
         <v>55</v>
@@ -9863,7 +9863,7 @@
         <v>46203</v>
       </c>
       <c r="B185" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C185" t="s">
         <v>50</v>
@@ -9898,7 +9898,7 @@
         <v>46203</v>
       </c>
       <c r="B186" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D186" t="s">
         <v>62</v>
@@ -9930,7 +9930,7 @@
         <v>46203</v>
       </c>
       <c r="B187" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D187" t="s">
         <v>58</v>
@@ -9962,7 +9962,7 @@
         <v>46203</v>
       </c>
       <c r="B188" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C188" t="s">
         <v>51</v>
@@ -9997,7 +9997,7 @@
         <v>46203</v>
       </c>
       <c r="B189" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D189" t="s">
         <v>55</v>
@@ -10029,7 +10029,7 @@
         <v>46203</v>
       </c>
       <c r="B190" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D190" t="s">
         <v>61</v>
@@ -10061,7 +10061,7 @@
         <v>46203</v>
       </c>
       <c r="B191" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D191" t="s">
         <v>61</v>
@@ -10093,7 +10093,7 @@
         <v>46203</v>
       </c>
       <c r="B192" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D192" t="s">
         <v>55</v>
@@ -10125,7 +10125,7 @@
         <v>46203</v>
       </c>
       <c r="B193" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C193" t="s">
         <v>18</v>
@@ -10160,7 +10160,7 @@
         <v>46203</v>
       </c>
       <c r="B194" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C194" t="s">
         <v>18</v>
@@ -10195,7 +10195,7 @@
         <v>46203</v>
       </c>
       <c r="B195" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C195" t="s">
         <v>44</v>
@@ -10230,7 +10230,7 @@
         <v>46203</v>
       </c>
       <c r="B196" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C196" t="s">
         <v>18</v>
@@ -10265,7 +10265,7 @@
         <v>46203</v>
       </c>
       <c r="B197" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C197" t="s">
         <v>18</v>
@@ -10300,7 +10300,7 @@
         <v>46203</v>
       </c>
       <c r="B198" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C198" t="s">
         <v>32</v>
@@ -10335,7 +10335,7 @@
         <v>46203</v>
       </c>
       <c r="B199" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D199" t="s">
         <v>56</v>
@@ -10367,7 +10367,7 @@
         <v>46203</v>
       </c>
       <c r="B200" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C200" t="s">
         <v>18</v>
@@ -10402,7 +10402,7 @@
         <v>46203</v>
       </c>
       <c r="B201" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C201" t="s">
         <v>50</v>
@@ -10437,7 +10437,7 @@
         <v>46203</v>
       </c>
       <c r="B202" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C202" t="s">
         <v>24</v>
@@ -10472,7 +10472,7 @@
         <v>46203</v>
       </c>
       <c r="B203" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C203" t="s">
         <v>16</v>
@@ -10507,7 +10507,7 @@
         <v>46203</v>
       </c>
       <c r="B204" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D204" t="s">
         <v>55</v>
@@ -10539,7 +10539,7 @@
         <v>46203</v>
       </c>
       <c r="B205" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C205" t="s">
         <v>24</v>
@@ -10574,7 +10574,7 @@
         <v>46203</v>
       </c>
       <c r="B206" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C206" t="s">
         <v>18</v>
@@ -10609,7 +10609,7 @@
         <v>46203</v>
       </c>
       <c r="B207" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D207" t="s">
         <v>55</v>
@@ -10641,7 +10641,7 @@
         <v>46203</v>
       </c>
       <c r="B208" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C208" t="s">
         <v>40</v>
@@ -10676,7 +10676,7 @@
         <v>46203</v>
       </c>
       <c r="B209" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C209" t="s">
         <v>24</v>
@@ -10711,7 +10711,7 @@
         <v>46203</v>
       </c>
       <c r="B210" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C210" t="s">
         <v>36</v>
@@ -10746,7 +10746,7 @@
         <v>46203</v>
       </c>
       <c r="B211" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D211" t="s">
         <v>56</v>
@@ -10778,7 +10778,7 @@
         <v>46203</v>
       </c>
       <c r="B212" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D212" t="s">
         <v>55</v>
@@ -10810,7 +10810,7 @@
         <v>46203</v>
       </c>
       <c r="B213" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D213" t="s">
         <v>61</v>
@@ -10842,7 +10842,7 @@
         <v>46203</v>
       </c>
       <c r="B214" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D214" t="s">
         <v>56</v>
@@ -10874,7 +10874,7 @@
         <v>46203</v>
       </c>
       <c r="B215" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D215" t="s">
         <v>56</v>
@@ -10906,7 +10906,7 @@
         <v>46203</v>
       </c>
       <c r="B216" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D216" t="s">
         <v>57</v>
@@ -10938,7 +10938,7 @@
         <v>46203</v>
       </c>
       <c r="B217" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D217" t="s">
         <v>56</v>
@@ -10970,7 +10970,7 @@
         <v>46203</v>
       </c>
       <c r="B218" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D218" t="s">
         <v>55</v>
@@ -11002,7 +11002,7 @@
         <v>46203</v>
       </c>
       <c r="B219" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D219" t="s">
         <v>58</v>
@@ -11034,7 +11034,7 @@
         <v>46203</v>
       </c>
       <c r="B220" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C220" t="s">
         <v>51</v>
@@ -11069,7 +11069,7 @@
         <v>46203</v>
       </c>
       <c r="B221" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D221" t="s">
         <v>63</v>
@@ -11101,7 +11101,7 @@
         <v>46203</v>
       </c>
       <c r="B222" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D222" t="s">
         <v>55</v>
@@ -11133,7 +11133,7 @@
         <v>46203</v>
       </c>
       <c r="B223" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C223" t="s">
         <v>35</v>
@@ -11168,7 +11168,7 @@
         <v>46203</v>
       </c>
       <c r="B224" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D224" t="s">
         <v>55</v>
@@ -11200,7 +11200,7 @@
         <v>46203</v>
       </c>
       <c r="B225" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D225" t="s">
         <v>55</v>
@@ -11232,7 +11232,7 @@
         <v>46203</v>
       </c>
       <c r="B226" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D226" t="s">
         <v>55</v>
@@ -11264,7 +11264,7 @@
         <v>46203</v>
       </c>
       <c r="B227" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C227" t="s">
         <v>30</v>
@@ -11299,7 +11299,7 @@
         <v>46203</v>
       </c>
       <c r="B228" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D228" t="s">
         <v>55</v>
@@ -11331,7 +11331,7 @@
         <v>46203</v>
       </c>
       <c r="B229" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C229" t="s">
         <v>30</v>
@@ -11366,7 +11366,7 @@
         <v>46203</v>
       </c>
       <c r="B230" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C230" t="s">
         <v>38</v>
@@ -11401,7 +11401,7 @@
         <v>46203</v>
       </c>
       <c r="B231" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C231" t="s">
         <v>37</v>
@@ -11436,7 +11436,7 @@
         <v>46203</v>
       </c>
       <c r="B232" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D232" t="s">
         <v>56</v>
@@ -11468,7 +11468,7 @@
         <v>46203</v>
       </c>
       <c r="B233" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C233" t="s">
         <v>24</v>
@@ -11503,7 +11503,7 @@
         <v>46203</v>
       </c>
       <c r="B234" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C234" t="s">
         <v>40</v>
@@ -11538,7 +11538,7 @@
         <v>46203</v>
       </c>
       <c r="B235" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C235" t="s">
         <v>40</v>
@@ -11573,7 +11573,7 @@
         <v>46203</v>
       </c>
       <c r="B236" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C236" t="s">
         <v>27</v>
@@ -11608,7 +11608,7 @@
         <v>46203</v>
       </c>
       <c r="B237" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C237" t="s">
         <v>42</v>
@@ -11643,7 +11643,7 @@
         <v>46203</v>
       </c>
       <c r="B238" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C238" t="s">
         <v>16</v>
@@ -11678,7 +11678,7 @@
         <v>46203</v>
       </c>
       <c r="B239" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C239" t="s">
         <v>40</v>
@@ -11713,7 +11713,7 @@
         <v>46203</v>
       </c>
       <c r="B240" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C240" t="s">
         <v>46</v>
@@ -11748,7 +11748,7 @@
         <v>46203</v>
       </c>
       <c r="B241" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D241" t="s">
         <v>57</v>
@@ -11780,7 +11780,7 @@
         <v>46203</v>
       </c>
       <c r="B242" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C242" t="s">
         <v>49</v>
@@ -11815,7 +11815,7 @@
         <v>46203</v>
       </c>
       <c r="B243" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C243" t="s">
         <v>18</v>
@@ -11850,7 +11850,7 @@
         <v>46203</v>
       </c>
       <c r="B244" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D244" t="s">
         <v>56</v>
@@ -11882,7 +11882,7 @@
         <v>46203</v>
       </c>
       <c r="B245" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D245" t="s">
         <v>56</v>
@@ -11914,7 +11914,7 @@
         <v>46203</v>
       </c>
       <c r="B246" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D246" t="s">
         <v>56</v>
@@ -11946,7 +11946,7 @@
         <v>46203</v>
       </c>
       <c r="B247" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D247" t="s">
         <v>56</v>
@@ -11978,7 +11978,7 @@
         <v>46203</v>
       </c>
       <c r="B248" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D248" t="s">
         <v>56</v>
@@ -12010,7 +12010,7 @@
         <v>46203</v>
       </c>
       <c r="B249" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D249" t="s">
         <v>55</v>
@@ -12042,7 +12042,7 @@
         <v>46203</v>
       </c>
       <c r="B250" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D250" t="s">
         <v>56</v>
@@ -12074,7 +12074,7 @@
         <v>46203</v>
       </c>
       <c r="B251" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D251" t="s">
         <v>56</v>
@@ -12106,7 +12106,7 @@
         <v>46204</v>
       </c>
       <c r="B252" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C252" t="s">
         <v>52</v>
@@ -12141,7 +12141,7 @@
         <v>46204</v>
       </c>
       <c r="B253" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C253" t="s">
         <v>19</v>
@@ -12176,7 +12176,7 @@
         <v>46204</v>
       </c>
       <c r="B254" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C254" t="s">
         <v>18</v>
@@ -12211,7 +12211,7 @@
         <v>46204</v>
       </c>
       <c r="B255" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C255" t="s">
         <v>19</v>
@@ -12246,7 +12246,7 @@
         <v>46204</v>
       </c>
       <c r="B256" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C256" t="s">
         <v>26</v>
@@ -12281,7 +12281,7 @@
         <v>46204</v>
       </c>
       <c r="B257" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C257" t="s">
         <v>35</v>
@@ -12316,7 +12316,7 @@
         <v>46204</v>
       </c>
       <c r="B258" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C258" t="s">
         <v>48</v>
@@ -12351,7 +12351,7 @@
         <v>46204</v>
       </c>
       <c r="B259" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C259" t="s">
         <v>40</v>
@@ -12386,7 +12386,7 @@
         <v>46204</v>
       </c>
       <c r="B260" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C260" t="s">
         <v>53</v>
@@ -12421,7 +12421,7 @@
         <v>46204</v>
       </c>
       <c r="B261" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D261" t="s">
         <v>58</v>
@@ -12453,7 +12453,7 @@
         <v>46204</v>
       </c>
       <c r="B262" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C262" t="s">
         <v>39</v>
@@ -12488,7 +12488,7 @@
         <v>46204</v>
       </c>
       <c r="B263" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C263" t="s">
         <v>29</v>
@@ -12523,7 +12523,7 @@
         <v>46204</v>
       </c>
       <c r="B264" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D264" t="s">
         <v>58</v>
@@ -12555,7 +12555,7 @@
         <v>46204</v>
       </c>
       <c r="B265" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C265" t="s">
         <v>18</v>
@@ -12590,7 +12590,7 @@
         <v>46204</v>
       </c>
       <c r="B266" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C266" t="s">
         <v>32</v>
@@ -12625,7 +12625,7 @@
         <v>46204</v>
       </c>
       <c r="B267" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C267" t="s">
         <v>16</v>
@@ -12660,7 +12660,7 @@
         <v>46204</v>
       </c>
       <c r="B268" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C268" t="s">
         <v>33</v>
@@ -12695,7 +12695,7 @@
         <v>46204</v>
       </c>
       <c r="B269" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D269" t="s">
         <v>55</v>
@@ -12727,7 +12727,7 @@
         <v>46204</v>
       </c>
       <c r="B270" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D270" t="s">
         <v>55</v>
@@ -12759,7 +12759,7 @@
         <v>46204</v>
       </c>
       <c r="B271" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D271" t="s">
         <v>55</v>
@@ -12791,7 +12791,7 @@
         <v>46204</v>
       </c>
       <c r="B272" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D272" t="s">
         <v>56</v>
@@ -12823,7 +12823,7 @@
         <v>46204</v>
       </c>
       <c r="B273" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C273" t="s">
         <v>27</v>
@@ -12858,7 +12858,7 @@
         <v>46204</v>
       </c>
       <c r="B274" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D274" t="s">
         <v>56</v>
@@ -12890,7 +12890,7 @@
         <v>46204</v>
       </c>
       <c r="B275" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D275" t="s">
         <v>56</v>
@@ -12922,7 +12922,7 @@
         <v>46204</v>
       </c>
       <c r="B276" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C276" t="s">
         <v>25</v>
@@ -12957,7 +12957,7 @@
         <v>46204</v>
       </c>
       <c r="B277" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C277" t="s">
         <v>49</v>
@@ -12992,7 +12992,7 @@
         <v>46204</v>
       </c>
       <c r="B278" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D278" t="s">
         <v>56</v>
@@ -13024,7 +13024,7 @@
         <v>46204</v>
       </c>
       <c r="B279" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D279" t="s">
         <v>56</v>
@@ -13056,7 +13056,7 @@
         <v>46204</v>
       </c>
       <c r="B280" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D280" t="s">
         <v>56</v>
@@ -13088,7 +13088,7 @@
         <v>46204</v>
       </c>
       <c r="B281" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C281" t="s">
         <v>40</v>
@@ -13123,7 +13123,7 @@
         <v>46204</v>
       </c>
       <c r="B282" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D282" t="s">
         <v>55</v>
@@ -13155,7 +13155,7 @@
         <v>46204</v>
       </c>
       <c r="B283" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C283" t="s">
         <v>38</v>
@@ -13190,7 +13190,7 @@
         <v>46204</v>
       </c>
       <c r="B284" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C284" t="s">
         <v>36</v>
@@ -13225,7 +13225,7 @@
         <v>46204</v>
       </c>
       <c r="B285" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C285" t="s">
         <v>45</v>
@@ -13260,7 +13260,7 @@
         <v>46204</v>
       </c>
       <c r="B286" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C286" t="s">
         <v>40</v>
@@ -13295,7 +13295,7 @@
         <v>46204</v>
       </c>
       <c r="B287" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C287" t="s">
         <v>18</v>
@@ -13330,7 +13330,7 @@
         <v>46204</v>
       </c>
       <c r="B288" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C288" t="s">
         <v>40</v>
@@ -13365,7 +13365,7 @@
         <v>46204</v>
       </c>
       <c r="B289" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C289" t="s">
         <v>29</v>
@@ -13400,7 +13400,7 @@
         <v>46204</v>
       </c>
       <c r="B290" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C290" t="s">
         <v>23</v>
@@ -13435,7 +13435,7 @@
         <v>46204</v>
       </c>
       <c r="B291" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C291" t="s">
         <v>43</v>
@@ -13470,7 +13470,7 @@
         <v>46204</v>
       </c>
       <c r="B292" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C292" t="s">
         <v>53</v>
@@ -13505,7 +13505,7 @@
         <v>46204</v>
       </c>
       <c r="B293" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D293" t="s">
         <v>58</v>

</xml_diff>

<commit_message>
Audiências: sync 2026-07-01 — 424 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -8022,7 +8022,7 @@
         <v>46202</v>
       </c>
       <c r="B130" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C130" t="s">
         <v>46</v>
@@ -8057,7 +8057,7 @@
         <v>46202</v>
       </c>
       <c r="B131" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D131" t="s">
         <v>63</v>
@@ -8089,7 +8089,7 @@
         <v>46202</v>
       </c>
       <c r="B132" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D132" t="s">
         <v>56</v>
@@ -8121,7 +8121,7 @@
         <v>46202</v>
       </c>
       <c r="B133" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D133" t="s">
         <v>58</v>
@@ -8153,7 +8153,7 @@
         <v>46202</v>
       </c>
       <c r="B134" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C134" t="s">
         <v>29</v>
@@ -8188,7 +8188,7 @@
         <v>46202</v>
       </c>
       <c r="B135" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D135" t="s">
         <v>58</v>
@@ -8220,7 +8220,7 @@
         <v>46202</v>
       </c>
       <c r="B136" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C136" t="s">
         <v>47</v>
@@ -8255,7 +8255,7 @@
         <v>46202</v>
       </c>
       <c r="B137" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C137" t="s">
         <v>36</v>
@@ -8290,7 +8290,7 @@
         <v>46202</v>
       </c>
       <c r="B138" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C138" t="s">
         <v>48</v>
@@ -8325,7 +8325,7 @@
         <v>46202</v>
       </c>
       <c r="B139" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C139" t="s">
         <v>16</v>
@@ -8360,7 +8360,7 @@
         <v>46202</v>
       </c>
       <c r="B140" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C140" t="s">
         <v>27</v>
@@ -8395,7 +8395,7 @@
         <v>46202</v>
       </c>
       <c r="B141" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C141" t="s">
         <v>37</v>
@@ -8430,7 +8430,7 @@
         <v>46202</v>
       </c>
       <c r="B142" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C142" t="s">
         <v>33</v>
@@ -8465,7 +8465,7 @@
         <v>46202</v>
       </c>
       <c r="B143" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C143" t="s">
         <v>49</v>
@@ -8500,7 +8500,7 @@
         <v>46202</v>
       </c>
       <c r="B144" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C144" t="s">
         <v>18</v>
@@ -8535,7 +8535,7 @@
         <v>46202</v>
       </c>
       <c r="B145" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D145" t="s">
         <v>55</v>
@@ -8567,7 +8567,7 @@
         <v>46202</v>
       </c>
       <c r="B146" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C146" t="s">
         <v>32</v>
@@ -8602,7 +8602,7 @@
         <v>46202</v>
       </c>
       <c r="B147" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C147" t="s">
         <v>40</v>
@@ -8637,7 +8637,7 @@
         <v>46202</v>
       </c>
       <c r="B148" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C148" t="s">
         <v>25</v>
@@ -8672,7 +8672,7 @@
         <v>46202</v>
       </c>
       <c r="B149" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C149" t="s">
         <v>38</v>
@@ -8707,7 +8707,7 @@
         <v>46202</v>
       </c>
       <c r="B150" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D150" t="s">
         <v>55</v>
@@ -8739,7 +8739,7 @@
         <v>46202</v>
       </c>
       <c r="B151" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D151" t="s">
         <v>55</v>
@@ -8771,7 +8771,7 @@
         <v>46202</v>
       </c>
       <c r="B152" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C152" t="s">
         <v>26</v>
@@ -8806,7 +8806,7 @@
         <v>46202</v>
       </c>
       <c r="B153" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C153" t="s">
         <v>48</v>
@@ -8841,7 +8841,7 @@
         <v>46202</v>
       </c>
       <c r="B154" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D154" t="s">
         <v>56</v>
@@ -8873,7 +8873,7 @@
         <v>46202</v>
       </c>
       <c r="B155" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D155" t="s">
         <v>62</v>
@@ -8905,7 +8905,7 @@
         <v>46202</v>
       </c>
       <c r="B156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D156" t="s">
         <v>56</v>
@@ -8937,7 +8937,7 @@
         <v>46202</v>
       </c>
       <c r="B157" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D157" t="s">
         <v>57</v>
@@ -8969,7 +8969,7 @@
         <v>46202</v>
       </c>
       <c r="B158" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C158" t="s">
         <v>18</v>
@@ -9004,7 +9004,7 @@
         <v>46202</v>
       </c>
       <c r="B159" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D159" t="s">
         <v>55</v>
@@ -9036,7 +9036,7 @@
         <v>46202</v>
       </c>
       <c r="B160" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D160" t="s">
         <v>55</v>
@@ -9068,7 +9068,7 @@
         <v>46202</v>
       </c>
       <c r="B161" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D161" t="s">
         <v>56</v>
@@ -9100,7 +9100,7 @@
         <v>46202</v>
       </c>
       <c r="B162" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C162" t="s">
         <v>18</v>
@@ -9135,7 +9135,7 @@
         <v>46202</v>
       </c>
       <c r="B163" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D163" t="s">
         <v>58</v>
@@ -9167,7 +9167,7 @@
         <v>46203</v>
       </c>
       <c r="B164" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D164" t="s">
         <v>56</v>
@@ -9199,7 +9199,7 @@
         <v>46203</v>
       </c>
       <c r="B165" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D165" t="s">
         <v>56</v>
@@ -9231,7 +9231,7 @@
         <v>46203</v>
       </c>
       <c r="B166" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D166" t="s">
         <v>56</v>
@@ -9263,7 +9263,7 @@
         <v>46203</v>
       </c>
       <c r="B167" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D167" t="s">
         <v>56</v>
@@ -9295,7 +9295,7 @@
         <v>46203</v>
       </c>
       <c r="B168" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C168" t="s">
         <v>32</v>
@@ -9330,7 +9330,7 @@
         <v>46203</v>
       </c>
       <c r="B169" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C169" t="s">
         <v>29</v>
@@ -9365,7 +9365,7 @@
         <v>46203</v>
       </c>
       <c r="B170" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C170" t="s">
         <v>26</v>
@@ -9400,7 +9400,7 @@
         <v>46203</v>
       </c>
       <c r="B171" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D171" t="s">
         <v>55</v>
@@ -9432,7 +9432,7 @@
         <v>46203</v>
       </c>
       <c r="B172" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C172" t="s">
         <v>23</v>
@@ -9467,7 +9467,7 @@
         <v>46203</v>
       </c>
       <c r="B173" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C173" t="s">
         <v>38</v>
@@ -9502,7 +9502,7 @@
         <v>46203</v>
       </c>
       <c r="B174" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C174" t="s">
         <v>21</v>
@@ -9537,7 +9537,7 @@
         <v>46203</v>
       </c>
       <c r="B175" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D175" t="s">
         <v>56</v>
@@ -9569,7 +9569,7 @@
         <v>46203</v>
       </c>
       <c r="B176" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D176" t="s">
         <v>58</v>
@@ -9601,7 +9601,7 @@
         <v>46203</v>
       </c>
       <c r="B177" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D177" t="s">
         <v>58</v>
@@ -9633,7 +9633,7 @@
         <v>46203</v>
       </c>
       <c r="B178" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C178" t="s">
         <v>46</v>
@@ -9668,7 +9668,7 @@
         <v>46203</v>
       </c>
       <c r="B179" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D179" t="s">
         <v>55</v>
@@ -9700,7 +9700,7 @@
         <v>46203</v>
       </c>
       <c r="B180" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D180" t="s">
         <v>58</v>
@@ -9732,7 +9732,7 @@
         <v>46203</v>
       </c>
       <c r="B181" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D181" t="s">
         <v>56</v>
@@ -9764,7 +9764,7 @@
         <v>46203</v>
       </c>
       <c r="B182" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C182" t="s">
         <v>45</v>
@@ -9799,7 +9799,7 @@
         <v>46203</v>
       </c>
       <c r="B183" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D183" t="s">
         <v>55</v>
@@ -9831,7 +9831,7 @@
         <v>46203</v>
       </c>
       <c r="B184" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D184" t="s">
         <v>55</v>
@@ -9863,7 +9863,7 @@
         <v>46203</v>
       </c>
       <c r="B185" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C185" t="s">
         <v>50</v>
@@ -9898,7 +9898,7 @@
         <v>46203</v>
       </c>
       <c r="B186" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D186" t="s">
         <v>62</v>
@@ -9930,7 +9930,7 @@
         <v>46203</v>
       </c>
       <c r="B187" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D187" t="s">
         <v>58</v>
@@ -9962,7 +9962,7 @@
         <v>46203</v>
       </c>
       <c r="B188" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C188" t="s">
         <v>51</v>
@@ -9997,7 +9997,7 @@
         <v>46203</v>
       </c>
       <c r="B189" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D189" t="s">
         <v>55</v>
@@ -10029,7 +10029,7 @@
         <v>46203</v>
       </c>
       <c r="B190" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D190" t="s">
         <v>61</v>
@@ -10061,7 +10061,7 @@
         <v>46203</v>
       </c>
       <c r="B191" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D191" t="s">
         <v>61</v>
@@ -10093,7 +10093,7 @@
         <v>46203</v>
       </c>
       <c r="B192" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D192" t="s">
         <v>55</v>
@@ -10125,7 +10125,7 @@
         <v>46203</v>
       </c>
       <c r="B193" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C193" t="s">
         <v>18</v>
@@ -10160,7 +10160,7 @@
         <v>46203</v>
       </c>
       <c r="B194" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C194" t="s">
         <v>18</v>
@@ -10195,7 +10195,7 @@
         <v>46203</v>
       </c>
       <c r="B195" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C195" t="s">
         <v>44</v>
@@ -10230,7 +10230,7 @@
         <v>46203</v>
       </c>
       <c r="B196" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C196" t="s">
         <v>18</v>
@@ -10265,7 +10265,7 @@
         <v>46203</v>
       </c>
       <c r="B197" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C197" t="s">
         <v>18</v>
@@ -10300,7 +10300,7 @@
         <v>46203</v>
       </c>
       <c r="B198" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C198" t="s">
         <v>32</v>
@@ -10335,7 +10335,7 @@
         <v>46203</v>
       </c>
       <c r="B199" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D199" t="s">
         <v>56</v>
@@ -10367,7 +10367,7 @@
         <v>46203</v>
       </c>
       <c r="B200" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C200" t="s">
         <v>18</v>
@@ -10402,7 +10402,7 @@
         <v>46203</v>
       </c>
       <c r="B201" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C201" t="s">
         <v>50</v>
@@ -10437,7 +10437,7 @@
         <v>46203</v>
       </c>
       <c r="B202" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C202" t="s">
         <v>24</v>
@@ -10472,7 +10472,7 @@
         <v>46203</v>
       </c>
       <c r="B203" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C203" t="s">
         <v>16</v>
@@ -10507,7 +10507,7 @@
         <v>46203</v>
       </c>
       <c r="B204" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D204" t="s">
         <v>55</v>
@@ -10539,7 +10539,7 @@
         <v>46203</v>
       </c>
       <c r="B205" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C205" t="s">
         <v>24</v>
@@ -10574,7 +10574,7 @@
         <v>46203</v>
       </c>
       <c r="B206" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C206" t="s">
         <v>18</v>
@@ -10609,7 +10609,7 @@
         <v>46203</v>
       </c>
       <c r="B207" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D207" t="s">
         <v>55</v>
@@ -10641,7 +10641,7 @@
         <v>46203</v>
       </c>
       <c r="B208" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C208" t="s">
         <v>40</v>
@@ -10676,7 +10676,7 @@
         <v>46203</v>
       </c>
       <c r="B209" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C209" t="s">
         <v>24</v>
@@ -10711,7 +10711,7 @@
         <v>46203</v>
       </c>
       <c r="B210" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C210" t="s">
         <v>36</v>
@@ -10746,7 +10746,7 @@
         <v>46203</v>
       </c>
       <c r="B211" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D211" t="s">
         <v>56</v>
@@ -10778,7 +10778,7 @@
         <v>46203</v>
       </c>
       <c r="B212" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D212" t="s">
         <v>55</v>
@@ -10810,7 +10810,7 @@
         <v>46203</v>
       </c>
       <c r="B213" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D213" t="s">
         <v>61</v>
@@ -10842,7 +10842,7 @@
         <v>46203</v>
       </c>
       <c r="B214" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D214" t="s">
         <v>56</v>
@@ -10874,7 +10874,7 @@
         <v>46203</v>
       </c>
       <c r="B215" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D215" t="s">
         <v>56</v>
@@ -10906,7 +10906,7 @@
         <v>46203</v>
       </c>
       <c r="B216" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D216" t="s">
         <v>57</v>
@@ -10938,7 +10938,7 @@
         <v>46203</v>
       </c>
       <c r="B217" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D217" t="s">
         <v>56</v>
@@ -10970,7 +10970,7 @@
         <v>46203</v>
       </c>
       <c r="B218" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D218" t="s">
         <v>55</v>
@@ -11002,7 +11002,7 @@
         <v>46203</v>
       </c>
       <c r="B219" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D219" t="s">
         <v>58</v>
@@ -11034,7 +11034,7 @@
         <v>46203</v>
       </c>
       <c r="B220" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C220" t="s">
         <v>51</v>
@@ -11069,7 +11069,7 @@
         <v>46203</v>
       </c>
       <c r="B221" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D221" t="s">
         <v>63</v>
@@ -11101,7 +11101,7 @@
         <v>46203</v>
       </c>
       <c r="B222" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D222" t="s">
         <v>55</v>
@@ -11133,7 +11133,7 @@
         <v>46203</v>
       </c>
       <c r="B223" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C223" t="s">
         <v>35</v>
@@ -11168,7 +11168,7 @@
         <v>46203</v>
       </c>
       <c r="B224" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D224" t="s">
         <v>55</v>
@@ -11200,7 +11200,7 @@
         <v>46203</v>
       </c>
       <c r="B225" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D225" t="s">
         <v>55</v>
@@ -11232,7 +11232,7 @@
         <v>46203</v>
       </c>
       <c r="B226" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D226" t="s">
         <v>55</v>
@@ -11264,7 +11264,7 @@
         <v>46203</v>
       </c>
       <c r="B227" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C227" t="s">
         <v>30</v>
@@ -11299,7 +11299,7 @@
         <v>46203</v>
       </c>
       <c r="B228" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D228" t="s">
         <v>55</v>
@@ -11331,7 +11331,7 @@
         <v>46203</v>
       </c>
       <c r="B229" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C229" t="s">
         <v>30</v>
@@ -11366,7 +11366,7 @@
         <v>46203</v>
       </c>
       <c r="B230" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C230" t="s">
         <v>38</v>
@@ -11401,7 +11401,7 @@
         <v>46203</v>
       </c>
       <c r="B231" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C231" t="s">
         <v>37</v>
@@ -11436,7 +11436,7 @@
         <v>46203</v>
       </c>
       <c r="B232" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D232" t="s">
         <v>56</v>
@@ -11468,7 +11468,7 @@
         <v>46203</v>
       </c>
       <c r="B233" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C233" t="s">
         <v>24</v>
@@ -11503,7 +11503,7 @@
         <v>46203</v>
       </c>
       <c r="B234" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C234" t="s">
         <v>40</v>
@@ -11538,7 +11538,7 @@
         <v>46203</v>
       </c>
       <c r="B235" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C235" t="s">
         <v>40</v>
@@ -11573,7 +11573,7 @@
         <v>46203</v>
       </c>
       <c r="B236" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C236" t="s">
         <v>27</v>
@@ -11608,7 +11608,7 @@
         <v>46203</v>
       </c>
       <c r="B237" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C237" t="s">
         <v>42</v>
@@ -11643,7 +11643,7 @@
         <v>46203</v>
       </c>
       <c r="B238" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C238" t="s">
         <v>16</v>
@@ -11678,7 +11678,7 @@
         <v>46203</v>
       </c>
       <c r="B239" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C239" t="s">
         <v>40</v>
@@ -11713,7 +11713,7 @@
         <v>46203</v>
       </c>
       <c r="B240" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C240" t="s">
         <v>46</v>
@@ -11748,7 +11748,7 @@
         <v>46203</v>
       </c>
       <c r="B241" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D241" t="s">
         <v>57</v>
@@ -11780,7 +11780,7 @@
         <v>46203</v>
       </c>
       <c r="B242" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C242" t="s">
         <v>49</v>
@@ -11815,7 +11815,7 @@
         <v>46203</v>
       </c>
       <c r="B243" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C243" t="s">
         <v>18</v>
@@ -11850,7 +11850,7 @@
         <v>46203</v>
       </c>
       <c r="B244" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D244" t="s">
         <v>56</v>
@@ -11882,7 +11882,7 @@
         <v>46203</v>
       </c>
       <c r="B245" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D245" t="s">
         <v>56</v>
@@ -11914,7 +11914,7 @@
         <v>46203</v>
       </c>
       <c r="B246" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D246" t="s">
         <v>56</v>
@@ -11946,7 +11946,7 @@
         <v>46203</v>
       </c>
       <c r="B247" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D247" t="s">
         <v>56</v>
@@ -11978,7 +11978,7 @@
         <v>46203</v>
       </c>
       <c r="B248" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D248" t="s">
         <v>56</v>
@@ -12010,7 +12010,7 @@
         <v>46203</v>
       </c>
       <c r="B249" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D249" t="s">
         <v>55</v>
@@ -12042,7 +12042,7 @@
         <v>46203</v>
       </c>
       <c r="B250" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D250" t="s">
         <v>56</v>
@@ -12074,7 +12074,7 @@
         <v>46203</v>
       </c>
       <c r="B251" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D251" t="s">
         <v>56</v>
@@ -12106,7 +12106,7 @@
         <v>46204</v>
       </c>
       <c r="B252" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C252" t="s">
         <v>52</v>
@@ -12141,7 +12141,7 @@
         <v>46204</v>
       </c>
       <c r="B253" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C253" t="s">
         <v>19</v>
@@ -12176,7 +12176,7 @@
         <v>46204</v>
       </c>
       <c r="B254" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C254" t="s">
         <v>18</v>
@@ -12211,7 +12211,7 @@
         <v>46204</v>
       </c>
       <c r="B255" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C255" t="s">
         <v>19</v>
@@ -12246,7 +12246,7 @@
         <v>46204</v>
       </c>
       <c r="B256" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C256" t="s">
         <v>26</v>
@@ -12281,7 +12281,7 @@
         <v>46204</v>
       </c>
       <c r="B257" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C257" t="s">
         <v>35</v>
@@ -12316,7 +12316,7 @@
         <v>46204</v>
       </c>
       <c r="B258" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C258" t="s">
         <v>48</v>
@@ -12351,7 +12351,7 @@
         <v>46204</v>
       </c>
       <c r="B259" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C259" t="s">
         <v>40</v>
@@ -12386,7 +12386,7 @@
         <v>46204</v>
       </c>
       <c r="B260" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C260" t="s">
         <v>53</v>
@@ -12421,7 +12421,7 @@
         <v>46204</v>
       </c>
       <c r="B261" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D261" t="s">
         <v>58</v>
@@ -12453,7 +12453,7 @@
         <v>46204</v>
       </c>
       <c r="B262" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C262" t="s">
         <v>39</v>
@@ -12488,7 +12488,7 @@
         <v>46204</v>
       </c>
       <c r="B263" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C263" t="s">
         <v>29</v>
@@ -12523,7 +12523,7 @@
         <v>46204</v>
       </c>
       <c r="B264" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D264" t="s">
         <v>58</v>
@@ -12555,7 +12555,7 @@
         <v>46204</v>
       </c>
       <c r="B265" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C265" t="s">
         <v>18</v>
@@ -12590,7 +12590,7 @@
         <v>46204</v>
       </c>
       <c r="B266" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C266" t="s">
         <v>32</v>
@@ -12625,7 +12625,7 @@
         <v>46204</v>
       </c>
       <c r="B267" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C267" t="s">
         <v>16</v>
@@ -12660,7 +12660,7 @@
         <v>46204</v>
       </c>
       <c r="B268" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C268" t="s">
         <v>33</v>
@@ -12695,7 +12695,7 @@
         <v>46204</v>
       </c>
       <c r="B269" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D269" t="s">
         <v>55</v>
@@ -12727,7 +12727,7 @@
         <v>46204</v>
       </c>
       <c r="B270" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D270" t="s">
         <v>55</v>
@@ -12759,7 +12759,7 @@
         <v>46204</v>
       </c>
       <c r="B271" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D271" t="s">
         <v>55</v>
@@ -12791,7 +12791,7 @@
         <v>46204</v>
       </c>
       <c r="B272" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D272" t="s">
         <v>56</v>
@@ -12823,7 +12823,7 @@
         <v>46204</v>
       </c>
       <c r="B273" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C273" t="s">
         <v>27</v>
@@ -12858,7 +12858,7 @@
         <v>46204</v>
       </c>
       <c r="B274" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D274" t="s">
         <v>56</v>
@@ -12890,7 +12890,7 @@
         <v>46204</v>
       </c>
       <c r="B275" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D275" t="s">
         <v>56</v>
@@ -12922,7 +12922,7 @@
         <v>46204</v>
       </c>
       <c r="B276" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C276" t="s">
         <v>25</v>
@@ -12957,7 +12957,7 @@
         <v>46204</v>
       </c>
       <c r="B277" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C277" t="s">
         <v>49</v>
@@ -12992,7 +12992,7 @@
         <v>46204</v>
       </c>
       <c r="B278" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D278" t="s">
         <v>56</v>
@@ -13024,7 +13024,7 @@
         <v>46204</v>
       </c>
       <c r="B279" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D279" t="s">
         <v>56</v>
@@ -13056,7 +13056,7 @@
         <v>46204</v>
       </c>
       <c r="B280" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D280" t="s">
         <v>56</v>
@@ -13088,7 +13088,7 @@
         <v>46204</v>
       </c>
       <c r="B281" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C281" t="s">
         <v>40</v>
@@ -13123,7 +13123,7 @@
         <v>46204</v>
       </c>
       <c r="B282" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D282" t="s">
         <v>55</v>
@@ -13155,7 +13155,7 @@
         <v>46204</v>
       </c>
       <c r="B283" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C283" t="s">
         <v>38</v>
@@ -13190,7 +13190,7 @@
         <v>46204</v>
       </c>
       <c r="B284" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C284" t="s">
         <v>36</v>
@@ -13225,7 +13225,7 @@
         <v>46204</v>
       </c>
       <c r="B285" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C285" t="s">
         <v>45</v>
@@ -13260,7 +13260,7 @@
         <v>46204</v>
       </c>
       <c r="B286" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C286" t="s">
         <v>40</v>
@@ -13295,7 +13295,7 @@
         <v>46204</v>
       </c>
       <c r="B287" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C287" t="s">
         <v>18</v>
@@ -13330,7 +13330,7 @@
         <v>46204</v>
       </c>
       <c r="B288" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C288" t="s">
         <v>40</v>
@@ -13365,7 +13365,7 @@
         <v>46204</v>
       </c>
       <c r="B289" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C289" t="s">
         <v>29</v>
@@ -13400,7 +13400,7 @@
         <v>46204</v>
       </c>
       <c r="B290" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C290" t="s">
         <v>23</v>
@@ -13435,7 +13435,7 @@
         <v>46204</v>
       </c>
       <c r="B291" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C291" t="s">
         <v>43</v>
@@ -13470,7 +13470,7 @@
         <v>46204</v>
       </c>
       <c r="B292" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C292" t="s">
         <v>53</v>
@@ -13505,7 +13505,7 @@
         <v>46204</v>
       </c>
       <c r="B293" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D293" t="s">
         <v>58</v>
@@ -13537,7 +13537,7 @@
         <v>46205</v>
       </c>
       <c r="B294" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D294" t="s">
         <v>56</v>
@@ -13569,7 +13569,7 @@
         <v>46205</v>
       </c>
       <c r="B295" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D295" t="s">
         <v>56</v>
@@ -13601,7 +13601,7 @@
         <v>46205</v>
       </c>
       <c r="B296" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D296" t="s">
         <v>56</v>
@@ -13633,7 +13633,7 @@
         <v>46205</v>
       </c>
       <c r="B297" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D297" t="s">
         <v>56</v>
@@ -13665,7 +13665,7 @@
         <v>46205</v>
       </c>
       <c r="B298" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C298" t="s">
         <v>44</v>
@@ -13700,7 +13700,7 @@
         <v>46205</v>
       </c>
       <c r="B299" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C299" t="s">
         <v>26</v>
@@ -13735,7 +13735,7 @@
         <v>46205</v>
       </c>
       <c r="B300" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C300" t="s">
         <v>43</v>
@@ -13770,7 +13770,7 @@
         <v>46205</v>
       </c>
       <c r="B301" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C301" t="s">
         <v>18</v>
@@ -13805,7 +13805,7 @@
         <v>46205</v>
       </c>
       <c r="B302" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D302" t="s">
         <v>55</v>
@@ -13837,7 +13837,7 @@
         <v>46205</v>
       </c>
       <c r="B303" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C303" t="s">
         <v>53</v>
@@ -13872,7 +13872,7 @@
         <v>46205</v>
       </c>
       <c r="B304" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C304" t="s">
         <v>23</v>
@@ -13907,7 +13907,7 @@
         <v>46205</v>
       </c>
       <c r="B305" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D305" t="s">
         <v>55</v>
@@ -13939,7 +13939,7 @@
         <v>46205</v>
       </c>
       <c r="B306" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C306" t="s">
         <v>52</v>
@@ -13974,7 +13974,7 @@
         <v>46205</v>
       </c>
       <c r="B307" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C307" t="s">
         <v>29</v>
@@ -14009,7 +14009,7 @@
         <v>46205</v>
       </c>
       <c r="B308" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D308" t="s">
         <v>56</v>
@@ -14041,7 +14041,7 @@
         <v>46205</v>
       </c>
       <c r="B309" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C309" t="s">
         <v>40</v>
@@ -14076,7 +14076,7 @@
         <v>46205</v>
       </c>
       <c r="B310" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D310" t="s">
         <v>55</v>
@@ -14108,7 +14108,7 @@
         <v>46205</v>
       </c>
       <c r="B311" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C311" t="s">
         <v>40</v>
@@ -14143,7 +14143,7 @@
         <v>46205</v>
       </c>
       <c r="B312" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D312" t="s">
         <v>56</v>
@@ -14175,7 +14175,7 @@
         <v>46205</v>
       </c>
       <c r="B313" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C313" t="s">
         <v>40</v>
@@ -14210,7 +14210,7 @@
         <v>46205</v>
       </c>
       <c r="B314" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C314" t="s">
         <v>40</v>
@@ -14245,7 +14245,7 @@
         <v>46205</v>
       </c>
       <c r="B315" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C315" t="s">
         <v>24</v>
@@ -14280,7 +14280,7 @@
         <v>46205</v>
       </c>
       <c r="B316" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C316" t="s">
         <v>48</v>
@@ -14315,7 +14315,7 @@
         <v>46205</v>
       </c>
       <c r="B317" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C317" t="s">
         <v>27</v>
@@ -14350,7 +14350,7 @@
         <v>46205</v>
       </c>
       <c r="B318" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C318" t="s">
         <v>30</v>
@@ -14385,7 +14385,7 @@
         <v>46205</v>
       </c>
       <c r="B319" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C319" t="s">
         <v>18</v>
@@ -14420,7 +14420,7 @@
         <v>46205</v>
       </c>
       <c r="B320" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D320" t="s">
         <v>55</v>
@@ -14452,7 +14452,7 @@
         <v>46205</v>
       </c>
       <c r="B321" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D321" t="s">
         <v>56</v>
@@ -14484,7 +14484,7 @@
         <v>46205</v>
       </c>
       <c r="B322" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C322" t="s">
         <v>47</v>
@@ -14519,7 +14519,7 @@
         <v>46205</v>
       </c>
       <c r="B323" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C323" t="s">
         <v>54</v>
@@ -14554,7 +14554,7 @@
         <v>46205</v>
       </c>
       <c r="B324" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C324" t="s">
         <v>51</v>
@@ -14589,7 +14589,7 @@
         <v>46205</v>
       </c>
       <c r="B325" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C325" t="s">
         <v>54</v>

</xml_diff>

<commit_message>
Audiências: sync 2026-07-02 — 424 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -9167,7 +9167,7 @@
         <v>46203</v>
       </c>
       <c r="B164" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D164" t="s">
         <v>56</v>
@@ -9199,7 +9199,7 @@
         <v>46203</v>
       </c>
       <c r="B165" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D165" t="s">
         <v>56</v>
@@ -9231,7 +9231,7 @@
         <v>46203</v>
       </c>
       <c r="B166" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D166" t="s">
         <v>56</v>
@@ -9263,7 +9263,7 @@
         <v>46203</v>
       </c>
       <c r="B167" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D167" t="s">
         <v>56</v>
@@ -9295,7 +9295,7 @@
         <v>46203</v>
       </c>
       <c r="B168" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C168" t="s">
         <v>32</v>
@@ -9330,7 +9330,7 @@
         <v>46203</v>
       </c>
       <c r="B169" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C169" t="s">
         <v>29</v>
@@ -9365,7 +9365,7 @@
         <v>46203</v>
       </c>
       <c r="B170" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C170" t="s">
         <v>26</v>
@@ -9400,7 +9400,7 @@
         <v>46203</v>
       </c>
       <c r="B171" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D171" t="s">
         <v>55</v>
@@ -9432,7 +9432,7 @@
         <v>46203</v>
       </c>
       <c r="B172" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C172" t="s">
         <v>23</v>
@@ -9467,7 +9467,7 @@
         <v>46203</v>
       </c>
       <c r="B173" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C173" t="s">
         <v>38</v>
@@ -9502,7 +9502,7 @@
         <v>46203</v>
       </c>
       <c r="B174" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C174" t="s">
         <v>21</v>
@@ -9537,7 +9537,7 @@
         <v>46203</v>
       </c>
       <c r="B175" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D175" t="s">
         <v>56</v>
@@ -9569,7 +9569,7 @@
         <v>46203</v>
       </c>
       <c r="B176" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D176" t="s">
         <v>58</v>
@@ -9601,7 +9601,7 @@
         <v>46203</v>
       </c>
       <c r="B177" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D177" t="s">
         <v>58</v>
@@ -9633,7 +9633,7 @@
         <v>46203</v>
       </c>
       <c r="B178" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C178" t="s">
         <v>46</v>
@@ -9668,7 +9668,7 @@
         <v>46203</v>
       </c>
       <c r="B179" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D179" t="s">
         <v>55</v>
@@ -9700,7 +9700,7 @@
         <v>46203</v>
       </c>
       <c r="B180" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D180" t="s">
         <v>58</v>
@@ -9732,7 +9732,7 @@
         <v>46203</v>
       </c>
       <c r="B181" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D181" t="s">
         <v>56</v>
@@ -9764,7 +9764,7 @@
         <v>46203</v>
       </c>
       <c r="B182" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C182" t="s">
         <v>45</v>
@@ -9799,7 +9799,7 @@
         <v>46203</v>
       </c>
       <c r="B183" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D183" t="s">
         <v>55</v>
@@ -9831,7 +9831,7 @@
         <v>46203</v>
       </c>
       <c r="B184" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D184" t="s">
         <v>55</v>
@@ -9863,7 +9863,7 @@
         <v>46203</v>
       </c>
       <c r="B185" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C185" t="s">
         <v>50</v>
@@ -9898,7 +9898,7 @@
         <v>46203</v>
       </c>
       <c r="B186" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D186" t="s">
         <v>62</v>
@@ -9930,7 +9930,7 @@
         <v>46203</v>
       </c>
       <c r="B187" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D187" t="s">
         <v>58</v>
@@ -9962,7 +9962,7 @@
         <v>46203</v>
       </c>
       <c r="B188" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C188" t="s">
         <v>51</v>
@@ -9997,7 +9997,7 @@
         <v>46203</v>
       </c>
       <c r="B189" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D189" t="s">
         <v>55</v>
@@ -10029,7 +10029,7 @@
         <v>46203</v>
       </c>
       <c r="B190" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D190" t="s">
         <v>61</v>
@@ -10061,7 +10061,7 @@
         <v>46203</v>
       </c>
       <c r="B191" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D191" t="s">
         <v>61</v>
@@ -10093,7 +10093,7 @@
         <v>46203</v>
       </c>
       <c r="B192" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D192" t="s">
         <v>55</v>
@@ -10125,7 +10125,7 @@
         <v>46203</v>
       </c>
       <c r="B193" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C193" t="s">
         <v>18</v>
@@ -10160,7 +10160,7 @@
         <v>46203</v>
       </c>
       <c r="B194" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C194" t="s">
         <v>18</v>
@@ -10195,7 +10195,7 @@
         <v>46203</v>
       </c>
       <c r="B195" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C195" t="s">
         <v>44</v>
@@ -10230,7 +10230,7 @@
         <v>46203</v>
       </c>
       <c r="B196" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C196" t="s">
         <v>18</v>
@@ -10265,7 +10265,7 @@
         <v>46203</v>
       </c>
       <c r="B197" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C197" t="s">
         <v>18</v>
@@ -10300,7 +10300,7 @@
         <v>46203</v>
       </c>
       <c r="B198" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C198" t="s">
         <v>32</v>
@@ -10335,7 +10335,7 @@
         <v>46203</v>
       </c>
       <c r="B199" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D199" t="s">
         <v>56</v>
@@ -10367,7 +10367,7 @@
         <v>46203</v>
       </c>
       <c r="B200" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C200" t="s">
         <v>18</v>
@@ -10402,7 +10402,7 @@
         <v>46203</v>
       </c>
       <c r="B201" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C201" t="s">
         <v>50</v>
@@ -10437,7 +10437,7 @@
         <v>46203</v>
       </c>
       <c r="B202" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C202" t="s">
         <v>24</v>
@@ -10472,7 +10472,7 @@
         <v>46203</v>
       </c>
       <c r="B203" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C203" t="s">
         <v>16</v>
@@ -10507,7 +10507,7 @@
         <v>46203</v>
       </c>
       <c r="B204" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D204" t="s">
         <v>55</v>
@@ -10539,7 +10539,7 @@
         <v>46203</v>
       </c>
       <c r="B205" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C205" t="s">
         <v>24</v>
@@ -10574,7 +10574,7 @@
         <v>46203</v>
       </c>
       <c r="B206" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C206" t="s">
         <v>18</v>
@@ -10609,7 +10609,7 @@
         <v>46203</v>
       </c>
       <c r="B207" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D207" t="s">
         <v>55</v>
@@ -10641,7 +10641,7 @@
         <v>46203</v>
       </c>
       <c r="B208" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C208" t="s">
         <v>40</v>
@@ -10676,7 +10676,7 @@
         <v>46203</v>
       </c>
       <c r="B209" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C209" t="s">
         <v>24</v>
@@ -10711,7 +10711,7 @@
         <v>46203</v>
       </c>
       <c r="B210" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C210" t="s">
         <v>36</v>
@@ -10746,7 +10746,7 @@
         <v>46203</v>
       </c>
       <c r="B211" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D211" t="s">
         <v>56</v>
@@ -10778,7 +10778,7 @@
         <v>46203</v>
       </c>
       <c r="B212" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D212" t="s">
         <v>55</v>
@@ -10810,7 +10810,7 @@
         <v>46203</v>
       </c>
       <c r="B213" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D213" t="s">
         <v>61</v>
@@ -10842,7 +10842,7 @@
         <v>46203</v>
       </c>
       <c r="B214" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D214" t="s">
         <v>56</v>
@@ -10874,7 +10874,7 @@
         <v>46203</v>
       </c>
       <c r="B215" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D215" t="s">
         <v>56</v>
@@ -10906,7 +10906,7 @@
         <v>46203</v>
       </c>
       <c r="B216" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D216" t="s">
         <v>57</v>
@@ -10938,7 +10938,7 @@
         <v>46203</v>
       </c>
       <c r="B217" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D217" t="s">
         <v>56</v>
@@ -10970,7 +10970,7 @@
         <v>46203</v>
       </c>
       <c r="B218" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D218" t="s">
         <v>55</v>
@@ -11002,7 +11002,7 @@
         <v>46203</v>
       </c>
       <c r="B219" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D219" t="s">
         <v>58</v>
@@ -11034,7 +11034,7 @@
         <v>46203</v>
       </c>
       <c r="B220" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C220" t="s">
         <v>51</v>
@@ -11069,7 +11069,7 @@
         <v>46203</v>
       </c>
       <c r="B221" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D221" t="s">
         <v>63</v>
@@ -11101,7 +11101,7 @@
         <v>46203</v>
       </c>
       <c r="B222" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D222" t="s">
         <v>55</v>
@@ -11133,7 +11133,7 @@
         <v>46203</v>
       </c>
       <c r="B223" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C223" t="s">
         <v>35</v>
@@ -11168,7 +11168,7 @@
         <v>46203</v>
       </c>
       <c r="B224" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D224" t="s">
         <v>55</v>
@@ -11200,7 +11200,7 @@
         <v>46203</v>
       </c>
       <c r="B225" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D225" t="s">
         <v>55</v>
@@ -11232,7 +11232,7 @@
         <v>46203</v>
       </c>
       <c r="B226" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D226" t="s">
         <v>55</v>
@@ -11264,7 +11264,7 @@
         <v>46203</v>
       </c>
       <c r="B227" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C227" t="s">
         <v>30</v>
@@ -11299,7 +11299,7 @@
         <v>46203</v>
       </c>
       <c r="B228" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D228" t="s">
         <v>55</v>
@@ -11331,7 +11331,7 @@
         <v>46203</v>
       </c>
       <c r="B229" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C229" t="s">
         <v>30</v>
@@ -11366,7 +11366,7 @@
         <v>46203</v>
       </c>
       <c r="B230" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C230" t="s">
         <v>38</v>
@@ -11401,7 +11401,7 @@
         <v>46203</v>
       </c>
       <c r="B231" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C231" t="s">
         <v>37</v>
@@ -11436,7 +11436,7 @@
         <v>46203</v>
       </c>
       <c r="B232" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D232" t="s">
         <v>56</v>
@@ -11468,7 +11468,7 @@
         <v>46203</v>
       </c>
       <c r="B233" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C233" t="s">
         <v>24</v>
@@ -11503,7 +11503,7 @@
         <v>46203</v>
       </c>
       <c r="B234" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C234" t="s">
         <v>40</v>
@@ -11538,7 +11538,7 @@
         <v>46203</v>
       </c>
       <c r="B235" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C235" t="s">
         <v>40</v>
@@ -11573,7 +11573,7 @@
         <v>46203</v>
       </c>
       <c r="B236" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C236" t="s">
         <v>27</v>
@@ -11608,7 +11608,7 @@
         <v>46203</v>
       </c>
       <c r="B237" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C237" t="s">
         <v>42</v>
@@ -11643,7 +11643,7 @@
         <v>46203</v>
       </c>
       <c r="B238" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C238" t="s">
         <v>16</v>
@@ -11678,7 +11678,7 @@
         <v>46203</v>
       </c>
       <c r="B239" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C239" t="s">
         <v>40</v>
@@ -11713,7 +11713,7 @@
         <v>46203</v>
       </c>
       <c r="B240" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C240" t="s">
         <v>46</v>
@@ -11748,7 +11748,7 @@
         <v>46203</v>
       </c>
       <c r="B241" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D241" t="s">
         <v>57</v>
@@ -11780,7 +11780,7 @@
         <v>46203</v>
       </c>
       <c r="B242" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C242" t="s">
         <v>49</v>
@@ -11815,7 +11815,7 @@
         <v>46203</v>
       </c>
       <c r="B243" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C243" t="s">
         <v>18</v>
@@ -11850,7 +11850,7 @@
         <v>46203</v>
       </c>
       <c r="B244" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D244" t="s">
         <v>56</v>
@@ -11882,7 +11882,7 @@
         <v>46203</v>
       </c>
       <c r="B245" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D245" t="s">
         <v>56</v>
@@ -11914,7 +11914,7 @@
         <v>46203</v>
       </c>
       <c r="B246" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D246" t="s">
         <v>56</v>
@@ -11946,7 +11946,7 @@
         <v>46203</v>
       </c>
       <c r="B247" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D247" t="s">
         <v>56</v>
@@ -11978,7 +11978,7 @@
         <v>46203</v>
       </c>
       <c r="B248" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D248" t="s">
         <v>56</v>
@@ -12010,7 +12010,7 @@
         <v>46203</v>
       </c>
       <c r="B249" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D249" t="s">
         <v>55</v>
@@ -12042,7 +12042,7 @@
         <v>46203</v>
       </c>
       <c r="B250" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D250" t="s">
         <v>56</v>
@@ -12074,7 +12074,7 @@
         <v>46203</v>
       </c>
       <c r="B251" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D251" t="s">
         <v>56</v>
@@ -12106,7 +12106,7 @@
         <v>46204</v>
       </c>
       <c r="B252" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C252" t="s">
         <v>52</v>
@@ -12141,7 +12141,7 @@
         <v>46204</v>
       </c>
       <c r="B253" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C253" t="s">
         <v>19</v>
@@ -12176,7 +12176,7 @@
         <v>46204</v>
       </c>
       <c r="B254" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C254" t="s">
         <v>18</v>
@@ -12211,7 +12211,7 @@
         <v>46204</v>
       </c>
       <c r="B255" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C255" t="s">
         <v>19</v>
@@ -12246,7 +12246,7 @@
         <v>46204</v>
       </c>
       <c r="B256" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C256" t="s">
         <v>26</v>
@@ -12281,7 +12281,7 @@
         <v>46204</v>
       </c>
       <c r="B257" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C257" t="s">
         <v>35</v>
@@ -12316,7 +12316,7 @@
         <v>46204</v>
       </c>
       <c r="B258" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C258" t="s">
         <v>48</v>
@@ -12351,7 +12351,7 @@
         <v>46204</v>
       </c>
       <c r="B259" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C259" t="s">
         <v>40</v>
@@ -12386,7 +12386,7 @@
         <v>46204</v>
       </c>
       <c r="B260" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C260" t="s">
         <v>53</v>
@@ -12421,7 +12421,7 @@
         <v>46204</v>
       </c>
       <c r="B261" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D261" t="s">
         <v>58</v>
@@ -12453,7 +12453,7 @@
         <v>46204</v>
       </c>
       <c r="B262" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C262" t="s">
         <v>39</v>
@@ -12488,7 +12488,7 @@
         <v>46204</v>
       </c>
       <c r="B263" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C263" t="s">
         <v>29</v>
@@ -12523,7 +12523,7 @@
         <v>46204</v>
       </c>
       <c r="B264" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D264" t="s">
         <v>58</v>
@@ -12555,7 +12555,7 @@
         <v>46204</v>
       </c>
       <c r="B265" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C265" t="s">
         <v>18</v>
@@ -12590,7 +12590,7 @@
         <v>46204</v>
       </c>
       <c r="B266" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C266" t="s">
         <v>32</v>
@@ -12625,7 +12625,7 @@
         <v>46204</v>
       </c>
       <c r="B267" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C267" t="s">
         <v>16</v>
@@ -12660,7 +12660,7 @@
         <v>46204</v>
       </c>
       <c r="B268" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C268" t="s">
         <v>33</v>
@@ -12695,7 +12695,7 @@
         <v>46204</v>
       </c>
       <c r="B269" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D269" t="s">
         <v>55</v>
@@ -12727,7 +12727,7 @@
         <v>46204</v>
       </c>
       <c r="B270" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D270" t="s">
         <v>55</v>
@@ -12759,7 +12759,7 @@
         <v>46204</v>
       </c>
       <c r="B271" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D271" t="s">
         <v>55</v>
@@ -12791,7 +12791,7 @@
         <v>46204</v>
       </c>
       <c r="B272" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D272" t="s">
         <v>56</v>
@@ -12823,7 +12823,7 @@
         <v>46204</v>
       </c>
       <c r="B273" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C273" t="s">
         <v>27</v>
@@ -12858,7 +12858,7 @@
         <v>46204</v>
       </c>
       <c r="B274" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D274" t="s">
         <v>56</v>
@@ -12890,7 +12890,7 @@
         <v>46204</v>
       </c>
       <c r="B275" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D275" t="s">
         <v>56</v>
@@ -12922,7 +12922,7 @@
         <v>46204</v>
       </c>
       <c r="B276" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C276" t="s">
         <v>25</v>
@@ -12957,7 +12957,7 @@
         <v>46204</v>
       </c>
       <c r="B277" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C277" t="s">
         <v>49</v>
@@ -12992,7 +12992,7 @@
         <v>46204</v>
       </c>
       <c r="B278" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D278" t="s">
         <v>56</v>
@@ -13024,7 +13024,7 @@
         <v>46204</v>
       </c>
       <c r="B279" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D279" t="s">
         <v>56</v>
@@ -13056,7 +13056,7 @@
         <v>46204</v>
       </c>
       <c r="B280" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D280" t="s">
         <v>56</v>
@@ -13088,7 +13088,7 @@
         <v>46204</v>
       </c>
       <c r="B281" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C281" t="s">
         <v>40</v>
@@ -13123,7 +13123,7 @@
         <v>46204</v>
       </c>
       <c r="B282" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D282" t="s">
         <v>55</v>
@@ -13155,7 +13155,7 @@
         <v>46204</v>
       </c>
       <c r="B283" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C283" t="s">
         <v>38</v>
@@ -13190,7 +13190,7 @@
         <v>46204</v>
       </c>
       <c r="B284" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C284" t="s">
         <v>36</v>
@@ -13225,7 +13225,7 @@
         <v>46204</v>
       </c>
       <c r="B285" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C285" t="s">
         <v>45</v>
@@ -13260,7 +13260,7 @@
         <v>46204</v>
       </c>
       <c r="B286" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C286" t="s">
         <v>40</v>
@@ -13295,7 +13295,7 @@
         <v>46204</v>
       </c>
       <c r="B287" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C287" t="s">
         <v>18</v>
@@ -13330,7 +13330,7 @@
         <v>46204</v>
       </c>
       <c r="B288" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C288" t="s">
         <v>40</v>
@@ -13365,7 +13365,7 @@
         <v>46204</v>
       </c>
       <c r="B289" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C289" t="s">
         <v>29</v>
@@ -13400,7 +13400,7 @@
         <v>46204</v>
       </c>
       <c r="B290" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C290" t="s">
         <v>23</v>
@@ -13435,7 +13435,7 @@
         <v>46204</v>
       </c>
       <c r="B291" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C291" t="s">
         <v>43</v>
@@ -13470,7 +13470,7 @@
         <v>46204</v>
       </c>
       <c r="B292" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C292" t="s">
         <v>53</v>
@@ -13505,7 +13505,7 @@
         <v>46204</v>
       </c>
       <c r="B293" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D293" t="s">
         <v>58</v>
@@ -13537,7 +13537,7 @@
         <v>46205</v>
       </c>
       <c r="B294" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D294" t="s">
         <v>56</v>
@@ -13569,7 +13569,7 @@
         <v>46205</v>
       </c>
       <c r="B295" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D295" t="s">
         <v>56</v>
@@ -13601,7 +13601,7 @@
         <v>46205</v>
       </c>
       <c r="B296" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D296" t="s">
         <v>56</v>
@@ -13633,7 +13633,7 @@
         <v>46205</v>
       </c>
       <c r="B297" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D297" t="s">
         <v>56</v>
@@ -13665,7 +13665,7 @@
         <v>46205</v>
       </c>
       <c r="B298" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C298" t="s">
         <v>44</v>
@@ -13700,7 +13700,7 @@
         <v>46205</v>
       </c>
       <c r="B299" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C299" t="s">
         <v>26</v>
@@ -13735,7 +13735,7 @@
         <v>46205</v>
       </c>
       <c r="B300" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C300" t="s">
         <v>43</v>
@@ -13770,7 +13770,7 @@
         <v>46205</v>
       </c>
       <c r="B301" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C301" t="s">
         <v>18</v>
@@ -13805,7 +13805,7 @@
         <v>46205</v>
       </c>
       <c r="B302" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D302" t="s">
         <v>55</v>
@@ -13837,7 +13837,7 @@
         <v>46205</v>
       </c>
       <c r="B303" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C303" t="s">
         <v>53</v>
@@ -13872,7 +13872,7 @@
         <v>46205</v>
       </c>
       <c r="B304" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C304" t="s">
         <v>23</v>
@@ -13907,7 +13907,7 @@
         <v>46205</v>
       </c>
       <c r="B305" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D305" t="s">
         <v>55</v>
@@ -13939,7 +13939,7 @@
         <v>46205</v>
       </c>
       <c r="B306" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C306" t="s">
         <v>52</v>
@@ -13974,7 +13974,7 @@
         <v>46205</v>
       </c>
       <c r="B307" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C307" t="s">
         <v>29</v>
@@ -14009,7 +14009,7 @@
         <v>46205</v>
       </c>
       <c r="B308" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D308" t="s">
         <v>56</v>
@@ -14041,7 +14041,7 @@
         <v>46205</v>
       </c>
       <c r="B309" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C309" t="s">
         <v>40</v>
@@ -14076,7 +14076,7 @@
         <v>46205</v>
       </c>
       <c r="B310" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D310" t="s">
         <v>55</v>
@@ -14108,7 +14108,7 @@
         <v>46205</v>
       </c>
       <c r="B311" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C311" t="s">
         <v>40</v>
@@ -14143,7 +14143,7 @@
         <v>46205</v>
       </c>
       <c r="B312" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D312" t="s">
         <v>56</v>
@@ -14175,7 +14175,7 @@
         <v>46205</v>
       </c>
       <c r="B313" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C313" t="s">
         <v>40</v>
@@ -14210,7 +14210,7 @@
         <v>46205</v>
       </c>
       <c r="B314" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C314" t="s">
         <v>40</v>
@@ -14245,7 +14245,7 @@
         <v>46205</v>
       </c>
       <c r="B315" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C315" t="s">
         <v>24</v>
@@ -14280,7 +14280,7 @@
         <v>46205</v>
       </c>
       <c r="B316" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C316" t="s">
         <v>48</v>
@@ -14315,7 +14315,7 @@
         <v>46205</v>
       </c>
       <c r="B317" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C317" t="s">
         <v>27</v>
@@ -14350,7 +14350,7 @@
         <v>46205</v>
       </c>
       <c r="B318" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C318" t="s">
         <v>30</v>
@@ -14385,7 +14385,7 @@
         <v>46205</v>
       </c>
       <c r="B319" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C319" t="s">
         <v>18</v>
@@ -14420,7 +14420,7 @@
         <v>46205</v>
       </c>
       <c r="B320" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D320" t="s">
         <v>55</v>
@@ -14452,7 +14452,7 @@
         <v>46205</v>
       </c>
       <c r="B321" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D321" t="s">
         <v>56</v>
@@ -14484,7 +14484,7 @@
         <v>46205</v>
       </c>
       <c r="B322" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C322" t="s">
         <v>47</v>
@@ -14519,7 +14519,7 @@
         <v>46205</v>
       </c>
       <c r="B323" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C323" t="s">
         <v>54</v>
@@ -14554,7 +14554,7 @@
         <v>46205</v>
       </c>
       <c r="B324" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C324" t="s">
         <v>51</v>
@@ -14589,7 +14589,7 @@
         <v>46205</v>
       </c>
       <c r="B325" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C325" t="s">
         <v>54</v>
@@ -14624,7 +14624,7 @@
         <v>46206</v>
       </c>
       <c r="B326" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D326" t="s">
         <v>58</v>
@@ -14656,7 +14656,7 @@
         <v>46206</v>
       </c>
       <c r="B327" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D327" t="s">
         <v>57</v>
@@ -14688,7 +14688,7 @@
         <v>46206</v>
       </c>
       <c r="B328" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C328" t="s">
         <v>18</v>
@@ -14723,7 +14723,7 @@
         <v>46206</v>
       </c>
       <c r="B329" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C329" t="s">
         <v>37</v>
@@ -14758,7 +14758,7 @@
         <v>46206</v>
       </c>
       <c r="B330" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C330" t="s">
         <v>37</v>
@@ -14793,7 +14793,7 @@
         <v>46206</v>
       </c>
       <c r="B331" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C331" t="s">
         <v>37</v>
@@ -14828,7 +14828,7 @@
         <v>46206</v>
       </c>
       <c r="B332" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C332" t="s">
         <v>29</v>
@@ -14863,7 +14863,7 @@
         <v>46206</v>
       </c>
       <c r="B333" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C333" t="s">
         <v>24</v>
@@ -14898,7 +14898,7 @@
         <v>46206</v>
       </c>
       <c r="B334" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D334" t="s">
         <v>56</v>
@@ -14930,7 +14930,7 @@
         <v>46206</v>
       </c>
       <c r="B335" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D335" t="s">
         <v>56</v>
@@ -14962,7 +14962,7 @@
         <v>46206</v>
       </c>
       <c r="B336" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D336" t="s">
         <v>56</v>
@@ -14994,7 +14994,7 @@
         <v>46206</v>
       </c>
       <c r="B337" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D337" t="s">
         <v>63</v>
@@ -15026,7 +15026,7 @@
         <v>46206</v>
       </c>
       <c r="B338" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D338" t="s">
         <v>61</v>
@@ -15058,7 +15058,7 @@
         <v>46206</v>
       </c>
       <c r="B339" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D339" t="s">
         <v>56</v>

</xml_diff>

<commit_message>
Audiências: sync 2026-07-03 — 424 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -12106,7 +12106,7 @@
         <v>46204</v>
       </c>
       <c r="B252" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C252" t="s">
         <v>52</v>
@@ -12141,7 +12141,7 @@
         <v>46204</v>
       </c>
       <c r="B253" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C253" t="s">
         <v>19</v>
@@ -12176,7 +12176,7 @@
         <v>46204</v>
       </c>
       <c r="B254" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C254" t="s">
         <v>18</v>
@@ -12211,7 +12211,7 @@
         <v>46204</v>
       </c>
       <c r="B255" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C255" t="s">
         <v>19</v>
@@ -12246,7 +12246,7 @@
         <v>46204</v>
       </c>
       <c r="B256" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C256" t="s">
         <v>26</v>
@@ -12281,7 +12281,7 @@
         <v>46204</v>
       </c>
       <c r="B257" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C257" t="s">
         <v>35</v>
@@ -12316,7 +12316,7 @@
         <v>46204</v>
       </c>
       <c r="B258" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C258" t="s">
         <v>48</v>
@@ -12351,7 +12351,7 @@
         <v>46204</v>
       </c>
       <c r="B259" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C259" t="s">
         <v>40</v>
@@ -12386,7 +12386,7 @@
         <v>46204</v>
       </c>
       <c r="B260" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C260" t="s">
         <v>53</v>
@@ -12421,7 +12421,7 @@
         <v>46204</v>
       </c>
       <c r="B261" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D261" t="s">
         <v>58</v>
@@ -12453,7 +12453,7 @@
         <v>46204</v>
       </c>
       <c r="B262" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C262" t="s">
         <v>39</v>
@@ -12488,7 +12488,7 @@
         <v>46204</v>
       </c>
       <c r="B263" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C263" t="s">
         <v>29</v>
@@ -12523,7 +12523,7 @@
         <v>46204</v>
       </c>
       <c r="B264" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D264" t="s">
         <v>58</v>
@@ -12555,7 +12555,7 @@
         <v>46204</v>
       </c>
       <c r="B265" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C265" t="s">
         <v>18</v>
@@ -12590,7 +12590,7 @@
         <v>46204</v>
       </c>
       <c r="B266" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C266" t="s">
         <v>32</v>
@@ -12625,7 +12625,7 @@
         <v>46204</v>
       </c>
       <c r="B267" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C267" t="s">
         <v>16</v>
@@ -12660,7 +12660,7 @@
         <v>46204</v>
       </c>
       <c r="B268" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C268" t="s">
         <v>33</v>
@@ -12695,7 +12695,7 @@
         <v>46204</v>
       </c>
       <c r="B269" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D269" t="s">
         <v>55</v>
@@ -12727,7 +12727,7 @@
         <v>46204</v>
       </c>
       <c r="B270" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D270" t="s">
         <v>55</v>
@@ -12759,7 +12759,7 @@
         <v>46204</v>
       </c>
       <c r="B271" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D271" t="s">
         <v>55</v>
@@ -12791,7 +12791,7 @@
         <v>46204</v>
       </c>
       <c r="B272" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D272" t="s">
         <v>56</v>
@@ -12823,7 +12823,7 @@
         <v>46204</v>
       </c>
       <c r="B273" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C273" t="s">
         <v>27</v>
@@ -12858,7 +12858,7 @@
         <v>46204</v>
       </c>
       <c r="B274" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D274" t="s">
         <v>56</v>
@@ -12890,7 +12890,7 @@
         <v>46204</v>
       </c>
       <c r="B275" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D275" t="s">
         <v>56</v>
@@ -12922,7 +12922,7 @@
         <v>46204</v>
       </c>
       <c r="B276" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C276" t="s">
         <v>25</v>
@@ -12957,7 +12957,7 @@
         <v>46204</v>
       </c>
       <c r="B277" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C277" t="s">
         <v>49</v>
@@ -12992,7 +12992,7 @@
         <v>46204</v>
       </c>
       <c r="B278" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D278" t="s">
         <v>56</v>
@@ -13024,7 +13024,7 @@
         <v>46204</v>
       </c>
       <c r="B279" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D279" t="s">
         <v>56</v>
@@ -13056,7 +13056,7 @@
         <v>46204</v>
       </c>
       <c r="B280" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D280" t="s">
         <v>56</v>
@@ -13088,7 +13088,7 @@
         <v>46204</v>
       </c>
       <c r="B281" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C281" t="s">
         <v>40</v>
@@ -13123,7 +13123,7 @@
         <v>46204</v>
       </c>
       <c r="B282" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D282" t="s">
         <v>55</v>
@@ -13155,7 +13155,7 @@
         <v>46204</v>
       </c>
       <c r="B283" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C283" t="s">
         <v>38</v>
@@ -13190,7 +13190,7 @@
         <v>46204</v>
       </c>
       <c r="B284" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C284" t="s">
         <v>36</v>
@@ -13225,7 +13225,7 @@
         <v>46204</v>
       </c>
       <c r="B285" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C285" t="s">
         <v>45</v>
@@ -13260,7 +13260,7 @@
         <v>46204</v>
       </c>
       <c r="B286" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C286" t="s">
         <v>40</v>
@@ -13295,7 +13295,7 @@
         <v>46204</v>
       </c>
       <c r="B287" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C287" t="s">
         <v>18</v>
@@ -13330,7 +13330,7 @@
         <v>46204</v>
       </c>
       <c r="B288" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C288" t="s">
         <v>40</v>
@@ -13365,7 +13365,7 @@
         <v>46204</v>
       </c>
       <c r="B289" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C289" t="s">
         <v>29</v>
@@ -13400,7 +13400,7 @@
         <v>46204</v>
       </c>
       <c r="B290" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C290" t="s">
         <v>23</v>
@@ -13435,7 +13435,7 @@
         <v>46204</v>
       </c>
       <c r="B291" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C291" t="s">
         <v>43</v>
@@ -13470,7 +13470,7 @@
         <v>46204</v>
       </c>
       <c r="B292" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C292" t="s">
         <v>53</v>
@@ -13505,7 +13505,7 @@
         <v>46204</v>
       </c>
       <c r="B293" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D293" t="s">
         <v>58</v>
@@ -13537,7 +13537,7 @@
         <v>46205</v>
       </c>
       <c r="B294" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D294" t="s">
         <v>56</v>
@@ -13569,7 +13569,7 @@
         <v>46205</v>
       </c>
       <c r="B295" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D295" t="s">
         <v>56</v>
@@ -13601,7 +13601,7 @@
         <v>46205</v>
       </c>
       <c r="B296" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D296" t="s">
         <v>56</v>
@@ -13633,7 +13633,7 @@
         <v>46205</v>
       </c>
       <c r="B297" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D297" t="s">
         <v>56</v>
@@ -13665,7 +13665,7 @@
         <v>46205</v>
       </c>
       <c r="B298" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C298" t="s">
         <v>44</v>
@@ -13700,7 +13700,7 @@
         <v>46205</v>
       </c>
       <c r="B299" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C299" t="s">
         <v>26</v>
@@ -13735,7 +13735,7 @@
         <v>46205</v>
       </c>
       <c r="B300" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C300" t="s">
         <v>43</v>
@@ -13770,7 +13770,7 @@
         <v>46205</v>
       </c>
       <c r="B301" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C301" t="s">
         <v>18</v>
@@ -13805,7 +13805,7 @@
         <v>46205</v>
       </c>
       <c r="B302" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D302" t="s">
         <v>55</v>
@@ -13837,7 +13837,7 @@
         <v>46205</v>
       </c>
       <c r="B303" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C303" t="s">
         <v>53</v>
@@ -13872,7 +13872,7 @@
         <v>46205</v>
       </c>
       <c r="B304" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C304" t="s">
         <v>23</v>
@@ -13907,7 +13907,7 @@
         <v>46205</v>
       </c>
       <c r="B305" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D305" t="s">
         <v>55</v>
@@ -13939,7 +13939,7 @@
         <v>46205</v>
       </c>
       <c r="B306" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C306" t="s">
         <v>52</v>
@@ -13974,7 +13974,7 @@
         <v>46205</v>
       </c>
       <c r="B307" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C307" t="s">
         <v>29</v>
@@ -14009,7 +14009,7 @@
         <v>46205</v>
       </c>
       <c r="B308" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D308" t="s">
         <v>56</v>
@@ -14041,7 +14041,7 @@
         <v>46205</v>
       </c>
       <c r="B309" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C309" t="s">
         <v>40</v>
@@ -14076,7 +14076,7 @@
         <v>46205</v>
       </c>
       <c r="B310" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D310" t="s">
         <v>55</v>
@@ -14108,7 +14108,7 @@
         <v>46205</v>
       </c>
       <c r="B311" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C311" t="s">
         <v>40</v>
@@ -14143,7 +14143,7 @@
         <v>46205</v>
       </c>
       <c r="B312" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D312" t="s">
         <v>56</v>
@@ -14175,7 +14175,7 @@
         <v>46205</v>
       </c>
       <c r="B313" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C313" t="s">
         <v>40</v>
@@ -14210,7 +14210,7 @@
         <v>46205</v>
       </c>
       <c r="B314" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C314" t="s">
         <v>40</v>
@@ -14245,7 +14245,7 @@
         <v>46205</v>
       </c>
       <c r="B315" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C315" t="s">
         <v>24</v>
@@ -14280,7 +14280,7 @@
         <v>46205</v>
       </c>
       <c r="B316" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C316" t="s">
         <v>48</v>
@@ -14315,7 +14315,7 @@
         <v>46205</v>
       </c>
       <c r="B317" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C317" t="s">
         <v>27</v>
@@ -14350,7 +14350,7 @@
         <v>46205</v>
       </c>
       <c r="B318" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C318" t="s">
         <v>30</v>
@@ -14385,7 +14385,7 @@
         <v>46205</v>
       </c>
       <c r="B319" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C319" t="s">
         <v>18</v>
@@ -14420,7 +14420,7 @@
         <v>46205</v>
       </c>
       <c r="B320" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D320" t="s">
         <v>55</v>
@@ -14452,7 +14452,7 @@
         <v>46205</v>
       </c>
       <c r="B321" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D321" t="s">
         <v>56</v>
@@ -14484,7 +14484,7 @@
         <v>46205</v>
       </c>
       <c r="B322" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C322" t="s">
         <v>47</v>
@@ -14519,7 +14519,7 @@
         <v>46205</v>
       </c>
       <c r="B323" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C323" t="s">
         <v>54</v>
@@ -14554,7 +14554,7 @@
         <v>46205</v>
       </c>
       <c r="B324" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C324" t="s">
         <v>51</v>
@@ -14589,7 +14589,7 @@
         <v>46205</v>
       </c>
       <c r="B325" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C325" t="s">
         <v>54</v>
@@ -14624,7 +14624,7 @@
         <v>46206</v>
       </c>
       <c r="B326" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D326" t="s">
         <v>58</v>
@@ -14656,7 +14656,7 @@
         <v>46206</v>
       </c>
       <c r="B327" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D327" t="s">
         <v>57</v>
@@ -14688,7 +14688,7 @@
         <v>46206</v>
       </c>
       <c r="B328" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C328" t="s">
         <v>18</v>
@@ -14723,7 +14723,7 @@
         <v>46206</v>
       </c>
       <c r="B329" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C329" t="s">
         <v>37</v>
@@ -14758,7 +14758,7 @@
         <v>46206</v>
       </c>
       <c r="B330" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C330" t="s">
         <v>37</v>
@@ -14793,7 +14793,7 @@
         <v>46206</v>
       </c>
       <c r="B331" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C331" t="s">
         <v>37</v>
@@ -14828,7 +14828,7 @@
         <v>46206</v>
       </c>
       <c r="B332" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C332" t="s">
         <v>29</v>
@@ -14863,7 +14863,7 @@
         <v>46206</v>
       </c>
       <c r="B333" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C333" t="s">
         <v>24</v>
@@ -14898,7 +14898,7 @@
         <v>46206</v>
       </c>
       <c r="B334" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D334" t="s">
         <v>56</v>
@@ -14930,7 +14930,7 @@
         <v>46206</v>
       </c>
       <c r="B335" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D335" t="s">
         <v>56</v>
@@ -14962,7 +14962,7 @@
         <v>46206</v>
       </c>
       <c r="B336" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D336" t="s">
         <v>56</v>
@@ -14994,7 +14994,7 @@
         <v>46206</v>
       </c>
       <c r="B337" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D337" t="s">
         <v>63</v>
@@ -15026,7 +15026,7 @@
         <v>46206</v>
       </c>
       <c r="B338" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D338" t="s">
         <v>61</v>
@@ -15058,7 +15058,7 @@
         <v>46206</v>
       </c>
       <c r="B339" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D339" t="s">
         <v>56</v>
@@ -15090,7 +15090,7 @@
         <v>46209</v>
       </c>
       <c r="B340" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C340" t="s">
         <v>40</v>
@@ -15125,7 +15125,7 @@
         <v>46209</v>
       </c>
       <c r="B341" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C341" t="s">
         <v>45</v>
@@ -15160,7 +15160,7 @@
         <v>46209</v>
       </c>
       <c r="B342" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C342" t="s">
         <v>40</v>
@@ -15195,7 +15195,7 @@
         <v>46209</v>
       </c>
       <c r="B343" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C343" t="s">
         <v>40</v>
@@ -15230,7 +15230,7 @@
         <v>46209</v>
       </c>
       <c r="B344" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C344" t="s">
         <v>29</v>
@@ -15265,7 +15265,7 @@
         <v>46209</v>
       </c>
       <c r="B345" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C345" t="s">
         <v>19</v>
@@ -15300,7 +15300,7 @@
         <v>46209</v>
       </c>
       <c r="B346" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C346" t="s">
         <v>19</v>
@@ -15335,7 +15335,7 @@
         <v>46209</v>
       </c>
       <c r="B347" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C347" t="s">
         <v>35</v>
@@ -15370,7 +15370,7 @@
         <v>46209</v>
       </c>
       <c r="B348" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C348" t="s">
         <v>40</v>
@@ -15405,7 +15405,7 @@
         <v>46209</v>
       </c>
       <c r="B349" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C349" t="s">
         <v>40</v>
@@ -15440,7 +15440,7 @@
         <v>46209</v>
       </c>
       <c r="B350" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C350" t="s">
         <v>40</v>
@@ -15475,7 +15475,7 @@
         <v>46209</v>
       </c>
       <c r="B351" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C351" t="s">
         <v>19</v>
@@ -15510,7 +15510,7 @@
         <v>46209</v>
       </c>
       <c r="B352" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C352" t="s">
         <v>40</v>
@@ -15545,7 +15545,7 @@
         <v>46209</v>
       </c>
       <c r="B353" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C353" t="s">
         <v>40</v>
@@ -15580,7 +15580,7 @@
         <v>46209</v>
       </c>
       <c r="B354" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C354" t="s">
         <v>29</v>
@@ -15615,7 +15615,7 @@
         <v>46209</v>
       </c>
       <c r="B355" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C355" t="s">
         <v>41</v>
@@ -15650,7 +15650,7 @@
         <v>46209</v>
       </c>
       <c r="B356" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C356" t="s">
         <v>48</v>
@@ -15685,7 +15685,7 @@
         <v>46209</v>
       </c>
       <c r="B357" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C357" t="s">
         <v>40</v>
@@ -15720,7 +15720,7 @@
         <v>46209</v>
       </c>
       <c r="B358" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C358" t="s">
         <v>40</v>
@@ -15755,7 +15755,7 @@
         <v>46209</v>
       </c>
       <c r="B359" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C359" t="s">
         <v>43</v>
@@ -15790,7 +15790,7 @@
         <v>46209</v>
       </c>
       <c r="B360" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C360" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Audiências: sync 2026-07-21 — 29 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="144">
   <si>
     <t>data</t>
   </si>
@@ -49,211 +49,328 @@
     <t>horario</t>
   </si>
   <si>
-    <t>Fatal</t>
-  </si>
-  <si>
-    <t>BCF</t>
+    <t>D-1</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>JNE</t>
+  </si>
+  <si>
+    <t>RCF</t>
+  </si>
+  <si>
+    <t>TLI</t>
   </si>
   <si>
     <t>RYL</t>
   </si>
   <si>
-    <t>Correspondente - Carlos Florian</t>
-  </si>
-  <si>
-    <t>NBG</t>
+    <t>Correspondente - Ana</t>
+  </si>
+  <si>
+    <t>Correspondente - Zalaf</t>
+  </si>
+  <si>
+    <t>RRU</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>DPR</t>
+  </si>
+  <si>
+    <t>Correspondente - Hebert</t>
   </si>
   <si>
     <t>ARC</t>
   </si>
   <si>
+    <t>JQS</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>ANB</t>
+  </si>
+  <si>
     <t>GSM</t>
   </si>
   <si>
-    <t>JPE</t>
-  </si>
-  <si>
-    <t>MBF</t>
-  </si>
-  <si>
-    <t>FCG</t>
-  </si>
-  <si>
-    <t>BSO</t>
-  </si>
-  <si>
-    <t>CAL</t>
-  </si>
-  <si>
-    <t>TFR</t>
+    <t>PSI</t>
+  </si>
+  <si>
+    <t>TAM</t>
+  </si>
+  <si>
+    <t>Grupo B1</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
+    <t>Grupo A3</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>Grupo D1</t>
+  </si>
+  <si>
+    <t>Grupo C</t>
   </si>
   <si>
     <t>Grupo B2</t>
   </si>
   <si>
-    <t>Grupo E2</t>
-  </si>
-  <si>
-    <t>Grupo E1</t>
-  </si>
-  <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>Grupo C</t>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda</t>
+  </si>
+  <si>
+    <t>Whirlpool S.A.</t>
+  </si>
+  <si>
+    <t>Mahle Behr Gerenciamento Térmico Brasil Ltda.</t>
+  </si>
+  <si>
+    <t>Guariroba Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Mahle Metal Leve S.A.</t>
+  </si>
+  <si>
+    <t>Viterra Bioenergia S.A.</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Pilkington Brasil Ltda.</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
+  </si>
+  <si>
+    <t>Americanas S.A.</t>
+  </si>
+  <si>
+    <t>Companhia Act De Participacoes E Companhia Aix De Participacoes</t>
+  </si>
+  <si>
+    <t>Santa Juliana Bioenergia Ltda.</t>
   </si>
   <si>
     <t>Embraer S.A.</t>
   </si>
   <si>
-    <t>Fertilizantes Tocantins S.A</t>
-  </si>
-  <si>
-    <t>Syngenta Proteção De Cultivos Ltda.</t>
-  </si>
-  <si>
-    <t>Salitre Fertilizantes Ltda</t>
-  </si>
-  <si>
-    <t>Moema Bioenergia S.A. - Moema</t>
-  </si>
-  <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Ouroeste Bioenergia LTDA.</t>
-  </si>
-  <si>
-    <t>Mahle Metal Leve S.A.</t>
-  </si>
-  <si>
-    <t>Telefonica Brasil S.A.</t>
-  </si>
-  <si>
-    <t>Perícia Técnica</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Telepresencial</t>
+    <t>Salitre Fertilizantes Ltda.</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
   </si>
   <si>
     <t>Audiência Inicial - Telepresencial</t>
   </si>
   <si>
+    <t>Sessão de Julgamento TJ - Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Semipresencial</t>
+  </si>
+  <si>
     <t>Audiência Instrução - Telepresencial</t>
   </si>
   <si>
-    <t>Audiência Inicial - Presencial</t>
-  </si>
-  <si>
-    <t>Audiência Una - Telepresencial</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>0011835-11.2025.5.15.0084</t>
-  </si>
-  <si>
-    <t>0010484-23.2026.5.03.0174</t>
-  </si>
-  <si>
-    <t>0010064-52.2026.5.15.0087</t>
-  </si>
-  <si>
-    <t>0011091-26.2026.5.03.0048</t>
-  </si>
-  <si>
-    <t>0010659-07.2026.5.15.0037</t>
-  </si>
-  <si>
-    <t>0010148-68.2026.5.15.0082</t>
-  </si>
-  <si>
-    <t>1000584-41.2026.5.02.0363</t>
-  </si>
-  <si>
-    <t>0012537-21.2025.5.15.0095</t>
-  </si>
-  <si>
-    <t>0000438-80.2026.5.05.0121</t>
-  </si>
-  <si>
-    <t>0010626-17.2026.5.15.0037</t>
-  </si>
-  <si>
-    <t>0012372-63.2025.5.15.0130</t>
-  </si>
-  <si>
-    <t>0011566-58.2026.5.15.0044</t>
-  </si>
-  <si>
-    <t>1000839-77.2026.5.02.0434</t>
-  </si>
-  <si>
-    <t>1000288-07.2026.5.02.0464</t>
-  </si>
-  <si>
-    <t>1000133-67.2026.5.02.0055</t>
-  </si>
-  <si>
-    <t>0011186-18.2026.5.15.0082</t>
-  </si>
-  <si>
-    <t>Cristiane Paula De Sousa Araujo Carvalho</t>
-  </si>
-  <si>
-    <t>Francinaldo Alves Dos Santos</t>
-  </si>
-  <si>
-    <t>Jessica Nunes Da Silva</t>
-  </si>
-  <si>
-    <t>Luiz Augusto Dias</t>
-  </si>
-  <si>
-    <t>Evandro Martins Ribeiro</t>
-  </si>
-  <si>
-    <t>Erivan Agustinho Furtado</t>
-  </si>
-  <si>
-    <t>Gabriel Da Corte</t>
-  </si>
-  <si>
-    <t>Heleno Dirceu Martins</t>
-  </si>
-  <si>
-    <t>Leandro Dos Santos Lima</t>
-  </si>
-  <si>
-    <t>Jose Ovidio Ferreira De Aquino</t>
-  </si>
-  <si>
-    <t>Marcelo Augusto De Souza Primo</t>
-  </si>
-  <si>
-    <t>Pedro Soares Dos Santos</t>
-  </si>
-  <si>
-    <t>Luiz Carlos Baptista</t>
-  </si>
-  <si>
-    <t>Sarita Ferreira Ventura</t>
-  </si>
-  <si>
-    <t>Luciana De Lima Machado</t>
-  </si>
-  <si>
-    <t>Adilson Maximiano Nogueira</t>
-  </si>
-  <si>
-    <t>08:00:00</t>
-  </si>
-  <si>
-    <t>08:10:00</t>
+    <t>Audiência Inicial -  Presencial</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Semipresencial</t>
+  </si>
+  <si>
+    <t>1000237-89.2026.5.02.0433</t>
+  </si>
+  <si>
+    <t>0010719-78.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>0010721-48.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>0010725-85.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>0010726-70.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>5016566.75.2024.4.04.7201</t>
+  </si>
+  <si>
+    <t>1000618-51.2026.5.02.0319</t>
+  </si>
+  <si>
+    <t>0010643-83.2026.5.15.0027</t>
+  </si>
+  <si>
+    <t>0011871-29.2024.5.15.0071</t>
+  </si>
+  <si>
+    <t>0011194-92.2025.5.15.0061</t>
+  </si>
+  <si>
+    <t>0011297-43.2026.5.15.0133</t>
+  </si>
+  <si>
+    <t>0010155-46.2026.5.15.0119</t>
+  </si>
+  <si>
+    <t>0011718-25.2024.5.15.0126</t>
+  </si>
+  <si>
+    <t>1000516-14.2026.5.02.0712</t>
+  </si>
+  <si>
+    <t>0011727-56.2025.5.15.0027</t>
+  </si>
+  <si>
+    <t>1000075-55.2023.5.02.0383</t>
+  </si>
+  <si>
+    <t>0011696-36.2025.5.15.0027</t>
+  </si>
+  <si>
+    <t>0000017-35.2026.5.09.0071</t>
+  </si>
+  <si>
+    <t>0011309-54.2026.5.03.0048</t>
+  </si>
+  <si>
+    <t>0011710-87.2025.5.03.0048</t>
+  </si>
+  <si>
+    <t>0011711-72.2025.5.03.0048</t>
+  </si>
+  <si>
+    <t>0011712-57.2025.5.03.0048</t>
+  </si>
+  <si>
+    <t>0010530-11.2025.5.15.0013</t>
+  </si>
+  <si>
+    <t>0010879-39.2025.5.03.0048</t>
+  </si>
+  <si>
+    <t>1000149-48.2026.5.02.0434</t>
+  </si>
+  <si>
+    <t>0011544-84.2024.5.15.0071</t>
+  </si>
+  <si>
+    <t>0011542-17.2024.5.15.0071</t>
+  </si>
+  <si>
+    <t>1000464-72.2026.5.02.0015</t>
+  </si>
+  <si>
+    <t>1001737-36.2025.5.02.0431</t>
+  </si>
+  <si>
+    <t>Alex Almeida De Lima</t>
+  </si>
+  <si>
+    <t>Gleydson Freitas Sousa</t>
+  </si>
+  <si>
+    <t>Itamar Jose Da Rocha</t>
+  </si>
+  <si>
+    <t>Tiago De Castro Fonseca</t>
+  </si>
+  <si>
+    <t>Elias Jorge Democh</t>
+  </si>
+  <si>
+    <t>Instituto Nacional Do Seguro Social - Inss</t>
+  </si>
+  <si>
+    <t>Zivanildo Bezerra Barbosa</t>
+  </si>
+  <si>
+    <t>Lucas Vinicius Inamorato</t>
+  </si>
+  <si>
+    <t>Doclesio Custodio Santana</t>
+  </si>
+  <si>
+    <t>Marcio Pereira Santos</t>
+  </si>
+  <si>
+    <t>Claudio Junio Rocha Da Silva</t>
+  </si>
+  <si>
+    <t>Anderson De Santana Franco</t>
+  </si>
+  <si>
+    <t>Mario Jose Da Silva Filho</t>
+  </si>
+  <si>
+    <t>Mauro Francisco Da Silva</t>
+  </si>
+  <si>
+    <t>Dorival De Souza Morais</t>
+  </si>
+  <si>
+    <t>Maria Eslaine Silva Ribeiro Flor</t>
+  </si>
+  <si>
+    <t>Roberto Pereira Da Silva</t>
+  </si>
+  <si>
+    <t>Gilmar Lourenco</t>
+  </si>
+  <si>
+    <t>Kelson Jose De Oliveira Junior</t>
+  </si>
+  <si>
+    <t>Bruno Daniel Da Cruz</t>
+  </si>
+  <si>
+    <t>Adriano Leite Silva</t>
+  </si>
+  <si>
+    <t>Thiago Sebastiao Gervasio De Oliveira</t>
+  </si>
+  <si>
+    <t>Diego Vinicius Stabile David</t>
+  </si>
+  <si>
+    <t>Jose Cicero Barbosa</t>
+  </si>
+  <si>
+    <t>Jonata Tadeu Oliveira Da Costa</t>
+  </si>
+  <si>
+    <t>Giacomo Geroldo Quito</t>
+  </si>
+  <si>
+    <t>Luciano Marco Costa Huerta</t>
+  </si>
+  <si>
+    <t>Leandro De Oliveira Carminatti</t>
+  </si>
+  <si>
+    <t>08:20:00</t>
   </si>
   <si>
     <t>08:30:00</t>
@@ -262,7 +379,13 @@
     <t>08:35:00</t>
   </si>
   <si>
-    <t>09:10:00</t>
+    <t>08:40:00</t>
+  </si>
+  <si>
+    <t>08:45:00</t>
+  </si>
+  <si>
+    <t>09:00:00</t>
   </si>
   <si>
     <t>09:20:00</t>
@@ -271,25 +394,58 @@
     <t>09:30:00</t>
   </si>
   <si>
-    <t>09:35:00</t>
-  </si>
-  <si>
-    <t>09:50:00</t>
-  </si>
-  <si>
     <t>10:00:00</t>
   </si>
   <si>
-    <t>10:15:00</t>
-  </si>
-  <si>
-    <t>12:00:00</t>
-  </si>
-  <si>
-    <t>12:20:00</t>
-  </si>
-  <si>
-    <t>16:00:00</t>
+    <t>10:20:00</t>
+  </si>
+  <si>
+    <t>10:40:00</t>
+  </si>
+  <si>
+    <t>10:45:00</t>
+  </si>
+  <si>
+    <t>12:05:00</t>
+  </si>
+  <si>
+    <t>13:00:00</t>
+  </si>
+  <si>
+    <t>13:30:00</t>
+  </si>
+  <si>
+    <t>13:35:00</t>
+  </si>
+  <si>
+    <t>13:50:00</t>
+  </si>
+  <si>
+    <t>13:55:00</t>
+  </si>
+  <si>
+    <t>14:00:00</t>
+  </si>
+  <si>
+    <t>14:04:00</t>
+  </si>
+  <si>
+    <t>14:15:00</t>
+  </si>
+  <si>
+    <t>15:00:00</t>
+  </si>
+  <si>
+    <t>15:10:00</t>
+  </si>
+  <si>
+    <t>15:15:00</t>
+  </si>
+  <si>
+    <t>15:20:00</t>
+  </si>
+  <si>
+    <t>15:40:00</t>
   </si>
 </sst>
 </file>
@@ -625,7 +781,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -665,7 +821,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -674,33 +830,33 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="G2" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="H2" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="I2" t="s">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="J2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="K2" t="s">
-        <v>78</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
@@ -709,453 +865,453 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="G3" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="H3" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I3" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="J3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="K3" t="s">
-        <v>79</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="H4" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="I4" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="J4" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="K4" t="s">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="H5" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="I5" t="s">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="J5" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="K5" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="F6" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="H6" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="I6" t="s">
-        <v>66</v>
+        <v>94</v>
       </c>
       <c r="J6" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="K6" t="s">
-        <v>82</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="H7" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="I7" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="J7" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="K7" t="s">
-        <v>83</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="F8" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="G8" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="H8" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="I8" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="J8" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="K8" t="s">
-        <v>84</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="G9" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="H9" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="J9" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="K9" t="s">
-        <v>85</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="F10" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="G10" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="H10" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="I10" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="J10" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="K10" t="s">
-        <v>86</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E11" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="F11" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="G11" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="H11" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="I11" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="J11" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="K11" t="s">
-        <v>86</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B12" t="s">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="F12" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="G12" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="H12" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="I12" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="J12" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="K12" t="s">
-        <v>87</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E13" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="F13" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="G13" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="H13" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="I13" t="s">
-        <v>73</v>
+        <v>101</v>
       </c>
       <c r="J13" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="K13" t="s">
-        <v>88</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D14" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="F14" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="G14" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="H14" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="I14" t="s">
-        <v>74</v>
+        <v>102</v>
       </c>
       <c r="J14" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="K14" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B15" t="s">
         <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D15" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F15" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="G15" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="H15" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="I15" t="s">
-        <v>75</v>
+        <v>103</v>
       </c>
       <c r="J15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K15" t="s">
-        <v>89</v>
+        <v>130</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B16" t="s">
         <v>11</v>
@@ -1164,63 +1320,518 @@
         <v>23</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E16" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F16" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="G16" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="H16" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="I16" t="s">
-        <v>76</v>
+        <v>104</v>
       </c>
       <c r="J16" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="K16" t="s">
-        <v>90</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B17" t="s">
         <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" t="s">
+        <v>47</v>
+      </c>
+      <c r="F17" t="s">
+        <v>59</v>
+      </c>
+      <c r="G17" t="s">
+        <v>59</v>
+      </c>
+      <c r="H17" t="s">
+        <v>76</v>
+      </c>
+      <c r="I17" t="s">
+        <v>105</v>
+      </c>
+      <c r="J17" t="s">
+        <v>47</v>
+      </c>
+      <c r="K17" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" t="s">
+        <v>57</v>
+      </c>
+      <c r="G18" t="s">
+        <v>57</v>
+      </c>
+      <c r="H18" t="s">
+        <v>77</v>
+      </c>
+      <c r="I18" t="s">
+        <v>106</v>
+      </c>
+      <c r="J18" t="s">
+        <v>41</v>
+      </c>
+      <c r="K18" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
         <v>25</v>
       </c>
-      <c r="E17" t="s">
+      <c r="D19" t="s">
+        <v>35</v>
+      </c>
+      <c r="E19" t="s">
+        <v>48</v>
+      </c>
+      <c r="F19" t="s">
+        <v>57</v>
+      </c>
+      <c r="G19" t="s">
+        <v>57</v>
+      </c>
+      <c r="H19" t="s">
+        <v>78</v>
+      </c>
+      <c r="I19" t="s">
+        <v>107</v>
+      </c>
+      <c r="J19" t="s">
+        <v>48</v>
+      </c>
+      <c r="K19" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E20" t="s">
+        <v>49</v>
+      </c>
+      <c r="F20" t="s">
+        <v>53</v>
+      </c>
+      <c r="G20" t="s">
+        <v>53</v>
+      </c>
+      <c r="H20" t="s">
+        <v>79</v>
+      </c>
+      <c r="I20" t="s">
+        <v>108</v>
+      </c>
+      <c r="J20" t="s">
+        <v>49</v>
+      </c>
+      <c r="K20" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E21" t="s">
+        <v>49</v>
+      </c>
+      <c r="F21" t="s">
+        <v>59</v>
+      </c>
+      <c r="G21" t="s">
+        <v>59</v>
+      </c>
+      <c r="H21" t="s">
+        <v>80</v>
+      </c>
+      <c r="I21" t="s">
+        <v>109</v>
+      </c>
+      <c r="J21" t="s">
+        <v>49</v>
+      </c>
+      <c r="K21" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22" t="s">
+        <v>49</v>
+      </c>
+      <c r="F22" t="s">
+        <v>59</v>
+      </c>
+      <c r="G22" t="s">
+        <v>59</v>
+      </c>
+      <c r="H22" t="s">
+        <v>81</v>
+      </c>
+      <c r="I22" t="s">
+        <v>110</v>
+      </c>
+      <c r="J22" t="s">
+        <v>49</v>
+      </c>
+      <c r="K22" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B23" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" t="s">
+        <v>31</v>
+      </c>
+      <c r="E23" t="s">
+        <v>49</v>
+      </c>
+      <c r="F23" t="s">
+        <v>59</v>
+      </c>
+      <c r="G23" t="s">
+        <v>59</v>
+      </c>
+      <c r="H23" t="s">
+        <v>82</v>
+      </c>
+      <c r="I23" t="s">
+        <v>111</v>
+      </c>
+      <c r="J23" t="s">
+        <v>49</v>
+      </c>
+      <c r="K23" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24" t="s">
+        <v>50</v>
+      </c>
+      <c r="F24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" t="s">
+        <v>60</v>
+      </c>
+      <c r="H24" t="s">
+        <v>83</v>
+      </c>
+      <c r="I24" t="s">
+        <v>112</v>
+      </c>
+      <c r="J24" t="s">
+        <v>50</v>
+      </c>
+      <c r="K24" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" t="s">
+        <v>31</v>
+      </c>
+      <c r="E25" t="s">
+        <v>51</v>
+      </c>
+      <c r="F25" t="s">
+        <v>59</v>
+      </c>
+      <c r="G25" t="s">
+        <v>59</v>
+      </c>
+      <c r="H25" t="s">
+        <v>84</v>
+      </c>
+      <c r="I25" t="s">
+        <v>113</v>
+      </c>
+      <c r="J25" t="s">
+        <v>51</v>
+      </c>
+      <c r="K25" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
+      <c r="A26" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B26" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" t="s">
+        <v>27</v>
+      </c>
+      <c r="D26" t="s">
+        <v>30</v>
+      </c>
+      <c r="E26" t="s">
+        <v>37</v>
+      </c>
+      <c r="F26" t="s">
+        <v>52</v>
+      </c>
+      <c r="G26" t="s">
+        <v>52</v>
+      </c>
+      <c r="H26" t="s">
+        <v>85</v>
+      </c>
+      <c r="I26" t="s">
+        <v>114</v>
+      </c>
+      <c r="J26" t="s">
+        <v>37</v>
+      </c>
+      <c r="K26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B27" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" t="s">
+        <v>28</v>
+      </c>
+      <c r="D27" t="s">
         <v>33</v>
       </c>
-      <c r="F17" t="s">
-        <v>40</v>
-      </c>
-      <c r="G17" t="s">
-        <v>40</v>
-      </c>
-      <c r="H17" t="s">
-        <v>61</v>
-      </c>
-      <c r="I17" t="s">
-        <v>77</v>
-      </c>
-      <c r="J17" t="s">
+      <c r="E27" t="s">
+        <v>42</v>
+      </c>
+      <c r="F27" t="s">
+        <v>57</v>
+      </c>
+      <c r="G27" t="s">
+        <v>57</v>
+      </c>
+      <c r="H27" t="s">
+        <v>86</v>
+      </c>
+      <c r="I27" t="s">
+        <v>115</v>
+      </c>
+      <c r="J27" t="s">
+        <v>42</v>
+      </c>
+      <c r="K27" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
+      <c r="A28" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B28" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" t="s">
         <v>33</v>
       </c>
-      <c r="K17" t="s">
-        <v>91</v>
+      <c r="E28" t="s">
+        <v>42</v>
+      </c>
+      <c r="F28" t="s">
+        <v>57</v>
+      </c>
+      <c r="G28" t="s">
+        <v>57</v>
+      </c>
+      <c r="H28" t="s">
+        <v>87</v>
+      </c>
+      <c r="I28" t="s">
+        <v>115</v>
+      </c>
+      <c r="J28" t="s">
+        <v>42</v>
+      </c>
+      <c r="K28" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
+      <c r="A29" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B29" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="s">
+        <v>30</v>
+      </c>
+      <c r="E29" t="s">
+        <v>37</v>
+      </c>
+      <c r="F29" t="s">
+        <v>59</v>
+      </c>
+      <c r="G29" t="s">
+        <v>59</v>
+      </c>
+      <c r="H29" t="s">
+        <v>88</v>
+      </c>
+      <c r="I29" t="s">
+        <v>116</v>
+      </c>
+      <c r="J29" t="s">
+        <v>37</v>
+      </c>
+      <c r="K29" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
+      <c r="A30" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B30" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" t="s">
+        <v>29</v>
+      </c>
+      <c r="D30" t="s">
+        <v>30</v>
+      </c>
+      <c r="E30" t="s">
+        <v>37</v>
+      </c>
+      <c r="F30" t="s">
+        <v>59</v>
+      </c>
+      <c r="G30" t="s">
+        <v>59</v>
+      </c>
+      <c r="H30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I30" t="s">
+        <v>117</v>
+      </c>
+      <c r="J30" t="s">
+        <v>37</v>
+      </c>
+      <c r="K30" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Audiências: sync 2026-07-23 — 14 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="85">
   <si>
     <t>data</t>
   </si>
@@ -52,235 +52,223 @@
     <t>D-1</t>
   </si>
   <si>
+    <t>VCR</t>
+  </si>
+  <si>
+    <t>AAP</t>
+  </si>
+  <si>
+    <t>Correspondente - doc9</t>
+  </si>
+  <si>
     <t>MBF</t>
   </si>
   <si>
-    <t>Correspondente - Carlos Florian</t>
+    <t>FCG</t>
+  </si>
+  <si>
+    <t>DPR</t>
+  </si>
+  <si>
+    <t>GSM</t>
+  </si>
+  <si>
+    <t>ALF</t>
+  </si>
+  <si>
+    <t>CAL</t>
   </si>
   <si>
     <t>RRU</t>
   </si>
   <si>
-    <t>Correspondente - Hebert</t>
-  </si>
-  <si>
-    <t>RYL</t>
-  </si>
-  <si>
-    <t>TFR</t>
-  </si>
-  <si>
-    <t>VRO</t>
-  </si>
-  <si>
-    <t>ARC</t>
-  </si>
-  <si>
     <t>ANB</t>
   </si>
   <si>
-    <t>GSM</t>
-  </si>
-  <si>
-    <t>VSI</t>
-  </si>
-  <si>
-    <t>GSF</t>
-  </si>
-  <si>
     <t>JPE</t>
   </si>
   <si>
+    <t>Grupo B2</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
     <t>Grupo E2</t>
   </si>
   <si>
-    <t>Grupo E1</t>
-  </si>
-  <si>
     <t>Grupo B1</t>
   </si>
   <si>
-    <t>Grupo C</t>
-  </si>
-  <si>
     <t>Grupo D1</t>
   </si>
   <si>
-    <t>Grupo A3</t>
+    <t>Embraer S.A.</t>
+  </si>
+  <si>
+    <t>Robert Bosch Limitada</t>
+  </si>
+  <si>
+    <t>Sistenge Construções E Comércio Ltda</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda</t>
+  </si>
+  <si>
+    <t>Syngenta Seeds Ltda.</t>
+  </si>
+  <si>
+    <t>Bridgestone do Brasil Indústria e Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A.</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda.</t>
+  </si>
+  <si>
+    <t>L. Sant'Angelo Pinturas Ltda.</t>
   </si>
   <si>
     <t>Santa Juliana Bioenergia Ltda.</t>
   </si>
   <si>
-    <t>Syngenta Proteção De Cultivos Ltda.</t>
-  </si>
-  <si>
-    <t>Moema Bioenergia S.A.</t>
+    <t>Bit Services Inovação E Tecnologia Ltda.</t>
   </si>
   <si>
     <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
   </si>
   <si>
-    <t>Ouroeste Bioenergia Ltda.</t>
-  </si>
-  <si>
-    <t>Telefônica Brasil S.A</t>
-  </si>
-  <si>
-    <t>Mahle Metal Leve S.A.</t>
-  </si>
-  <si>
-    <t>Mitre Vendas Corretagem De Imóveis Ltda.</t>
-  </si>
-  <si>
-    <t>Bit Services Inovação E Tecnologia Ltda.</t>
-  </si>
-  <si>
-    <t>Telefônica Brasil S.A.</t>
-  </si>
-  <si>
-    <t>Whirlpool S.A.</t>
-  </si>
-  <si>
-    <t>Audiência Inicial - Telepresencial</t>
-  </si>
-  <si>
-    <t>Audiência Una - Semipresencial</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Telepresencial</t>
+    <t>Perícia Técnica</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
   </si>
   <si>
     <t>Audiência Una - Presencial</t>
   </si>
   <si>
-    <t>Audiência Inicial - Presencial</t>
-  </si>
-  <si>
-    <t>Sessão de Julgamento TRT - Presencial</t>
-  </si>
-  <si>
-    <t>Audiência de Conciliação - Telepresencial</t>
-  </si>
-  <si>
-    <t>0011127-68.2026.5.03.0048</t>
-  </si>
-  <si>
-    <t>1000662-82.2026.5.02.0703</t>
-  </si>
-  <si>
-    <t>0011129-41.2026.5.15.0133</t>
-  </si>
-  <si>
-    <t>1000314-07.2026.5.02.0431</t>
-  </si>
-  <si>
-    <t>0010478-06.2026.5.15.0037</t>
-  </si>
-  <si>
-    <t>1000586-34.2026.5.02.0032</t>
-  </si>
-  <si>
-    <t>1000645-84.2026.5.02.0464</t>
-  </si>
-  <si>
-    <t>1000858-43.2026.5.02.0609</t>
-  </si>
-  <si>
-    <t>1001499-82.2025.5.02.0086</t>
-  </si>
-  <si>
-    <t>1000894-28.2026.5.02.0434</t>
-  </si>
-  <si>
-    <t>1001012-15.2024.5.02.0065</t>
-  </si>
-  <si>
-    <t>1000807-38.2025.5.02.0004</t>
-  </si>
-  <si>
-    <t>1000895-13.2026.5.02.0434</t>
-  </si>
-  <si>
-    <t>1001314-38.2023.5.02.0434</t>
-  </si>
-  <si>
-    <t>Elenilson Costa Franca</t>
-  </si>
-  <si>
-    <t>Edilson Stanize</t>
-  </si>
-  <si>
-    <t>Antoniel Silva Dos Santos</t>
-  </si>
-  <si>
-    <t>Evandro Fernandes Augusto</t>
-  </si>
-  <si>
-    <t>Joyce Leticia Gentile Pavao Correia</t>
-  </si>
-  <si>
-    <t>Kleber Faria Dos Santos</t>
-  </si>
-  <si>
-    <t>Gerson Dourado Santos</t>
-  </si>
-  <si>
-    <t>Rodrigo Lopes Da Silva</t>
-  </si>
-  <si>
-    <t>Lidia Teixeira Neves</t>
-  </si>
-  <si>
-    <t>Eduardo Antonio De Souza Braga</t>
-  </si>
-  <si>
-    <t>Andre Fernandes Rodrigues</t>
-  </si>
-  <si>
-    <t>Carla Di Francesco Verdolini</t>
-  </si>
-  <si>
-    <t>Flavio Eduardo Basilio</t>
-  </si>
-  <si>
-    <t>Elenilton Junio De Jesus Silva</t>
-  </si>
-  <si>
-    <t>08:15:00</t>
-  </si>
-  <si>
-    <t>08:20:00</t>
-  </si>
-  <si>
-    <t>09:00:00</t>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>0011835-11.2025.5.15.0084</t>
+  </si>
+  <si>
+    <t>0011270-80.2026.5.15.0094</t>
+  </si>
+  <si>
+    <t>0000748-68.2026.5.19.0001</t>
+  </si>
+  <si>
+    <t>0010755-23.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>0010783-88.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>0010786-43.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>0010429-51.2025.5.03.0063</t>
+  </si>
+  <si>
+    <t>1001324-86.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>0012273-93.2025.5.15.0130</t>
+  </si>
+  <si>
+    <t>0011280-39.2025.5.03.0080</t>
+  </si>
+  <si>
+    <t>1000537-26.2026.5.02.0603</t>
+  </si>
+  <si>
+    <t>0010871-95.2022.5.03.0168</t>
+  </si>
+  <si>
+    <t>1001751-48.2025.5.02.0066</t>
+  </si>
+  <si>
+    <t>1001754-06.2024.5.02.0432</t>
+  </si>
+  <si>
+    <t>Cristiane Paula De Sousa Araujo Carvalho</t>
+  </si>
+  <si>
+    <t>Clovis Adilson Antonicelli</t>
+  </si>
+  <si>
+    <t>Fernando Santana</t>
+  </si>
+  <si>
+    <t>Marllon De Pinho Da Silva</t>
+  </si>
+  <si>
+    <t>Edley Henrique Silva</t>
+  </si>
+  <si>
+    <t>Milton Vieira De Almeida</t>
+  </si>
+  <si>
+    <t>Kenede Basilio De Araujo</t>
+  </si>
+  <si>
+    <t>Fabiano De Moura Goncalves</t>
+  </si>
+  <si>
+    <t>Francisco Elenilson Alves</t>
+  </si>
+  <si>
+    <t>Adrian Silva De Aquino</t>
+  </si>
+  <si>
+    <t>Domingos Rufino Franco</t>
+  </si>
+  <si>
+    <t>Andrelino Pereira De Mendonca</t>
+  </si>
+  <si>
+    <t>Rosana Lopes De Oliveira Cruz</t>
+  </si>
+  <si>
+    <t>Anderson Rodrigues</t>
+  </si>
+  <si>
+    <t>08:00:00</t>
+  </si>
+  <si>
+    <t>08:50:00</t>
+  </si>
+  <si>
+    <t>09:10:00</t>
+  </si>
+  <si>
+    <t>09:20:00</t>
   </si>
   <si>
     <t>09:30:00</t>
   </si>
   <si>
-    <t>09:50:00</t>
-  </si>
-  <si>
     <t>10:00:00</t>
   </si>
   <si>
     <t>10:10:00</t>
   </si>
   <si>
-    <t>11:00:00</t>
-  </si>
-  <si>
-    <t>13:00:00</t>
-  </si>
-  <si>
-    <t>13:10:00</t>
-  </si>
-  <si>
-    <t>15:42:00</t>
+    <t>10:30:00</t>
+  </si>
+  <si>
+    <t>14:20:00</t>
+  </si>
+  <si>
+    <t>14:40:00</t>
+  </si>
+  <si>
+    <t>15:00:00</t>
   </si>
 </sst>
 </file>
@@ -656,7 +644,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -665,33 +653,33 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="J2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
@@ -700,33 +688,33 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="I3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="J3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
@@ -735,33 +723,33 @@
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I4" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="J4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K4" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
@@ -770,10 +758,10 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F5" t="s">
         <v>44</v>
@@ -782,366 +770,366 @@
         <v>44</v>
       </c>
       <c r="H5" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I5" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K5" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H6" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I6" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="J6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="K6" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I7" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="J7" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="K7" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G8" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H8" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="I8" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="J8" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="K8" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E9" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G9" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="I9" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="J9" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="K9" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D10" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E10" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H10" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="I10" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="J10" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K10" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H11" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="I11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K11" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B12" t="s">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E12" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F12" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="G12" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H12" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I12" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="J12" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="K12" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E13" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F13" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G13" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H13" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="I13" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="J13" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="K13" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F14" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G14" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="H14" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I14" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="J14" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="K14" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B15" t="s">
         <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D15" t="s">
         <v>27</v>
       </c>
       <c r="E15" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="F15" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="G15" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="H15" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I15" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="J15" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="K15" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Audiências: sync 2026-07-27 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9FDA973-1726-4978-B32E-61783B1A0FFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CC9C934-ACFD-4205-90EA-1198CCBE566F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9A160F25-2670-4677-BD90-34B27A142245}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72218CE6-47E0-40A4-8063-C4D7752BDE5A}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="200">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,92 +95,557 @@
     <t>Link/Observações</t>
   </si>
   <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>0010556-64.2023.5.15.0082</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Miguel Jose De Souza</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DO RIO PRETO</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>CEJUSC</t>
+  </si>
+  <si>
+    <t>Instrução</t>
+  </si>
+  <si>
+    <t>Reclamação Trabalhista</t>
+  </si>
+  <si>
+    <t>CENTRAL</t>
+  </si>
+  <si>
+    <t>R$             177.690,57</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/88415253122?pwd=QzlTNmxwdWpEeGVFZmdwM0lDUFJ4Zz09 ID da reunião: 884 1525 3122 Senha de acesso: 510562</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>1000973-20.2026.5.02.0462</t>
+  </si>
+  <si>
+    <t>Mahle Metal Leve S.A.</t>
+  </si>
+  <si>
+    <t>Sonia Soares Almeida</t>
+  </si>
+  <si>
+    <t>SÃO BERNARDO DO CAMPO</t>
+  </si>
+  <si>
+    <t>02ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Inicial</t>
+  </si>
+  <si>
+    <t>R$             191.275,42</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>Correspondente - Carlos Florian</t>
+  </si>
+  <si>
+    <t>TLI</t>
+  </si>
+  <si>
+    <t>Presencial | Advogada - Dra. Luciana França, (11) 96351-8524</t>
+  </si>
+  <si>
+    <t>1001013-02.2026.5.02.0462</t>
+  </si>
+  <si>
+    <t>Davi Joao Da Silva</t>
+  </si>
+  <si>
+    <t>05ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             629.417,60</t>
+  </si>
+  <si>
+    <t>PSI</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Telepresencial</t>
+  </si>
+  <si>
+    <t>0014731-48.2025.5.15.0077</t>
+  </si>
+  <si>
+    <t>Robert Bosch Limitada</t>
+  </si>
+  <si>
+    <t>Ismael Jose Dos Santos</t>
+  </si>
+  <si>
+    <t>INDAIATUBA</t>
+  </si>
+  <si>
+    <t>VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             810.894,79</t>
+  </si>
+  <si>
+    <t>ALF</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/88215751954?pwd=GWf0av1x8hFikMFre3DVbJa2NJn80H.1 ID da reunião 882 1575 1954 Senha  150077</t>
+  </si>
+  <si>
+    <t>0011763-13.2026.5.15.0044</t>
+  </si>
+  <si>
+    <t>Matheus Felipe Januario Domingues</t>
+  </si>
+  <si>
+    <t>R$             356.093,25</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/81757243738?pwd=UXAvdEpveHlrNU05M2ZsZnRrYy9Vdz09 ID DA REUNIÃO: 817 5724 3738 SENHA: 954332</t>
+  </si>
+  <si>
+    <t>0000846-69.2026.5.05.0251</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda</t>
+  </si>
+  <si>
+    <t>Gilson Meireles Dos Santos</t>
+  </si>
+  <si>
+    <t>CONCEIÇÃO DO COITÉ</t>
+  </si>
+  <si>
+    <t>BA</t>
+  </si>
+  <si>
+    <t>R$               18.131,17</t>
+  </si>
+  <si>
+    <t>JNE</t>
+  </si>
+  <si>
+    <t>JRT</t>
+  </si>
+  <si>
+    <t>https://trt5-jus-br.zoom.us/my/segundonucleo4sala2</t>
+  </si>
+  <si>
+    <t>0010954-47.2026.5.15.0133</t>
+  </si>
+  <si>
+    <t>Edivaldo Aparecido De Oliveira</t>
+  </si>
+  <si>
+    <t>04ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             262.000,00</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/88542672682?pwd=7pQ4QRhZmRG9RAQAWKowymbwNawa7t.1 ID da reunião: 885 4267 2682 Senha de acesso: 050728</t>
+  </si>
+  <si>
+    <t>0001673-39.2025.5.13.0010</t>
+  </si>
+  <si>
+    <t>Willan Hilario Marcelino</t>
+  </si>
+  <si>
+    <t>GUARABIRA</t>
+  </si>
+  <si>
+    <t>PB</t>
+  </si>
+  <si>
+    <t>CEJUSC 2º GRAU</t>
+  </si>
+  <si>
+    <t>Recursal</t>
+  </si>
+  <si>
+    <t>R$               46.279,00</t>
+  </si>
+  <si>
+    <t>FCG</t>
+  </si>
+  <si>
+    <t>https://trt13-jus-br.zoom.us/my/cejusc13.sala5</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Presencial</t>
+  </si>
+  <si>
+    <t>0010064-52.2026.5.15.0087</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
+  </si>
+  <si>
+    <t>Jessica Nunes Da Silva</t>
+  </si>
+  <si>
+    <t>PAULÍNIA</t>
+  </si>
+  <si>
+    <t>01ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>1ª Instância</t>
+  </si>
+  <si>
+    <t>R$             102.270,09</t>
+  </si>
+  <si>
+    <t>DPR</t>
+  </si>
+  <si>
+    <t>JRM</t>
+  </si>
+  <si>
+    <t>Presencial</t>
+  </si>
+  <si>
+    <t>0010295-44.2026.5.15.0131</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Marcos Paulo Leite</t>
+  </si>
+  <si>
+    <t>CAMPINAS</t>
+  </si>
+  <si>
+    <t>12ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             283.750,20</t>
+  </si>
+  <si>
+    <t>Grupo B1</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/83676367506?pwd=VlRlWmFnUGhwdWp3Y2xvaVkxdDFDZz09 ID da reunião: 836 7636 7506 Senha: 24680</t>
+  </si>
+  <si>
+    <t>0000761-97.2026.5.17.0009</t>
+  </si>
+  <si>
+    <t>Fertilizantes Tocantins S.A</t>
+  </si>
+  <si>
+    <t>Edilcivane Pereira Ottoni</t>
+  </si>
+  <si>
+    <t>VITÓRIA</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>09ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Conhecimento</t>
+  </si>
+  <si>
+    <t>R$                 5.659,29</t>
+  </si>
+  <si>
+    <t>Correspondente - doc9</t>
+  </si>
+  <si>
+    <t>CAL</t>
+  </si>
+  <si>
+    <t>Presencial | Advogado - Ricardo Baracho Moreira ricardo.baracho@gmail.com (27) 998923622</t>
+  </si>
+  <si>
+    <t>0011575-56.2024.5.15.0087</t>
+  </si>
+  <si>
+    <t>Wesley Felipe Cezar Xavier</t>
+  </si>
+  <si>
+    <t>ORGÃO ESPECIAL</t>
+  </si>
+  <si>
+    <t>2ª Instância</t>
+  </si>
+  <si>
+    <t>R$             150.650,00</t>
+  </si>
+  <si>
+    <t>JPL</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/81907928214?pwd=DdJyPKEOQWb3pMKbKp713raBQMIpao.1 ID:  819  0792  8214  Senha: 935266.</t>
+  </si>
+  <si>
+    <t>0010718-92.2023.5.15.0071</t>
+  </si>
+  <si>
+    <t>Claudio Richard De Godoy</t>
+  </si>
+  <si>
+    <t>MOGI GUAÇU</t>
+  </si>
+  <si>
+    <t>R$             100.000,00</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/88971005711?pwd=FCU0CcOJlu66H4VR8hrXW2o1KrrqXb.1 ID: 889  7100  5711  Senha: 962801</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>0000010-77.2026.5.09.0092</t>
+  </si>
+  <si>
+    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
+  </si>
+  <si>
+    <t>Darlan Silva Quintiliano</t>
+  </si>
+  <si>
+    <t>CIANORTE</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>R$               32.000,00</t>
+  </si>
+  <si>
+    <t>Grupo C</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>https://trt9-jus-br.zoom.us/j/5580468805?pwd=aXhxc3lyQ2F2K0FTWEVoU3ZOWDhlUT09</t>
+  </si>
+  <si>
     <t>Audiência Instrução - Telepresencial</t>
   </si>
   <si>
-    <t>0000431-17.2026.5.10.0811</t>
-  </si>
-  <si>
-    <t>Produtécnica Nordeste Comércio De Insumos Agrícolas Ltda.</t>
-  </si>
-  <si>
-    <t>Jhony Carlos Lucena Cardoso</t>
-  </si>
-  <si>
-    <t>ARAGUAINA</t>
-  </si>
-  <si>
-    <t>TO</t>
-  </si>
-  <si>
-    <t>01ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>1ª Instância</t>
-  </si>
-  <si>
-    <t>Reclamação Trabalhista</t>
-  </si>
-  <si>
-    <t>CENTRAL</t>
-  </si>
-  <si>
-    <t>R$             125.820,62</t>
-  </si>
-  <si>
-    <t>Grupo E1</t>
+    <t>0010907-03.2025.5.15.0103</t>
+  </si>
+  <si>
+    <t>Viterra Bioenergia S.A.</t>
+  </si>
+  <si>
+    <t>Jeanio Berto Da Costa E Silva</t>
+  </si>
+  <si>
+    <t>ARAÇATUBA</t>
+  </si>
+  <si>
+    <t>03ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             149.560,43</t>
+  </si>
+  <si>
+    <t>RRU</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/87527564652?pwd=d3YrZ2diWXk5UjgzbmVkNExteWVMQT09 ID da reunião: 875 2756 4652 Senha de acesso: 246680</t>
+  </si>
+  <si>
+    <t>0010466-75.2022.5.15.0087</t>
+  </si>
+  <si>
+    <t>Sidkley Jose Da Silva</t>
+  </si>
+  <si>
+    <t>Execução</t>
+  </si>
+  <si>
+    <t>R$               63.758,95</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/86385704640?pwd=g1Ig2NoEnHBDvn3uZhXt1tmbVhuO14.1</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>0011112-47.2025.5.03.0012</t>
+  </si>
+  <si>
+    <t>Ferrero Do Brasil Indústria Doceira E Alimentar Ltda.</t>
+  </si>
+  <si>
+    <t>Lucimar Da Silva Costa</t>
+  </si>
+  <si>
+    <t>BELO HORIZONTE</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>R$             162.480,95</t>
+  </si>
+  <si>
+    <t>Grupo B3</t>
+  </si>
+  <si>
+    <t>ANB</t>
+  </si>
+  <si>
+    <t>Presencial | Advogado - Dr. Luiz Henrique Ribeiro Costa (31) 98616-2039 |Preposto - Túlio Moreno Lobo Jardim (31) 99755-9174</t>
+  </si>
+  <si>
+    <t>0010432-81.2026.5.03.0156</t>
+  </si>
+  <si>
+    <t>Frutal Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Joao Batista Loiola De Sousa</t>
+  </si>
+  <si>
+    <t>FRUTAL</t>
+  </si>
+  <si>
+    <t>R$             401.858,88</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vtfrutal</t>
+  </si>
+  <si>
+    <t>0010828-57.2024.5.15.0071</t>
+  </si>
+  <si>
+    <t>Luciano Vicentim Da Cruz</t>
+  </si>
+  <si>
+    <t>R$             274.940,69</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/87345253855?pwd=eOmaFv9ph0gYOdbdibavbZapr1i2NE.1 ID:  873  4525  3855  Senha: 223572</t>
+  </si>
+  <si>
+    <t>1002332-26.2025.5.02.0434</t>
+  </si>
+  <si>
+    <t>Cesar Luiz Do Amaral</t>
+  </si>
+  <si>
+    <t>SANTO ANDRÉ</t>
+  </si>
+  <si>
+    <t>R$             231.524,56</t>
+  </si>
+  <si>
+    <t>GSM</t>
+  </si>
+  <si>
+    <t>BSO</t>
+  </si>
+  <si>
+    <t>1000813-89.2020.5.02.0434</t>
+  </si>
+  <si>
+    <t>Alan Alves Sarmento</t>
+  </si>
+  <si>
+    <t>CEJUSC ABC</t>
+  </si>
+  <si>
+    <t>R$             580.213,37</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/87687135814?pwd=L21Bd0RobFB3V0I0VVpuMlBDUG5oUT09 ID da reunião: 876 8713 5814 Senha de acesso: 120826</t>
+  </si>
+  <si>
+    <t>0011034-70.2025.5.03.0071</t>
+  </si>
+  <si>
+    <t>Agrocerrado Produtos Agrícolas E Assistência Técnica Ltda.</t>
+  </si>
+  <si>
+    <t>Yure De Andrade Barbosa</t>
+  </si>
+  <si>
+    <t>PATOS DE MINAS</t>
+  </si>
+  <si>
+    <t>R$             339.933,31</t>
   </si>
   <si>
     <t>VRO</t>
   </si>
   <si>
-    <t>link pendente</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>1001059-81.2026.5.02.0432</t>
-  </si>
-  <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Danilo Vieira Dos Santos Andrade Alves</t>
-  </si>
-  <si>
-    <t>SANTO ANDRÉ</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>02ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Instrução</t>
-  </si>
-  <si>
-    <t>R$             494.873,71</t>
-  </si>
-  <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>GSM</t>
-  </si>
-  <si>
-    <t>TAM</t>
-  </si>
-  <si>
-    <t>Presencial</t>
+    <t>https://trt3-jus-br.zoom.us/my/vt.patosdeminas</t>
+  </si>
+  <si>
+    <t>0010034-31.2025.5.15.0126</t>
+  </si>
+  <si>
+    <t>Rafael Gustavo Silva</t>
+  </si>
+  <si>
+    <t>Central</t>
+  </si>
+  <si>
+    <t>R$             203.419,69</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/9973700634?pwd=dENDekhCNjFLekRnSExiTzhmK1VLdz09 ID da reunião: 997 370 0634 Senha: 592209</t>
+  </si>
+  <si>
+    <t>0010505-52.2024.5.15.0071</t>
+  </si>
+  <si>
+    <t>Fabio Moreira</t>
+  </si>
+  <si>
+    <t>R$             563.053,70</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/83830687320?pwd=aH38p2gWpjsX9F8as5Kbdm0NEYva5j.1 ID:  838  3068  7320  Senha: 344918</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -200,6 +665,14 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -279,10 +752,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -305,8 +779,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -638,11 +1116,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51B4729B-FAA5-4A97-A1A6-CF400177BBD1}">
-  <dimension ref="A1:R3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13735AE5-06B2-4737-BCA1-0F280F973E76}">
+  <dimension ref="A1:R25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="52.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="130.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="60" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -698,15 +1195,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="84.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>104778</v>
+        <v>92215</v>
       </c>
       <c r="B2" s="5">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="C2" s="6">
-        <v>0.4375</v>
+        <v>0.35416666666666669</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>18</v>
@@ -748,39 +1245,39 @@
         <v>30</v>
       </c>
       <c r="Q2" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="R2" s="7" t="s">
         <v>31</v>
       </c>
+      <c r="R2" s="8" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="3" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
-        <v>105181</v>
+        <v>105287</v>
       </c>
       <c r="B3" s="5">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="C3" s="6">
-        <v>0.4513888888888889</v>
+        <v>0.37569444444444444</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="J3" s="7" t="s">
         <v>38</v>
@@ -806,11 +1303,1265 @@
       <c r="Q3" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="R3" s="7" t="s">
+      <c r="R3" s="8" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>105371</v>
+      </c>
+      <c r="B4" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0.38541666666666669</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>104298</v>
+      </c>
+      <c r="B5" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.40625</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P5" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="R5" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>105365</v>
+      </c>
+      <c r="B6" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0.40625</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="R6" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>105474</v>
+      </c>
+      <c r="B7" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C7" s="6">
+        <v>0.42916666666666664</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="R7" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>105014</v>
+      </c>
+      <c r="B8" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q8" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="R8" s="8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>103125</v>
+      </c>
+      <c r="B9" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N9" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="O9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P9" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="R9" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>103838</v>
+      </c>
+      <c r="B10" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0.47222222222222221</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="O10" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P10" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q10" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="R10" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>104044</v>
+      </c>
+      <c r="B11" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.4861111111111111</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N11" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="O11" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="P11" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q11" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="R11" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>105165</v>
+      </c>
+      <c r="B12" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.5625</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="O12" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P12" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q12" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="R12" s="8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>99370</v>
+      </c>
+      <c r="B13" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.5625</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N13" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="O13" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P13" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q13" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="R13" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>92711</v>
+      </c>
+      <c r="B14" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.625</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N14" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="O14" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P14" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q14" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="R14" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>103737</v>
+      </c>
+      <c r="B15" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.625</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="O15" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="P15" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q15" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="R15" s="8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
+        <v>101919</v>
+      </c>
+      <c r="B16" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.625</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N16" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="O16" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P16" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q16" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="R16" s="8" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>82990</v>
+      </c>
+      <c r="B17" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.62847222222222221</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N17" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="O17" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P17" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="R17" s="8" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>103309</v>
+      </c>
+      <c r="B18" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.63541666666666663</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="O18" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="R18" s="8" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>104995</v>
+      </c>
+      <c r="B19" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.63541666666666663</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M19" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N19" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="O19" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P19" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q19" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="R19" s="8" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>97789</v>
+      </c>
+      <c r="B20" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N20" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="O20" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P20" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q20" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="R20" s="8" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="4">
+        <v>103509</v>
+      </c>
+      <c r="B21" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0.65277777777777779</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J21" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N21" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="O21" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="P21" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q21" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="R21" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="4">
+        <v>77958</v>
+      </c>
+      <c r="B22" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0.65416666666666667</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N22" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="O22" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="P22" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q22" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="R22" s="8" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="4">
+        <v>101625</v>
+      </c>
+      <c r="B23" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.65972222222222221</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N23" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="O23" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P23" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q23" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="R23" s="8" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="4">
+        <v>99569</v>
+      </c>
+      <c r="B24" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C24" s="6">
+        <v>0.68055555555555558</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="N24" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="O24" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P24" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q24" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="R24" s="8" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="4">
+        <v>97460</v>
+      </c>
+      <c r="B25" s="5">
+        <v>46230</v>
+      </c>
+      <c r="C25" s="6">
+        <v>0.6875</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N25" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="O25" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P25" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q25" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="R25" s="8" t="s">
+        <v>199</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="R2" r:id="rId1" display="https://us02web.zoom.us/j/88415253122?pwd=QzlTNmxwdWpEeGVFZmdwM0lDUFJ4Zz09%20ID%20da%20reunião:%20884%201525%203122%20Senha%20de%20acesso:%20510562" xr:uid="{591A07F9-2959-4919-93CB-A3AD9304DD90}"/>
+    <hyperlink ref="R5" r:id="rId2" display="https://trt15-jus-br.zoom.us/j/88215751954?pwd=GWf0av1x8hFikMFre3DVbJa2NJn80H.1%20ID%20da%20reunião%20882%201575%201954%20Senha%20%20150077" xr:uid="{067DD09A-0EC6-4278-890B-CF419561F02A}"/>
+    <hyperlink ref="R6" r:id="rId3" display="https://us02web.zoom.us/j/81757243738?pwd=UXAvdEpveHlrNU05M2ZsZnRrYy9Vdz09%20ID%20DA%20REUNIÃO:%20817%205724%203738%20SENHA:%20954332" xr:uid="{B2DD1349-1814-4899-9D35-77EB8EBCBC43}"/>
+    <hyperlink ref="R7" r:id="rId4" xr:uid="{C517338F-BF6E-4815-BB46-A88C49F929AC}"/>
+    <hyperlink ref="R8" r:id="rId5" display="https://trt15-jus-br.zoom.us/j/88542672682?pwd=7pQ4QRhZmRG9RAQAWKowymbwNawa7t.1%20ID%20da%20reunião:%20885%204267%202682%20Senha%20de%20acesso:%20050728" xr:uid="{59AEE509-077F-461E-9314-87D03BD0B448}"/>
+    <hyperlink ref="R9" r:id="rId6" xr:uid="{648E61A8-9F6E-4E73-8CD0-B4FBD6086661}"/>
+    <hyperlink ref="R11" r:id="rId7" display="https://trt15-jus-br.zoom.us/j/83676367506?pwd=VlRlWmFnUGhwdWp3Y2xvaVkxdDFDZz09%20ID%20da%20reunião:%20836%207636%207506%20Senha:%2024680" xr:uid="{E889D12B-1848-4153-AC54-D6C3647678FE}"/>
+    <hyperlink ref="R12" r:id="rId8" display="mailto:ricardo.baracho@gmail.com" xr:uid="{3A81362D-D5EA-4E7E-BC56-43321FD4C0FE}"/>
+    <hyperlink ref="R13" r:id="rId9" display="https://trt15-jus-br.zoom.us/j/81907928214?pwd=DdJyPKEOQWb3pMKbKp713raBQMIpao.1%20ID:%20%20819%20%200792%20%208214%20%20Senha:%20935266." xr:uid="{14E0A554-F290-43F7-A5B4-91284EF9793E}"/>
+    <hyperlink ref="R14" r:id="rId10" display="https://trt15-jus-br.zoom.us/j/88971005711?pwd=FCU0CcOJlu66H4VR8hrXW2o1KrrqXb.1%20ID:%20889%20%207100%20%205711%20%20Senha:%20962801" xr:uid="{B38FEA93-2EC5-432E-8D77-F6DC75149635}"/>
+    <hyperlink ref="R15" r:id="rId11" xr:uid="{E02D146A-9473-424B-AEE4-80949E395D81}"/>
+    <hyperlink ref="R16" r:id="rId12" display="https://trt15-jus-br.zoom.us/j/87527564652?pwd=d3YrZ2diWXk5UjgzbmVkNExteWVMQT09%20ID%20da%20reunião:%20875%202756%204652%20Senha%20de%20acesso:%20246680" xr:uid="{301A4E52-2401-49D3-AB83-5006CD159FC4}"/>
+    <hyperlink ref="R17" r:id="rId13" xr:uid="{EA8C0CEC-5A38-4E3C-B488-E87D867BFF7E}"/>
+    <hyperlink ref="R18" r:id="rId14" display="https://trt3-jus-br.zoom.us/my/varabh12" xr:uid="{99E2392B-36B5-4EEA-AE2F-A06B31DD07B3}"/>
+    <hyperlink ref="R19" r:id="rId15" xr:uid="{E70BECCF-3D50-4A17-81D8-494A89B803DD}"/>
+    <hyperlink ref="R20" r:id="rId16" display="https://trt15-jus-br.zoom.us/j/87345253855?pwd=eOmaFv9ph0gYOdbdibavbZapr1i2NE.1%20ID:%20%20873%20%204525%20%203855%20%20Senha:%20223572" xr:uid="{E0F1D676-88B0-4FDF-B3F6-708CA714FCFF}"/>
+    <hyperlink ref="R22" r:id="rId17" display="https://trt2-jus-br.zoom.us/j/87687135814?pwd=L21Bd0RobFB3V0I0VVpuMlBDUG5oUT09%20ID%20da%20reunião:%20876%208713%205814%20Senha%20de%20acesso:%20120826" xr:uid="{9DF4C4D4-34F6-42C0-B7B1-25ED187815ED}"/>
+    <hyperlink ref="R23" r:id="rId18" xr:uid="{61FFECE7-17FA-44C5-97E9-FF073B29FF08}"/>
+    <hyperlink ref="R24" r:id="rId19" display="https://trt15-jus-br.zoom.us/j/9973700634?pwd=dENDekhCNjFLekRnSExiTzhmK1VLdz09%20ID%20da%20reunião:%20997%20370%200634%20Senha:%20592209" xr:uid="{D2A4FA29-D901-4C8E-ABB0-AA40B517722E}"/>
+    <hyperlink ref="R25" r:id="rId20" display="https://trt15-jus-br.zoom.us/j/83830687320?pwd=aH38p2gWpjsX9F8as5Kbdm0NEYva5j.1%20ID:%20%20838%20%203068%20%207320%20%20Senha:%20344918" xr:uid="{217039DE-0FCC-46C4-B2A3-3167A281CD73}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Audiências: sync 2026-07-27 — 24 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="117">
   <si>
     <t>data</t>
   </si>
@@ -49,49 +49,322 @@
     <t>horario</t>
   </si>
   <si>
-    <t>Fatal</t>
-  </si>
-  <si>
-    <t>VRO</t>
+    <t>D-1</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>Correspondente - Carlos Florian</t>
+  </si>
+  <si>
+    <t>ALF</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>JNE</t>
+  </si>
+  <si>
+    <t>FCG</t>
+  </si>
+  <si>
+    <t>DPR</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>Correspondente - doc9</t>
+  </si>
+  <si>
+    <t>JPL</t>
+  </si>
+  <si>
+    <t>PSI</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>RRU</t>
+  </si>
+  <si>
+    <t>TLI</t>
   </si>
   <si>
     <t>GSM</t>
   </si>
   <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
     <t>Grupo E1</t>
   </si>
   <si>
     <t>Grupo B1</t>
   </si>
   <si>
-    <t>Produtécnica Nordeste Comércio De Insumos Agrícolas Ltda.</t>
+    <t>Grupo C</t>
+  </si>
+  <si>
+    <t>Grupo B3</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Mahle Metal Leve S.A.</t>
+  </si>
+  <si>
+    <t>Robert Bosch Limitada</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
   </si>
   <si>
     <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
   </si>
   <si>
+    <t>Fertilizantes Tocantins S.A</t>
+  </si>
+  <si>
+    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
+  </si>
+  <si>
+    <t>Viterra Bioenergia S.A.</t>
+  </si>
+  <si>
+    <t>Ferrero Do Brasil Indústria Doceira E Alimentar Ltda.</t>
+  </si>
+  <si>
+    <t>Frutal Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Agrocerrado Produtos Agrícolas E Assistência Técnica Ltda.</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Presencial</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Telepresencial</t>
+  </si>
+  <si>
     <t>Audiência Instrução - Telepresencial</t>
   </si>
   <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>0000431-17.2026.5.10.0811</t>
-  </si>
-  <si>
-    <t>1001059-81.2026.5.02.0432</t>
-  </si>
-  <si>
-    <t>Jhony Carlos Lucena Cardoso</t>
-  </si>
-  <si>
-    <t>Danilo Vieira Dos Santos Andrade Alves</t>
-  </si>
-  <si>
-    <t>10:30:00</t>
-  </si>
-  <si>
-    <t>10:50:00</t>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>0010556-64.2023.5.15.0082</t>
+  </si>
+  <si>
+    <t>1000973-20.2026.5.02.0462</t>
+  </si>
+  <si>
+    <t>1001013-02.2026.5.02.0462</t>
+  </si>
+  <si>
+    <t>0014731-48.2025.5.15.0077</t>
+  </si>
+  <si>
+    <t>0011763-13.2026.5.15.0044</t>
+  </si>
+  <si>
+    <t>0000846-69.2026.5.05.0251</t>
+  </si>
+  <si>
+    <t>0010954-47.2026.5.15.0133</t>
+  </si>
+  <si>
+    <t>0001673-39.2025.5.13.0010</t>
+  </si>
+  <si>
+    <t>0010064-52.2026.5.15.0087</t>
+  </si>
+  <si>
+    <t>0010295-44.2026.5.15.0131</t>
+  </si>
+  <si>
+    <t>0000761-97.2026.5.17.0009</t>
+  </si>
+  <si>
+    <t>0011575-56.2024.5.15.0087</t>
+  </si>
+  <si>
+    <t>0010718-92.2023.5.15.0071</t>
+  </si>
+  <si>
+    <t>0000010-77.2026.5.09.0092</t>
+  </si>
+  <si>
+    <t>0010907-03.2025.5.15.0103</t>
+  </si>
+  <si>
+    <t>0010466-75.2022.5.15.0087</t>
+  </si>
+  <si>
+    <t>0011112-47.2025.5.03.0012</t>
+  </si>
+  <si>
+    <t>0010432-81.2026.5.03.0156</t>
+  </si>
+  <si>
+    <t>0010828-57.2024.5.15.0071</t>
+  </si>
+  <si>
+    <t>1002332-26.2025.5.02.0434</t>
+  </si>
+  <si>
+    <t>1000813-89.2020.5.02.0434</t>
+  </si>
+  <si>
+    <t>0011034-70.2025.5.03.0071</t>
+  </si>
+  <si>
+    <t>0010034-31.2025.5.15.0126</t>
+  </si>
+  <si>
+    <t>0010505-52.2024.5.15.0071</t>
+  </si>
+  <si>
+    <t>Miguel Jose De Souza</t>
+  </si>
+  <si>
+    <t>Sonia Soares Almeida</t>
+  </si>
+  <si>
+    <t>Davi Joao Da Silva</t>
+  </si>
+  <si>
+    <t>Ismael Jose Dos Santos</t>
+  </si>
+  <si>
+    <t>Matheus Felipe Januario Domingues</t>
+  </si>
+  <si>
+    <t>Gilson Meireles Dos Santos</t>
+  </si>
+  <si>
+    <t>Edivaldo Aparecido De Oliveira</t>
+  </si>
+  <si>
+    <t>Willan Hilario Marcelino</t>
+  </si>
+  <si>
+    <t>Jessica Nunes Da Silva</t>
+  </si>
+  <si>
+    <t>Marcos Paulo Leite</t>
+  </si>
+  <si>
+    <t>Edilcivane Pereira Ottoni</t>
+  </si>
+  <si>
+    <t>Wesley Felipe Cezar Xavier</t>
+  </si>
+  <si>
+    <t>Claudio Richard De Godoy</t>
+  </si>
+  <si>
+    <t>Darlan Silva Quintiliano</t>
+  </si>
+  <si>
+    <t>Jeanio Berto Da Costa E Silva</t>
+  </si>
+  <si>
+    <t>Sidkley Jose Da Silva</t>
+  </si>
+  <si>
+    <t>Lucimar Da Silva Costa</t>
+  </si>
+  <si>
+    <t>Joao Batista Loiola De Sousa</t>
+  </si>
+  <si>
+    <t>Luciano Vicentim Da Cruz</t>
+  </si>
+  <si>
+    <t>Cesar Luiz Do Amaral</t>
+  </si>
+  <si>
+    <t>Alan Alves Sarmento</t>
+  </si>
+  <si>
+    <t>Yure De Andrade Barbosa</t>
+  </si>
+  <si>
+    <t>Rafael Gustavo Silva</t>
+  </si>
+  <si>
+    <t>Fabio Moreira</t>
+  </si>
+  <si>
+    <t>08:30:00</t>
+  </si>
+  <si>
+    <t>09:01:00</t>
+  </si>
+  <si>
+    <t>09:15:00</t>
+  </si>
+  <si>
+    <t>09:45:00</t>
+  </si>
+  <si>
+    <t>10:18:00</t>
+  </si>
+  <si>
+    <t>11:00:00</t>
+  </si>
+  <si>
+    <t>11:20:00</t>
+  </si>
+  <si>
+    <t>11:40:00</t>
+  </si>
+  <si>
+    <t>13:30:00</t>
+  </si>
+  <si>
+    <t>15:00:00</t>
+  </si>
+  <si>
+    <t>15:05:00</t>
+  </si>
+  <si>
+    <t>15:15:00</t>
+  </si>
+  <si>
+    <t>15:30:00</t>
+  </si>
+  <si>
+    <t>15:40:00</t>
+  </si>
+  <si>
+    <t>15:42:00</t>
+  </si>
+  <si>
+    <t>15:50:00</t>
+  </si>
+  <si>
+    <t>16:20:00</t>
+  </si>
+  <si>
+    <t>16:30:00</t>
   </si>
 </sst>
 </file>
@@ -427,7 +700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -467,7 +740,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="1">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -476,33 +749,33 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F2" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="H2" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="I2" t="s">
-        <v>22</v>
+        <v>75</v>
       </c>
       <c r="J2" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="K2" t="s">
-        <v>24</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="1">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
@@ -511,28 +784,798 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I3" t="s">
+        <v>76</v>
+      </c>
+      <c r="J3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" t="s">
+        <v>45</v>
+      </c>
+      <c r="H4" t="s">
+        <v>53</v>
+      </c>
+      <c r="I4" t="s">
+        <v>77</v>
+      </c>
+      <c r="J4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" t="s">
+        <v>46</v>
+      </c>
+      <c r="H5" t="s">
+        <v>54</v>
+      </c>
+      <c r="I5" t="s">
+        <v>78</v>
+      </c>
+      <c r="J5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" t="s">
+        <v>46</v>
+      </c>
+      <c r="H6" t="s">
+        <v>55</v>
+      </c>
+      <c r="I6" t="s">
+        <v>79</v>
+      </c>
+      <c r="J6" t="s">
+        <v>32</v>
+      </c>
+      <c r="K6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J7" t="s">
+        <v>35</v>
+      </c>
+      <c r="K7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
         <v>17</v>
       </c>
-      <c r="F3" t="s">
+      <c r="D9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" t="s">
+        <v>58</v>
+      </c>
+      <c r="I9" t="s">
+        <v>82</v>
+      </c>
+      <c r="J9" t="s">
+        <v>32</v>
+      </c>
+      <c r="K9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" t="s">
+        <v>47</v>
+      </c>
+      <c r="H10" t="s">
+        <v>59</v>
+      </c>
+      <c r="I10" t="s">
+        <v>83</v>
+      </c>
+      <c r="J10" t="s">
+        <v>36</v>
+      </c>
+      <c r="K10" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
         <v>19</v>
       </c>
-      <c r="G3" t="s">
+      <c r="D11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" t="s">
+        <v>46</v>
+      </c>
+      <c r="G11" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" t="s">
+        <v>60</v>
+      </c>
+      <c r="I11" t="s">
+        <v>84</v>
+      </c>
+      <c r="J11" t="s">
+        <v>37</v>
+      </c>
+      <c r="K11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" t="s">
+        <v>45</v>
+      </c>
+      <c r="H12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I12" t="s">
+        <v>85</v>
+      </c>
+      <c r="J12" t="s">
+        <v>38</v>
+      </c>
+      <c r="K12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" t="s">
+        <v>44</v>
+      </c>
+      <c r="H13" t="s">
+        <v>62</v>
+      </c>
+      <c r="I13" t="s">
+        <v>86</v>
+      </c>
+      <c r="J13" t="s">
+        <v>36</v>
+      </c>
+      <c r="K13" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G14" t="s">
+        <v>44</v>
+      </c>
+      <c r="H14" t="s">
+        <v>63</v>
+      </c>
+      <c r="I14" t="s">
+        <v>87</v>
+      </c>
+      <c r="J14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K14" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" t="s">
+        <v>39</v>
+      </c>
+      <c r="F15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G15" t="s">
+        <v>48</v>
+      </c>
+      <c r="H15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I15" t="s">
+        <v>88</v>
+      </c>
+      <c r="J15" t="s">
+        <v>39</v>
+      </c>
+      <c r="K15" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" t="s">
+        <v>49</v>
+      </c>
+      <c r="G16" t="s">
+        <v>49</v>
+      </c>
+      <c r="H16" t="s">
+        <v>65</v>
+      </c>
+      <c r="I16" t="s">
+        <v>89</v>
+      </c>
+      <c r="J16" t="s">
+        <v>40</v>
+      </c>
+      <c r="K16" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" t="s">
+        <v>44</v>
+      </c>
+      <c r="G17" t="s">
+        <v>44</v>
+      </c>
+      <c r="H17" t="s">
+        <v>66</v>
+      </c>
+      <c r="I17" t="s">
+        <v>90</v>
+      </c>
+      <c r="J17" t="s">
+        <v>36</v>
+      </c>
+      <c r="K17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" t="s">
+        <v>50</v>
+      </c>
+      <c r="G18" t="s">
+        <v>50</v>
+      </c>
+      <c r="H18" t="s">
+        <v>67</v>
+      </c>
+      <c r="I18" t="s">
+        <v>91</v>
+      </c>
+      <c r="J18" t="s">
+        <v>41</v>
+      </c>
+      <c r="K18" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" t="s">
+        <v>42</v>
+      </c>
+      <c r="F19" t="s">
+        <v>49</v>
+      </c>
+      <c r="G19" t="s">
+        <v>49</v>
+      </c>
+      <c r="H19" t="s">
+        <v>68</v>
+      </c>
+      <c r="I19" t="s">
+        <v>92</v>
+      </c>
+      <c r="J19" t="s">
+        <v>42</v>
+      </c>
+      <c r="K19" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20" t="s">
+        <v>44</v>
+      </c>
+      <c r="G20" t="s">
+        <v>44</v>
+      </c>
+      <c r="H20" t="s">
+        <v>69</v>
+      </c>
+      <c r="I20" t="s">
+        <v>93</v>
+      </c>
+      <c r="J20" t="s">
+        <v>33</v>
+      </c>
+      <c r="K20" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" t="s">
+        <v>29</v>
+      </c>
+      <c r="E21" t="s">
+        <v>37</v>
+      </c>
+      <c r="F21" t="s">
+        <v>50</v>
+      </c>
+      <c r="G21" t="s">
+        <v>50</v>
+      </c>
+      <c r="H21" t="s">
+        <v>70</v>
+      </c>
+      <c r="I21" t="s">
+        <v>94</v>
+      </c>
+      <c r="J21" t="s">
+        <v>37</v>
+      </c>
+      <c r="K21" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" t="s">
         <v>19</v>
       </c>
-      <c r="H3" t="s">
+      <c r="D22" t="s">
+        <v>29</v>
+      </c>
+      <c r="E22" t="s">
+        <v>37</v>
+      </c>
+      <c r="F22" t="s">
+        <v>44</v>
+      </c>
+      <c r="G22" t="s">
+        <v>44</v>
+      </c>
+      <c r="H22" t="s">
+        <v>71</v>
+      </c>
+      <c r="I22" t="s">
+        <v>95</v>
+      </c>
+      <c r="J22" t="s">
+        <v>37</v>
+      </c>
+      <c r="K22" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B23" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" t="s">
+        <v>28</v>
+      </c>
+      <c r="E23" t="s">
+        <v>43</v>
+      </c>
+      <c r="F23" t="s">
+        <v>48</v>
+      </c>
+      <c r="G23" t="s">
+        <v>48</v>
+      </c>
+      <c r="H23" t="s">
+        <v>72</v>
+      </c>
+      <c r="I23" t="s">
+        <v>96</v>
+      </c>
+      <c r="J23" t="s">
+        <v>43</v>
+      </c>
+      <c r="K23" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" t="s">
         <v>21</v>
       </c>
-      <c r="I3" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" t="s">
-        <v>25</v>
+      <c r="D24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" t="s">
+        <v>36</v>
+      </c>
+      <c r="F24" t="s">
+        <v>49</v>
+      </c>
+      <c r="G24" t="s">
+        <v>49</v>
+      </c>
+      <c r="H24" t="s">
+        <v>73</v>
+      </c>
+      <c r="I24" t="s">
+        <v>97</v>
+      </c>
+      <c r="J24" t="s">
+        <v>36</v>
+      </c>
+      <c r="K24" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" t="s">
+        <v>22</v>
+      </c>
+      <c r="D25" t="s">
+        <v>28</v>
+      </c>
+      <c r="E25" t="s">
+        <v>33</v>
+      </c>
+      <c r="F25" t="s">
+        <v>44</v>
+      </c>
+      <c r="G25" t="s">
+        <v>44</v>
+      </c>
+      <c r="H25" t="s">
+        <v>74</v>
+      </c>
+      <c r="I25" t="s">
+        <v>98</v>
+      </c>
+      <c r="J25" t="s">
+        <v>33</v>
+      </c>
+      <c r="K25" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Audiências: sync 2026-07-28 — 29 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="137">
   <si>
     <t>data</t>
   </si>
@@ -49,52 +49,64 @@
     <t>horario</t>
   </si>
   <si>
-    <t>Fatal</t>
+    <t>D-1</t>
+  </si>
+  <si>
+    <t>BSO</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>CAL</t>
+  </si>
+  <si>
+    <t>Correspondente - Ana</t>
+  </si>
+  <si>
+    <t>ANB</t>
+  </si>
+  <si>
+    <t>JPL</t>
   </si>
   <si>
     <t>MBF</t>
   </si>
   <si>
-    <t>Correspondente - Carlos Florian</t>
-  </si>
-  <si>
-    <t>ALF</t>
-  </si>
-  <si>
-    <t>RYL</t>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>ARC</t>
   </si>
   <si>
     <t>JNE</t>
   </si>
   <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>BCF</t>
+  </si>
+  <si>
+    <t>VCR</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>RRU</t>
+  </si>
+  <si>
+    <t>PSI</t>
+  </si>
+  <si>
     <t>FCG</t>
   </si>
   <si>
-    <t>DPR</t>
-  </si>
-  <si>
-    <t>JPE</t>
-  </si>
-  <si>
-    <t>Correspondente - doc9</t>
-  </si>
-  <si>
-    <t>JPL</t>
-  </si>
-  <si>
-    <t>PSI</t>
-  </si>
-  <si>
-    <t>VSI</t>
-  </si>
-  <si>
-    <t>RRU</t>
-  </si>
-  <si>
     <t>TLI</t>
   </si>
   <si>
-    <t>GSM</t>
+    <t>Grupo B1</t>
   </si>
   <si>
     <t>Grupo E2</t>
@@ -103,268 +115,316 @@
     <t>Grupo E1</t>
   </si>
   <si>
-    <t>Grupo B1</t>
+    <t>Grupo B2</t>
   </si>
   <si>
     <t>Grupo C</t>
   </si>
   <si>
-    <t>Grupo B3</t>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>A. Raymond Brasil Ltda.</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A</t>
+  </si>
+  <si>
+    <t>Mahle Metal Leve S.A.</t>
+  </si>
+  <si>
+    <t>Embraer S.A.</t>
+  </si>
+  <si>
+    <t>Syngenta Seeds Ltda.</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A. - Candeias - Can</t>
+  </si>
+  <si>
+    <t>Guariroba Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Telefonica Brasil S.A.</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda.</t>
+  </si>
+  <si>
+    <t>Viterra Bioenergia S.A.</t>
   </si>
   <si>
     <t>Moema Bioenergia S.A. - Moema</t>
   </si>
   <si>
-    <t>Mahle Metal Leve S.A.</t>
-  </si>
-  <si>
-    <t>Robert Bosch Limitada</t>
-  </si>
-  <si>
-    <t>Salitre Fertilizantes Ltda</t>
-  </si>
-  <si>
-    <t>Syngenta Proteção De Cultivos Ltda.</t>
-  </si>
-  <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Fertilizantes Tocantins S.A</t>
-  </si>
-  <si>
-    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
-  </si>
-  <si>
-    <t>Viterra Bioenergia S.A.</t>
-  </si>
-  <si>
-    <t>Ferrero Do Brasil Indústria Doceira E Alimentar Ltda.</t>
-  </si>
-  <si>
-    <t>Frutal Bioenergia Ltda.</t>
-  </si>
-  <si>
-    <t>Agrocerrado Produtos Agrícolas E Assistência Técnica Ltda.</t>
+    <t>Audiência Inicial - Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Semipresencial</t>
   </si>
   <si>
     <t>Audiência de Conciliação - Telepresencial</t>
   </si>
   <si>
-    <t>Audiência Una - Presencial</t>
+    <t>Audiência Inicial - Presencial</t>
   </si>
   <si>
     <t>Audiência Inicial -  Telepresencial</t>
   </si>
   <si>
-    <t>Audiência Inicial - Presencial</t>
-  </si>
-  <si>
-    <t>Audiência de Instrução - Telepresencial</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Telepresencial</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>0010556-64.2023.5.15.0082</t>
-  </si>
-  <si>
-    <t>1000973-20.2026.5.02.0462</t>
-  </si>
-  <si>
-    <t>1001013-02.2026.5.02.0462</t>
-  </si>
-  <si>
-    <t>0014731-48.2025.5.15.0077</t>
-  </si>
-  <si>
-    <t>0011763-13.2026.5.15.0044</t>
-  </si>
-  <si>
-    <t>0000846-69.2026.5.05.0251</t>
-  </si>
-  <si>
-    <t>0010954-47.2026.5.15.0133</t>
-  </si>
-  <si>
-    <t>0001673-39.2025.5.13.0010</t>
-  </si>
-  <si>
-    <t>0010064-52.2026.5.15.0087</t>
-  </si>
-  <si>
-    <t>0010295-44.2026.5.15.0131</t>
-  </si>
-  <si>
-    <t>0000761-97.2026.5.17.0009</t>
-  </si>
-  <si>
-    <t>0011575-56.2024.5.15.0087</t>
-  </si>
-  <si>
-    <t>0010718-92.2023.5.15.0071</t>
-  </si>
-  <si>
-    <t>0000010-77.2026.5.09.0092</t>
-  </si>
-  <si>
-    <t>0010907-03.2025.5.15.0103</t>
-  </si>
-  <si>
-    <t>0010466-75.2022.5.15.0087</t>
-  </si>
-  <si>
-    <t>0011112-47.2025.5.03.0012</t>
-  </si>
-  <si>
-    <t>0010432-81.2026.5.03.0156</t>
-  </si>
-  <si>
-    <t>0010828-57.2024.5.15.0071</t>
-  </si>
-  <si>
-    <t>1002332-26.2025.5.02.0434</t>
-  </si>
-  <si>
-    <t>1000813-89.2020.5.02.0434</t>
-  </si>
-  <si>
-    <t>0011034-70.2025.5.03.0071</t>
-  </si>
-  <si>
-    <t>0010034-31.2025.5.15.0126</t>
-  </si>
-  <si>
-    <t>0010505-52.2024.5.15.0071</t>
-  </si>
-  <si>
-    <t>Miguel Jose De Souza</t>
-  </si>
-  <si>
-    <t>Sonia Soares Almeida</t>
-  </si>
-  <si>
-    <t>Davi Joao Da Silva</t>
-  </si>
-  <si>
-    <t>Ismael Jose Dos Santos</t>
-  </si>
-  <si>
-    <t>Matheus Felipe Januario Domingues</t>
-  </si>
-  <si>
-    <t>Gilson Meireles Dos Santos</t>
-  </si>
-  <si>
-    <t>Edivaldo Aparecido De Oliveira</t>
-  </si>
-  <si>
-    <t>Willan Hilario Marcelino</t>
-  </si>
-  <si>
-    <t>Jessica Nunes Da Silva</t>
-  </si>
-  <si>
-    <t>Marcos Paulo Leite</t>
-  </si>
-  <si>
-    <t>Edilcivane Pereira Ottoni</t>
-  </si>
-  <si>
-    <t>Wesley Felipe Cezar Xavier</t>
-  </si>
-  <si>
-    <t>Claudio Richard De Godoy</t>
-  </si>
-  <si>
-    <t>Darlan Silva Quintiliano</t>
-  </si>
-  <si>
-    <t>Jeanio Berto Da Costa E Silva</t>
-  </si>
-  <si>
-    <t>Sidkley Jose Da Silva</t>
-  </si>
-  <si>
-    <t>Lucimar Da Silva Costa</t>
-  </si>
-  <si>
-    <t>Joao Batista Loiola De Sousa</t>
-  </si>
-  <si>
-    <t>Luciano Vicentim Da Cruz</t>
-  </si>
-  <si>
-    <t>Cesar Luiz Do Amaral</t>
-  </si>
-  <si>
-    <t>Alan Alves Sarmento</t>
-  </si>
-  <si>
-    <t>Yure De Andrade Barbosa</t>
-  </si>
-  <si>
-    <t>Rafael Gustavo Silva</t>
-  </si>
-  <si>
-    <t>Fabio Moreira</t>
-  </si>
-  <si>
-    <t>08:30:00</t>
-  </si>
-  <si>
-    <t>09:01:00</t>
-  </si>
-  <si>
-    <t>09:15:00</t>
+    <t>Audiência Inicial - Semipresencial</t>
+  </si>
+  <si>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Presencial</t>
+  </si>
+  <si>
+    <t>0010127-62.2026.5.15.0092</t>
+  </si>
+  <si>
+    <t>0010503-33.2026.5.15.0097</t>
+  </si>
+  <si>
+    <t>0011078-07.2025.5.03.0066</t>
+  </si>
+  <si>
+    <t>0011006-40.2023.5.15.0071</t>
+  </si>
+  <si>
+    <t>0011440-58.2021.5.15.0084</t>
+  </si>
+  <si>
+    <t>0010785-80.2024.5.03.0063</t>
+  </si>
+  <si>
+    <t>0000258-98.2025.5.05.0121</t>
+  </si>
+  <si>
+    <t>1000694-21.2026.5.02.0434</t>
+  </si>
+  <si>
+    <t>0000439-62.2026.5.05.0122</t>
+  </si>
+  <si>
+    <t>0000049-56.2026.5.05.0037</t>
+  </si>
+  <si>
+    <t>1000903-95.2026.5.02.0205</t>
+  </si>
+  <si>
+    <t>0010013-06.2025.5.15.0013</t>
+  </si>
+  <si>
+    <t>0011603-18.2025.5.15.0013</t>
+  </si>
+  <si>
+    <t>1001223-46.2026.5.02.0432</t>
+  </si>
+  <si>
+    <t>1001305-68.2026.5.02.0435</t>
+  </si>
+  <si>
+    <t>0010199-21.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>0010190-19.2026.5.15.0050</t>
+  </si>
+  <si>
+    <t>0010905-03.2023.5.15.0071</t>
+  </si>
+  <si>
+    <t>0010469-69.2026.5.15.0061</t>
+  </si>
+  <si>
+    <t>0010127-91.2026.5.15.0050</t>
+  </si>
+  <si>
+    <t>0011598-50.2024.5.15.0071</t>
+  </si>
+  <si>
+    <t>0010198-36.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>0011180-49.2023.5.15.0071</t>
+  </si>
+  <si>
+    <t>0010194-96.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>0010150-37.2026.5.15.0050</t>
+  </si>
+  <si>
+    <t>1001049-31.2026.5.02.0434</t>
+  </si>
+  <si>
+    <t>0011902-83.2023.5.15.0071</t>
+  </si>
+  <si>
+    <t>0012955-39.2025.5.15.0133</t>
+  </si>
+  <si>
+    <t>1000366-37.2025.5.02.0431</t>
+  </si>
+  <si>
+    <t>Weverson Frank Pinto De Carvalho</t>
+  </si>
+  <si>
+    <t>Leiliane Maria Da Rocha Nascimento Teixeira</t>
+  </si>
+  <si>
+    <t>Walleska Souza Menezes</t>
+  </si>
+  <si>
+    <t>Saulo De Tarso Da Silva</t>
+  </si>
+  <si>
+    <t>Maria Valdirene Santos Monteiro</t>
+  </si>
+  <si>
+    <t>Cristiano Felix Da Silva</t>
+  </si>
+  <si>
+    <t>Ryam Kedson Magalhaes Nascimento</t>
+  </si>
+  <si>
+    <t>Rubens Bernardes Da Silva</t>
+  </si>
+  <si>
+    <t>Vagner Bitencourt Dantas</t>
+  </si>
+  <si>
+    <t>Claudio Almeida Barbosa</t>
+  </si>
+  <si>
+    <t>Luciano Pompeo Pasqualini</t>
+  </si>
+  <si>
+    <t>Diego Vinicius Stabile David</t>
+  </si>
+  <si>
+    <t>Anderson Vilela Ribeiro</t>
+  </si>
+  <si>
+    <t>Edson Cavasso</t>
+  </si>
+  <si>
+    <t>Tiago Alves De Lima</t>
+  </si>
+  <si>
+    <t>Marcelo Antonio Lourenco</t>
+  </si>
+  <si>
+    <t>Luiz Marcos Dos Santos</t>
+  </si>
+  <si>
+    <t>Pablo Roberto Da Silva</t>
+  </si>
+  <si>
+    <t>Claudemir Moreira Mendes</t>
+  </si>
+  <si>
+    <t>Luiz Felipe Dos Santos Muniz</t>
+  </si>
+  <si>
+    <t>Osvaldo Ferreira</t>
+  </si>
+  <si>
+    <t>Jose Fidelis Ferreira</t>
+  </si>
+  <si>
+    <t>Viviane Domingues Lopes</t>
+  </si>
+  <si>
+    <t>Emerson Leandro De Jesus</t>
+  </si>
+  <si>
+    <t>Claudio Vinicius Ferreira Leite</t>
+  </si>
+  <si>
+    <t>Rafael Da Silva Sousa</t>
+  </si>
+  <si>
+    <t>Julio Cesar De Castro</t>
+  </si>
+  <si>
+    <t>Marcos Roberto Alves Da Silva</t>
+  </si>
+  <si>
+    <t>Akexsandra Lopes De Abreu</t>
+  </si>
+  <si>
+    <t>08:33:00</t>
+  </si>
+  <si>
+    <t>08:35:00</t>
+  </si>
+  <si>
+    <t>09:00:00</t>
+  </si>
+  <si>
+    <t>09:20:00</t>
+  </si>
+  <si>
+    <t>09:30:00</t>
+  </si>
+  <si>
+    <t>09:40:00</t>
   </si>
   <si>
     <t>09:45:00</t>
   </si>
   <si>
-    <t>10:18:00</t>
+    <t>10:00:00</t>
+  </si>
+  <si>
+    <t>10:13:00</t>
   </si>
   <si>
     <t>11:00:00</t>
   </si>
   <si>
-    <t>11:20:00</t>
-  </si>
-  <si>
-    <t>11:40:00</t>
+    <t>11:10:00</t>
+  </si>
+  <si>
+    <t>11:15:00</t>
+  </si>
+  <si>
+    <t>12:00:00</t>
   </si>
   <si>
     <t>13:30:00</t>
   </si>
   <si>
+    <t>13:35:00</t>
+  </si>
+  <si>
+    <t>14:00:00</t>
+  </si>
+  <si>
+    <t>14:15:00</t>
+  </si>
+  <si>
+    <t>14:30:00</t>
+  </si>
+  <si>
+    <t>14:40:00</t>
+  </si>
+  <si>
     <t>15:00:00</t>
   </si>
   <si>
-    <t>15:05:00</t>
-  </si>
-  <si>
-    <t>15:15:00</t>
-  </si>
-  <si>
-    <t>15:30:00</t>
-  </si>
-  <si>
-    <t>15:40:00</t>
+    <t>15:20:00</t>
   </si>
   <si>
     <t>15:42:00</t>
-  </si>
-  <si>
-    <t>15:50:00</t>
-  </si>
-  <si>
-    <t>16:20:00</t>
-  </si>
-  <si>
-    <t>16:30:00</t>
   </si>
 </sst>
 </file>
@@ -700,7 +760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -740,7 +800,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -749,33 +809,33 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="I2" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="J2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K2" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
@@ -784,628 +844,628 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="I3" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="J3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="K3" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H4" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="I4" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="J4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K4" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="H5" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="I5" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="J5" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="K5" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="I6" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="J6" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="K6" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="G7" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="H7" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I7" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="J7" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="K7" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="I8" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="J8" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="K8" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F9" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H9" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="I9" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="J9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K9" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F10" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="G10" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="H10" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I10" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="J10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K10" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E11" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F11" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G11" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="H11" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="I11" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="J11" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="K11" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B12" t="s">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="E12" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F12" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G12" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H12" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="I12" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="J12" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="K12" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E13" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F13" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="G13" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H13" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="I13" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="J13" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="K13" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E14" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F14" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="G14" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H14" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="I14" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="J14" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="K14" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B15" t="s">
         <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D15" t="s">
         <v>30</v>
       </c>
       <c r="E15" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F15" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="G15" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="H15" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I15" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="J15" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K15" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B16" t="s">
         <v>11</v>
       </c>
       <c r="C16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D16" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E16" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F16" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="G16" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="H16" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="I16" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="J16" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="K16" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B17" t="s">
         <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="F17" t="s">
+        <v>48</v>
+      </c>
+      <c r="G17" t="s">
+        <v>48</v>
+      </c>
+      <c r="H17" t="s">
+        <v>72</v>
+      </c>
+      <c r="I17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J17" t="s">
         <v>44</v>
       </c>
-      <c r="G17" t="s">
-        <v>44</v>
-      </c>
-      <c r="H17" t="s">
-        <v>66</v>
-      </c>
-      <c r="I17" t="s">
-        <v>90</v>
-      </c>
-      <c r="J17" t="s">
-        <v>36</v>
-      </c>
       <c r="K17" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B18" t="s">
         <v>11</v>
       </c>
       <c r="C18" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D18" t="s">
         <v>31</v>
       </c>
       <c r="E18" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H18" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="I18" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="J18" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="K18" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B19" t="s">
         <v>11</v>
       </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="D19" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E19" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F19" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G19" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H19" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I19" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="J19" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="K19" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B20" t="s">
         <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="F20" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G20" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H20" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="I20" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="J20" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="K20" t="s">
-        <v>111</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B21" t="s">
         <v>11</v>
@@ -1414,68 +1474,68 @@
         <v>26</v>
       </c>
       <c r="D21" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E21" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="F21" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G21" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H21" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="I21" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="J21" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="K21" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B22" t="s">
         <v>11</v>
       </c>
       <c r="C22" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="D22" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F22" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="G22" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="H22" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="I22" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="J22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K22" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B23" t="s">
         <v>11</v>
@@ -1484,10 +1544,10 @@
         <v>18</v>
       </c>
       <c r="D23" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E23" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F23" t="s">
         <v>48</v>
@@ -1496,86 +1556,261 @@
         <v>48</v>
       </c>
       <c r="H23" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="I23" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="J23" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K23" t="s">
-        <v>114</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B24" t="s">
         <v>11</v>
       </c>
       <c r="C24" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D24" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E24" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F24" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G24" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H24" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="I24" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="J24" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="K24" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B25" t="s">
         <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D25" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E25" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="F25" t="s">
+        <v>48</v>
+      </c>
+      <c r="G25" t="s">
+        <v>48</v>
+      </c>
+      <c r="H25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I25" t="s">
+        <v>109</v>
+      </c>
+      <c r="J25" t="s">
         <v>44</v>
       </c>
-      <c r="G25" t="s">
-        <v>44</v>
-      </c>
-      <c r="H25" t="s">
-        <v>74</v>
-      </c>
-      <c r="I25" t="s">
-        <v>98</v>
-      </c>
-      <c r="J25" t="s">
-        <v>33</v>
-      </c>
       <c r="K25" t="s">
-        <v>116</v>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
+      <c r="A26" s="1">
+        <v>46231</v>
+      </c>
+      <c r="B26" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" t="s">
+        <v>31</v>
+      </c>
+      <c r="E26" t="s">
+        <v>45</v>
+      </c>
+      <c r="F26" t="s">
+        <v>48</v>
+      </c>
+      <c r="G26" t="s">
+        <v>48</v>
+      </c>
+      <c r="H26" t="s">
+        <v>81</v>
+      </c>
+      <c r="I26" t="s">
+        <v>110</v>
+      </c>
+      <c r="J26" t="s">
+        <v>45</v>
+      </c>
+      <c r="K26" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27" s="1">
+        <v>46231</v>
+      </c>
+      <c r="B27" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" t="s">
+        <v>30</v>
+      </c>
+      <c r="E27" t="s">
+        <v>35</v>
+      </c>
+      <c r="F27" t="s">
+        <v>56</v>
+      </c>
+      <c r="G27" t="s">
+        <v>56</v>
+      </c>
+      <c r="H27" t="s">
+        <v>82</v>
+      </c>
+      <c r="I27" t="s">
+        <v>111</v>
+      </c>
+      <c r="J27" t="s">
+        <v>35</v>
+      </c>
+      <c r="K27" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
+      <c r="A28" s="1">
+        <v>46231</v>
+      </c>
+      <c r="B28" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" t="s">
+        <v>32</v>
+      </c>
+      <c r="E28" t="s">
+        <v>38</v>
+      </c>
+      <c r="F28" t="s">
+        <v>51</v>
+      </c>
+      <c r="G28" t="s">
+        <v>51</v>
+      </c>
+      <c r="H28" t="s">
+        <v>83</v>
+      </c>
+      <c r="I28" t="s">
+        <v>112</v>
+      </c>
+      <c r="J28" t="s">
+        <v>38</v>
+      </c>
+      <c r="K28" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
+      <c r="A29" s="1">
+        <v>46231</v>
+      </c>
+      <c r="B29" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E29" t="s">
+        <v>46</v>
+      </c>
+      <c r="F29" t="s">
+        <v>48</v>
+      </c>
+      <c r="G29" t="s">
+        <v>48</v>
+      </c>
+      <c r="H29" t="s">
+        <v>84</v>
+      </c>
+      <c r="I29" t="s">
+        <v>113</v>
+      </c>
+      <c r="J29" t="s">
+        <v>46</v>
+      </c>
+      <c r="K29" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
+      <c r="A30" s="1">
+        <v>46231</v>
+      </c>
+      <c r="B30" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" t="s">
+        <v>30</v>
+      </c>
+      <c r="E30" t="s">
+        <v>35</v>
+      </c>
+      <c r="F30" t="s">
+        <v>51</v>
+      </c>
+      <c r="G30" t="s">
+        <v>51</v>
+      </c>
+      <c r="H30" t="s">
+        <v>85</v>
+      </c>
+      <c r="I30" t="s">
+        <v>114</v>
+      </c>
+      <c r="J30" t="s">
+        <v>35</v>
+      </c>
+      <c r="K30" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Audiências: sync 2026-07-29 — 29 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="136">
   <si>
     <t>data</t>
   </si>
@@ -49,367 +49,364 @@
     <t>horario</t>
   </si>
   <si>
-    <t>Fatal</t>
-  </si>
-  <si>
-    <t>BSO</t>
+    <t>D-1</t>
+  </si>
+  <si>
+    <t>AAP</t>
+  </si>
+  <si>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>LMI</t>
+  </si>
+  <si>
+    <t>ANB</t>
+  </si>
+  <si>
+    <t>ARC</t>
   </si>
   <si>
     <t>RYL</t>
   </si>
   <si>
+    <t>FCG</t>
+  </si>
+  <si>
+    <t>TFR</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
     <t>CAL</t>
   </si>
   <si>
-    <t>Correspondente - Ana</t>
-  </si>
-  <si>
-    <t>ANB</t>
-  </si>
-  <si>
-    <t>JPL</t>
-  </si>
-  <si>
-    <t>MBF</t>
-  </si>
-  <si>
-    <t>Correspondente - Hebert</t>
-  </si>
-  <si>
-    <t>ARC</t>
+    <t>RRU</t>
+  </si>
+  <si>
+    <t>VCR</t>
+  </si>
+  <si>
+    <t>BCF</t>
   </si>
   <si>
     <t>JNE</t>
   </si>
   <si>
-    <t>VSI</t>
-  </si>
-  <si>
-    <t>BCF</t>
-  </si>
-  <si>
-    <t>VCR</t>
-  </si>
-  <si>
-    <t>JPE</t>
-  </si>
-  <si>
-    <t>RRU</t>
-  </si>
-  <si>
-    <t>PSI</t>
-  </si>
-  <si>
-    <t>FCG</t>
-  </si>
-  <si>
-    <t>TLI</t>
+    <t>Grupo E2</t>
   </si>
   <si>
     <t>Grupo B1</t>
   </si>
   <si>
-    <t>Grupo E2</t>
-  </si>
-  <si>
-    <t>Grupo E1</t>
+    <t>Grupo B3</t>
+  </si>
+  <si>
+    <t>Grupo C</t>
   </si>
   <si>
     <t>Grupo B2</t>
   </si>
   <si>
-    <t>Grupo C</t>
+    <t>Viterra Bioenergia S.A.</t>
   </si>
   <si>
     <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
   </si>
   <si>
-    <t>A. Raymond Brasil Ltda.</t>
-  </si>
-  <si>
-    <t>Fertilizantes Heringer S.A</t>
-  </si>
-  <si>
-    <t>Mahle Metal Leve S.A.</t>
+    <t>Companhia Brasileira De Cartuchos</t>
+  </si>
+  <si>
+    <t>Fertilizantes Tocantins S.A</t>
+  </si>
+  <si>
+    <t>Panificadora Cepam Ltda.</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Telefonica Brasil S.A.</t>
+  </si>
+  <si>
+    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda.</t>
+  </si>
+  <si>
+    <t>Guariroba Bioenergia Ltda.</t>
   </si>
   <si>
     <t>Embraer S.A.</t>
   </si>
   <si>
-    <t>Syngenta Seeds Ltda.</t>
-  </si>
-  <si>
-    <t>Fertilizantes Heringer S.A. - Candeias - Can</t>
-  </si>
-  <si>
-    <t>Guariroba Bioenergia Ltda.</t>
-  </si>
-  <si>
-    <t>Telefonica Brasil S.A.</t>
-  </si>
-  <si>
-    <t>Salitre Fertilizantes Ltda.</t>
-  </si>
-  <si>
-    <t>Viterra Bioenergia S.A.</t>
-  </si>
-  <si>
-    <t>Moema Bioenergia S.A. - Moema</t>
+    <t>Audiência de Conciliação - Semipresencial</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Presencial</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Presencial</t>
   </si>
   <si>
     <t>Audiência Inicial - Telepresencial</t>
   </si>
   <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
     <t>Audiência Instrução - Telepresencial</t>
   </si>
   <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>Sessão de Julgamento TRT - Semipresencial</t>
-  </si>
-  <si>
-    <t>Audiência de Conciliação - Telepresencial</t>
-  </si>
-  <si>
-    <t>Audiência Inicial - Presencial</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Telepresencial</t>
-  </si>
-  <si>
-    <t>Audiência Inicial - Semipresencial</t>
-  </si>
-  <si>
-    <t>Audiência Una - Telepresencial</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Presencial</t>
-  </si>
-  <si>
-    <t>0010127-62.2026.5.15.0092</t>
-  </si>
-  <si>
-    <t>0010503-33.2026.5.15.0097</t>
-  </si>
-  <si>
-    <t>0011078-07.2025.5.03.0066</t>
-  </si>
-  <si>
-    <t>0011006-40.2023.5.15.0071</t>
-  </si>
-  <si>
-    <t>0011440-58.2021.5.15.0084</t>
-  </si>
-  <si>
-    <t>0010785-80.2024.5.03.0063</t>
-  </si>
-  <si>
-    <t>0000258-98.2025.5.05.0121</t>
-  </si>
-  <si>
-    <t>1000694-21.2026.5.02.0434</t>
-  </si>
-  <si>
-    <t>0000439-62.2026.5.05.0122</t>
-  </si>
-  <si>
-    <t>0000049-56.2026.5.05.0037</t>
-  </si>
-  <si>
-    <t>1000903-95.2026.5.02.0205</t>
-  </si>
-  <si>
-    <t>0010013-06.2025.5.15.0013</t>
-  </si>
-  <si>
-    <t>0011603-18.2025.5.15.0013</t>
-  </si>
-  <si>
-    <t>1001223-46.2026.5.02.0432</t>
-  </si>
-  <si>
-    <t>1001305-68.2026.5.02.0435</t>
-  </si>
-  <si>
-    <t>0010199-21.2026.5.03.0080</t>
-  </si>
-  <si>
-    <t>0010190-19.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>0010905-03.2023.5.15.0071</t>
-  </si>
-  <si>
-    <t>0010469-69.2026.5.15.0061</t>
-  </si>
-  <si>
-    <t>0010127-91.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>0011598-50.2024.5.15.0071</t>
-  </si>
-  <si>
-    <t>0010198-36.2026.5.03.0080</t>
-  </si>
-  <si>
-    <t>0011180-49.2023.5.15.0071</t>
-  </si>
-  <si>
-    <t>0010194-96.2026.5.03.0080</t>
-  </si>
-  <si>
-    <t>0010150-37.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>1001049-31.2026.5.02.0434</t>
-  </si>
-  <si>
-    <t>0011902-83.2023.5.15.0071</t>
-  </si>
-  <si>
-    <t>0012955-39.2025.5.15.0133</t>
-  </si>
-  <si>
-    <t>1000366-37.2025.5.02.0431</t>
-  </si>
-  <si>
-    <t>Weverson Frank Pinto De Carvalho</t>
-  </si>
-  <si>
-    <t>Leiliane Maria Da Rocha Nascimento Teixeira</t>
-  </si>
-  <si>
-    <t>Walleska Souza Menezes</t>
-  </si>
-  <si>
-    <t>Saulo De Tarso Da Silva</t>
-  </si>
-  <si>
-    <t>Maria Valdirene Santos Monteiro</t>
-  </si>
-  <si>
-    <t>Cristiano Felix Da Silva</t>
-  </si>
-  <si>
-    <t>Ryam Kedson Magalhaes Nascimento</t>
-  </si>
-  <si>
-    <t>Rubens Bernardes Da Silva</t>
-  </si>
-  <si>
-    <t>Vagner Bitencourt Dantas</t>
-  </si>
-  <si>
-    <t>Claudio Almeida Barbosa</t>
-  </si>
-  <si>
-    <t>Luciano Pompeo Pasqualini</t>
-  </si>
-  <si>
-    <t>Diego Vinicius Stabile David</t>
-  </si>
-  <si>
-    <t>Anderson Vilela Ribeiro</t>
-  </si>
-  <si>
-    <t>Edson Cavasso</t>
-  </si>
-  <si>
-    <t>Tiago Alves De Lima</t>
-  </si>
-  <si>
-    <t>Marcelo Antonio Lourenco</t>
-  </si>
-  <si>
-    <t>Luiz Marcos Dos Santos</t>
-  </si>
-  <si>
-    <t>Pablo Roberto Da Silva</t>
-  </si>
-  <si>
-    <t>Claudemir Moreira Mendes</t>
-  </si>
-  <si>
-    <t>Luiz Felipe Dos Santos Muniz</t>
-  </si>
-  <si>
-    <t>Osvaldo Ferreira</t>
-  </si>
-  <si>
-    <t>Jose Fidelis Ferreira</t>
-  </si>
-  <si>
-    <t>Viviane Domingues Lopes</t>
-  </si>
-  <si>
-    <t>Emerson Leandro De Jesus</t>
-  </si>
-  <si>
-    <t>Claudio Vinicius Ferreira Leite</t>
-  </si>
-  <si>
-    <t>Rafael Da Silva Sousa</t>
-  </si>
-  <si>
-    <t>Julio Cesar De Castro</t>
-  </si>
-  <si>
-    <t>Marcos Roberto Alves Da Silva</t>
-  </si>
-  <si>
-    <t>Akexsandra Lopes De Abreu</t>
-  </si>
-  <si>
-    <t>08:33:00</t>
-  </si>
-  <si>
-    <t>08:35:00</t>
+    <t>Perícia Técnica</t>
+  </si>
+  <si>
+    <t>0010685-63.2026.5.15.0050</t>
+  </si>
+  <si>
+    <t>1000527-98.2026.5.02.0435</t>
+  </si>
+  <si>
+    <t>1000832-57.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>1000628-78.2025.5.02.0433</t>
+  </si>
+  <si>
+    <t>0000827-44.2026.5.08.0101</t>
+  </si>
+  <si>
+    <t>0010704-69.2026.5.15.0050</t>
+  </si>
+  <si>
+    <t>1001851-66.2025.5.02.0433</t>
+  </si>
+  <si>
+    <t>1002207-61.2025.5.02.0433</t>
+  </si>
+  <si>
+    <t>1001238-18.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>1001373-05.2026.5.02.0601</t>
+  </si>
+  <si>
+    <t>0011042-44.2026.5.15.0082</t>
+  </si>
+  <si>
+    <t>1001057-08.2026.5.02.0434</t>
+  </si>
+  <si>
+    <t>1000383-33.2026.5.02.0433</t>
+  </si>
+  <si>
+    <t>1000592-97.2025.5.02.0445</t>
+  </si>
+  <si>
+    <t>0001617-53.2025.5.09.0095</t>
+  </si>
+  <si>
+    <t>0001757-47.2025.5.09.0658</t>
+  </si>
+  <si>
+    <t>1000780-92.2026.5.02.0433</t>
+  </si>
+  <si>
+    <t>0010215-72.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>0010173-80.2026.5.15.0050</t>
+  </si>
+  <si>
+    <t>0010480-06.2026.5.15.0027</t>
+  </si>
+  <si>
+    <t>0010175-50.2026.5.15.0050</t>
+  </si>
+  <si>
+    <t>0010530-32.2026.5.15.0027</t>
+  </si>
+  <si>
+    <t>1019460-73.2020.8.26.0577</t>
+  </si>
+  <si>
+    <t>0010609-11.2026.5.15.0027</t>
+  </si>
+  <si>
+    <t>0010607-41.2026.5.15.0027</t>
+  </si>
+  <si>
+    <t>0010417-72.2026.5.15.0029</t>
+  </si>
+  <si>
+    <t>0010300-33.2026.5.15.0045</t>
+  </si>
+  <si>
+    <t>0012892-87.2025.5.15.0044</t>
+  </si>
+  <si>
+    <t>0010541-87.2019.5.15.0130</t>
+  </si>
+  <si>
+    <t>Michel Roque Martins Dias</t>
+  </si>
+  <si>
+    <t>Mistoncleso Cruz Da Silva</t>
+  </si>
+  <si>
+    <t>Marli Nogueira Da Silva</t>
+  </si>
+  <si>
+    <t>Adriano Jose Da Silva</t>
+  </si>
+  <si>
+    <t>Rildo Dos Santos Dias</t>
+  </si>
+  <si>
+    <t>Bruno Duque Vanderlei</t>
+  </si>
+  <si>
+    <t>Yago Henrique Almeida Luz</t>
+  </si>
+  <si>
+    <t>Giovani Gustavo Ferreira Da Silva</t>
+  </si>
+  <si>
+    <t>Reinaldo Monteiro</t>
+  </si>
+  <si>
+    <t>Carlos Alberto Arruda Croda</t>
+  </si>
+  <si>
+    <t>Renan De Azevedo Gomes</t>
+  </si>
+  <si>
+    <t>Elizeu Luiz Freire</t>
+  </si>
+  <si>
+    <t>Wesley Thiago Dos Santos Silva</t>
+  </si>
+  <si>
+    <t>Marisilda Henriques</t>
+  </si>
+  <si>
+    <t>Rafael Cordeiro Gripa</t>
+  </si>
+  <si>
+    <t>Arilson Moraes De Almeida</t>
+  </si>
+  <si>
+    <t>Flavio Luiz Cossa</t>
+  </si>
+  <si>
+    <t>Ronan Ramos Gregorio Almeida</t>
+  </si>
+  <si>
+    <t>Vinicius Andre Freitas Diniz</t>
+  </si>
+  <si>
+    <t>Ricardo Mauricio Contel</t>
+  </si>
+  <si>
+    <t>Valdir Pereira Leal</t>
+  </si>
+  <si>
+    <t>Thalia Francisca Ribeiro Da Silva E Silva</t>
+  </si>
+  <si>
+    <t>Daniel Dos Santos Barbosa</t>
+  </si>
+  <si>
+    <t>Tiago Vieira De Sousa</t>
+  </si>
+  <si>
+    <t>Damiao Euflausino Alves</t>
+  </si>
+  <si>
+    <t>Daniel Antonio</t>
+  </si>
+  <si>
+    <t>Matheus Alberto Silva</t>
+  </si>
+  <si>
+    <t>Marcos Lopes Da Silva</t>
+  </si>
+  <si>
+    <t>Gilson Trindade Gama</t>
+  </si>
+  <si>
+    <t>08:30:00</t>
+  </si>
+  <si>
+    <t>08:50:00</t>
   </si>
   <si>
     <t>09:00:00</t>
   </si>
   <si>
+    <t>09:15:00</t>
+  </si>
+  <si>
     <t>09:20:00</t>
   </si>
   <si>
-    <t>09:30:00</t>
-  </si>
-  <si>
-    <t>09:40:00</t>
-  </si>
-  <si>
-    <t>09:45:00</t>
+    <t>09:50:00</t>
   </si>
   <si>
     <t>10:00:00</t>
   </si>
   <si>
-    <t>10:13:00</t>
-  </si>
-  <si>
-    <t>11:00:00</t>
-  </si>
-  <si>
-    <t>11:10:00</t>
-  </si>
-  <si>
-    <t>11:15:00</t>
-  </si>
-  <si>
-    <t>12:00:00</t>
-  </si>
-  <si>
-    <t>13:30:00</t>
-  </si>
-  <si>
-    <t>13:35:00</t>
+    <t>10:10:00</t>
+  </si>
+  <si>
+    <t>10:30:00</t>
+  </si>
+  <si>
+    <t>11:20:00</t>
+  </si>
+  <si>
+    <t>11:50:00</t>
+  </si>
+  <si>
+    <t>13:00:00</t>
+  </si>
+  <si>
+    <t>13:27:00</t>
+  </si>
+  <si>
+    <t>13:34:00</t>
+  </si>
+  <si>
+    <t>13:42:00</t>
   </si>
   <si>
     <t>14:00:00</t>
   </si>
   <si>
-    <t>14:15:00</t>
+    <t>14:20:00</t>
   </si>
   <si>
     <t>14:30:00</t>
@@ -418,13 +415,13 @@
     <t>14:40:00</t>
   </si>
   <si>
-    <t>15:00:00</t>
-  </si>
-  <si>
-    <t>15:20:00</t>
-  </si>
-  <si>
-    <t>15:42:00</t>
+    <t>14:50:00</t>
+  </si>
+  <si>
+    <t>15:10:00</t>
+  </si>
+  <si>
+    <t>15:45:00</t>
   </si>
 </sst>
 </file>
@@ -800,7 +797,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -809,33 +806,33 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
@@ -844,33 +841,33 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
@@ -879,33 +876,33 @@
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
@@ -914,33 +911,33 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="K5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
@@ -949,25 +946,25 @@
         <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="H6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="K6" t="s">
         <v>117</v>
@@ -975,209 +972,209 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="G7" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J7" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="K7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="F8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J8" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="K8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G9" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E10" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F10" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G10" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="H10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J10" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E11" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F11" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="G11" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J11" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="K11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B12" t="s">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="E12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="H12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="K12" t="s">
         <v>122</v>
@@ -1185,34 +1182,34 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E13" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F13" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G13" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="H13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J13" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="K13" t="s">
         <v>123</v>
@@ -1220,19 +1217,19 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F14" t="s">
         <v>50</v>
@@ -1241,13 +1238,13 @@
         <v>50</v>
       </c>
       <c r="H14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J14" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="K14" t="s">
         <v>124</v>
@@ -1255,34 +1252,34 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B15" t="s">
         <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E15" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="F15" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G15" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J15" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="K15" t="s">
         <v>125</v>
@@ -1290,34 +1287,34 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B16" t="s">
         <v>11</v>
       </c>
       <c r="C16" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E16" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F16" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G16" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="H16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J16" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="K16" t="s">
         <v>126</v>
@@ -1325,34 +1322,34 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B17" t="s">
         <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D17" t="s">
         <v>31</v>
       </c>
       <c r="E17" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F17" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G17" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I17" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J17" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="K17" t="s">
         <v>127</v>
@@ -1360,34 +1357,34 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B18" t="s">
         <v>11</v>
       </c>
       <c r="C18" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E18" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="F18" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G18" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="H18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J18" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="K18" t="s">
         <v>128</v>
@@ -1395,69 +1392,69 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B19" t="s">
         <v>11</v>
       </c>
       <c r="C19" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D19" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E19" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F19" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G19" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J19" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="K19" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B20" t="s">
         <v>11</v>
       </c>
       <c r="C20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" t="s">
         <v>28</v>
       </c>
-      <c r="D20" t="s">
-        <v>31</v>
-      </c>
       <c r="E20" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="F20" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="G20" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="H20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J20" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="K20" t="s">
         <v>129</v>
@@ -1465,34 +1462,34 @@
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B21" t="s">
         <v>11</v>
       </c>
       <c r="C21" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D21" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E21" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J21" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="K21" t="s">
         <v>130</v>
@@ -1500,104 +1497,104 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B22" t="s">
         <v>11</v>
       </c>
       <c r="C22" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D22" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E22" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F22" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G22" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J22" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="K22" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B23" t="s">
         <v>11</v>
       </c>
       <c r="C23" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D23" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E23" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F23" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G23" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J23" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="K23" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B24" t="s">
         <v>11</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D24" t="s">
         <v>32</v>
       </c>
       <c r="E24" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F24" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G24" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="H24" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J24" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="K24" t="s">
         <v>131</v>
@@ -1605,34 +1602,34 @@
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B25" t="s">
         <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E25" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F25" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G25" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I25" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J25" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="K25" t="s">
         <v>132</v>
@@ -1640,104 +1637,104 @@
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B26" t="s">
         <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D26" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E26" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F26" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G26" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I26" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J26" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="K26" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B27" t="s">
         <v>11</v>
       </c>
       <c r="C27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D27" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E27" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F27" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G27" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="H27" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I27" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J27" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K27" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B28" t="s">
         <v>11</v>
       </c>
       <c r="C28" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D28" t="s">
         <v>32</v>
       </c>
       <c r="E28" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F28" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="G28" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="H28" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I28" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J28" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="K28" t="s">
         <v>134</v>
@@ -1745,72 +1742,72 @@
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B29" t="s">
         <v>11</v>
       </c>
       <c r="C29" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="D29" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E29" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="F29" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="G29" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H29" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I29" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J29" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="K29" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B30" t="s">
         <v>11</v>
       </c>
       <c r="C30" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D30" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E30" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F30" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="G30" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H30" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I30" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J30" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K30" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Audiências: sync 2026-07-30 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1948C94B-FE47-4E82-87E9-6CF121AB5BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{488BA91F-948D-437E-B5F4-98A236408E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5E957AC2-4C38-4A88-A791-11AA3C000AF5}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EDA056DD-E450-4C57-B6F0-B71371008E73}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="222">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,37 +95,145 @@
     <t>Link/Observações</t>
   </si>
   <si>
-    <t>Audiência de Conciliação - Semipresencial</t>
-  </si>
-  <si>
-    <t>0010685-63.2026.5.15.0050</t>
+    <t>Audiência Inicial -  Presencial</t>
+  </si>
+  <si>
+    <t>0011446-11.2026.5.15.0013</t>
+  </si>
+  <si>
+    <t>Embraer S.A.</t>
+  </si>
+  <si>
+    <t>Luciano Aparecido Pereira</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DOS CAMPOS</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>01ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Instrução</t>
+  </si>
+  <si>
+    <t>Reclamação Trabalhista</t>
+  </si>
+  <si>
+    <t>CENTRAL</t>
+  </si>
+  <si>
+    <t>R$                 3.190,34</t>
+  </si>
+  <si>
+    <t>Grupo B2</t>
+  </si>
+  <si>
+    <t>BCF</t>
+  </si>
+  <si>
+    <t>VCR</t>
+  </si>
+  <si>
+    <t>Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>1001605-70.2025.5.02.0433</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Everton Caldeira Marquesine</t>
+  </si>
+  <si>
+    <t>SANTO ANDRÉ</t>
+  </si>
+  <si>
+    <t>03ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             200.734,15</t>
+  </si>
+  <si>
+    <t>Grupo B1</t>
+  </si>
+  <si>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>TAM</t>
+  </si>
+  <si>
+    <t>0012525-60.2025.5.15.0045</t>
+  </si>
+  <si>
+    <t>Reinaldo Aparecido Dos Santos</t>
+  </si>
+  <si>
+    <t>02ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Inicial</t>
+  </si>
+  <si>
+    <t>R$             107.093,69</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Telepresencial</t>
+  </si>
+  <si>
+    <t>0000008-89.2026.5.09.0195</t>
+  </si>
+  <si>
+    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
+  </si>
+  <si>
+    <t>Everaldo Kovalchuk</t>
+  </si>
+  <si>
+    <t>CASCAVEL</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>R$               39.000,00</t>
+  </si>
+  <si>
+    <t>Grupo C</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>https://url.trt9.jus.br/szrfs ID da reunião: 896 7091 7043 Senha: 556658</t>
+  </si>
+  <si>
+    <t>0010718-53.2026.5.15.0050</t>
   </si>
   <si>
     <t>Viterra Bioenergia S.A.</t>
   </si>
   <si>
-    <t>Michel Roque Martins Dias</t>
+    <t>Marco Aurelio Claudio</t>
   </si>
   <si>
     <t>DRACENA</t>
   </si>
   <si>
-    <t>SP</t>
-  </si>
-  <si>
     <t>VARA DO TRABALHO</t>
   </si>
   <si>
     <t>Conhecimento</t>
   </si>
   <si>
-    <t>Reclamação Trabalhista</t>
-  </si>
-  <si>
-    <t>CENTRAL</t>
-  </si>
-  <si>
-    <t>R$             338.733,87</t>
+    <t>R$          1.025.120,00</t>
   </si>
   <si>
     <t>Grupo E2</t>
@@ -137,545 +245,473 @@
     <t>https://trt15-jus-br.zoom.us/j/87527564652?pwd=d3YrZ2diWXk5UjgzbmVkNExteWVMQT09 ID da reunião: 875 2756 4652 Senha de acesso: 246680</t>
   </si>
   <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>1000527-98.2026.5.02.0435</t>
-  </si>
-  <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Mistoncleso Cruz Da Silva</t>
-  </si>
-  <si>
-    <t>SANTO ANDRÉ</t>
-  </si>
-  <si>
-    <t>05ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Instrução</t>
-  </si>
-  <si>
-    <t>R$             183.783,60</t>
-  </si>
-  <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>Correspondente - Hebert</t>
-  </si>
-  <si>
-    <t>TAM</t>
-  </si>
-  <si>
-    <t>Presencial</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Presencial</t>
-  </si>
-  <si>
-    <t>1000832-57.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Companhia Brasileira De Cartuchos</t>
-  </si>
-  <si>
-    <t>Marli Nogueira Da Silva</t>
-  </si>
-  <si>
-    <t>RIBEIRÃO PIRES</t>
-  </si>
-  <si>
-    <t>R$             173.095,00</t>
-  </si>
-  <si>
-    <t>Grupo B3</t>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>0010598-92.2026.5.03.0066</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A</t>
+  </si>
+  <si>
+    <t>Marcos Paulo Da Silva</t>
+  </si>
+  <si>
+    <t>MANHUAÇU</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>R$               62.608,11</t>
+  </si>
+  <si>
+    <t>RRU</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/varamanhuacu</t>
+  </si>
+  <si>
+    <t>1000510-62.2026.5.02.0435</t>
+  </si>
+  <si>
+    <t>Cleiton Mendonca De Souza</t>
+  </si>
+  <si>
+    <t>R$             338.128,52</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>RFE</t>
+  </si>
+  <si>
+    <t>0010657-67.2026.5.15.0027</t>
+  </si>
+  <si>
+    <t>Guariroba Bioenergia Ltda. &amp; Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Fernando Henrique Grecco Dos Santos Garcia</t>
+  </si>
+  <si>
+    <t>VOTUPORANGA</t>
+  </si>
+  <si>
+    <t>R$             519.531,10</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>JNE</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/89939880446?pwd=ZHhwbjhhMUk2aGtDbmUwRTdELzhZUT09</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>0012012-63.2024.5.15.0066</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
+  </si>
+  <si>
+    <t>Edivane Dos Santos</t>
+  </si>
+  <si>
+    <t>RIBEIRÃO PRETO</t>
+  </si>
+  <si>
+    <t>CEJUSC</t>
+  </si>
+  <si>
+    <t>Execução</t>
+  </si>
+  <si>
+    <t>R$               81.480,00</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>JPL</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/7093890373?pwd=eEJTaWhnbTRwVXJrVTR0R0RyMUhkdz09 Id da reunião: 7093890373 Senha da sala: 345356</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>1000584-28.2026.5.02.0432</t>
+  </si>
+  <si>
+    <t>Welington Tavian Baptista</t>
+  </si>
+  <si>
+    <t>R$             939.102,40</t>
+  </si>
+  <si>
+    <t>GSM</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Semipresencial</t>
+  </si>
+  <si>
+    <t>0024058-02.2026.5.24.0022</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Monteverde</t>
+  </si>
+  <si>
+    <t>Taiane Lima Da Silva</t>
+  </si>
+  <si>
+    <t>DOURADOS</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>R$               92.200,00</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>https://trt24-jus-br.zoom.us/my/trt24douvt2sala2</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>0011078-07.2025.5.03.0066</t>
+  </si>
+  <si>
+    <t>Walleska Souza Menezes</t>
+  </si>
+  <si>
+    <t>VARA DO TRBALHO</t>
+  </si>
+  <si>
+    <t>R$               88.187,38</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Semipresencial</t>
+  </si>
+  <si>
+    <t>0011770-60.2025.5.15.0037</t>
+  </si>
+  <si>
+    <t>Ouroeste Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Isabela Carolina Bento Belini Vilela</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DO RIO PRETO</t>
+  </si>
+  <si>
+    <t>06ª TURMA</t>
+  </si>
+  <si>
+    <t>Recursal</t>
+  </si>
+  <si>
+    <t>R$             287.798,68</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/81390598525?pwd=rdGf0eRPC3KeSMHZlUecdE1edZpE5R.1 ID da reunião: 813 9059 8525 Senha: 127812</t>
+  </si>
+  <si>
+    <t>0012741-24.2025.5.15.0044</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Gilberlandio Cascimiro Barbosa</t>
+  </si>
+  <si>
+    <t>R$             236.985,97</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/85763756385?pwd=ZTBCT3ZkZVg1QUVqMFVBNFcxUDdmQT0  ID: 857 6375 6385 e Senha de acesso: 958777</t>
+  </si>
+  <si>
+    <t>0001208-68.2025.5.09.0195</t>
+  </si>
+  <si>
+    <t>Syngenta Seeds Ltda.</t>
+  </si>
+  <si>
+    <t>Cerli Coelho Gomes</t>
+  </si>
+  <si>
+    <t>1ª Instância</t>
+  </si>
+  <si>
+    <t>R$               58.494,52</t>
+  </si>
+  <si>
+    <t>TLI</t>
+  </si>
+  <si>
+    <t>https://url.trt9.jus.br/lauqj ID da reunião: 89116526039 Senha de acesso: AdbrJfUkLV</t>
+  </si>
+  <si>
+    <t>Perícia Técnica</t>
+  </si>
+  <si>
+    <t>1000639-09.2026.5.02.0034</t>
+  </si>
+  <si>
+    <t>Colégio Curumim S/S Ltda</t>
+  </si>
+  <si>
+    <t>Andre Luiz Da Silva Rocumback</t>
+  </si>
+  <si>
+    <t>SÃO PAULO</t>
+  </si>
+  <si>
+    <t>34ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               48.019,81</t>
+  </si>
+  <si>
+    <t>JRM</t>
+  </si>
+  <si>
+    <t>ALF</t>
+  </si>
+  <si>
+    <t>Iremos acompanhar</t>
+  </si>
+  <si>
+    <t>1002378-21.2025.5.02.0432</t>
+  </si>
+  <si>
+    <t>Marcilio Alan Ferreira Cavalcanti</t>
+  </si>
+  <si>
+    <t>R$             646.662,33</t>
   </si>
   <si>
     <t>LMI</t>
   </si>
   <si>
-    <t>1000628-78.2025.5.02.0433</t>
-  </si>
-  <si>
-    <t>Adriano Jose Da Silva</t>
-  </si>
-  <si>
-    <t>03ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$          2.518.007,92</t>
-  </si>
-  <si>
-    <t>ANB</t>
-  </si>
-  <si>
     <t>BSO</t>
   </si>
   <si>
-    <t>Audiência Una - Telepresencial</t>
-  </si>
-  <si>
-    <t>0000827-44.2026.5.08.0101</t>
-  </si>
-  <si>
-    <t>Fertilizantes Tocantins S.A</t>
-  </si>
-  <si>
-    <t>Rildo Dos Santos Dias</t>
-  </si>
-  <si>
-    <t>ABAETETUBA</t>
-  </si>
-  <si>
-    <t>PA</t>
-  </si>
-  <si>
-    <t>01ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             840.804,54</t>
-  </si>
-  <si>
-    <t>ARC</t>
-  </si>
-  <si>
-    <t>https://trt8-jus-br.zoom.us/j/85053969243?pwd=RVArVU1FbVNNeFhZMVdxd2x0dEpkdz09 ID: 850  5396  9243 Senha: 1VTAbaete.</t>
-  </si>
-  <si>
-    <t>0010704-69.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>Bruno Duque Vanderlei</t>
-  </si>
-  <si>
-    <t>R$             107.564,68</t>
+    <t>1001149-46.2026.5.02.0511</t>
+  </si>
+  <si>
+    <t>Ame Digital Brasil Ltda</t>
+  </si>
+  <si>
+    <t>Daiana Arruda Santos Silva</t>
+  </si>
+  <si>
+    <t>ITAPEVI</t>
+  </si>
+  <si>
+    <t>R$             159.297,56</t>
+  </si>
+  <si>
+    <t>Grupo D1</t>
+  </si>
+  <si>
+    <t>Correspondente - Carlos Florian</t>
+  </si>
+  <si>
+    <t>BBO</t>
+  </si>
+  <si>
+    <t>Presencial | Advogado - Dr. Jairo Felipe, (11) 98807-2750</t>
+  </si>
+  <si>
+    <t>0010921-49.2025.5.15.0050</t>
+  </si>
+  <si>
+    <t>Joao Maria Bonifacio Ribeiro</t>
+  </si>
+  <si>
+    <t>Liquidação</t>
+  </si>
+  <si>
+    <t>R$               35.645,00</t>
   </si>
   <si>
     <t>FCG</t>
   </si>
   <si>
-    <t>1001851-66.2025.5.02.0433</t>
-  </si>
-  <si>
-    <t>Yago Henrique Almeida Luz</t>
-  </si>
-  <si>
-    <t>R$             107.301,15</t>
-  </si>
-  <si>
-    <t>RFE</t>
-  </si>
-  <si>
-    <t>1002207-61.2025.5.02.0433</t>
-  </si>
-  <si>
-    <t>Giovani Gustavo Ferreira Da Silva</t>
-  </si>
-  <si>
-    <t>R$             432.485,73</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>1001238-18.2026.5.02.0431</t>
-  </si>
-  <si>
-    <t>Reinaldo Monteiro</t>
-  </si>
-  <si>
-    <t>R$             291.960,14</t>
-  </si>
-  <si>
-    <t>GSM</t>
-  </si>
-  <si>
-    <t>1001373-05.2026.5.02.0601</t>
-  </si>
-  <si>
-    <t>Panificadora Cepam Ltda.</t>
-  </si>
-  <si>
-    <t>Carlos Alberto Arruda Croda</t>
-  </si>
-  <si>
-    <t>SÃO PAULO</t>
-  </si>
-  <si>
-    <t>25ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>ZONA LESTE</t>
-  </si>
-  <si>
-    <t>R$                 8.626,39</t>
-  </si>
-  <si>
-    <t>RYL</t>
+    <t>https://trt15-jus-br.zoom.us/j/86722354209?pwd=V01VL0NmTFZSZEdhcFhjM0tIczd3dz09 ID da reunião: 867 2235 4209 Senha de acesso: 947812</t>
+  </si>
+  <si>
+    <t>1001275-39.2026.5.02.0433</t>
+  </si>
+  <si>
+    <t>Danilo Oliveira De Lima</t>
+  </si>
+  <si>
+    <t>R$               66.734,63</t>
+  </si>
+  <si>
+    <t>0011437-35.2025.5.15.0126</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A. - Paulinia - Pln</t>
+  </si>
+  <si>
+    <t>Jose Maria Pereira</t>
+  </si>
+  <si>
+    <t>PAULÍNIA</t>
+  </si>
+  <si>
+    <t>R$               70.308,57</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/83352065501?pwd=Lzc2WUJGSVpVWmJyZjB3Y0NvUmJPZz09 ID da reunião: 83352065501 Senha de acesso: 368465</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Presencial</t>
+  </si>
+  <si>
+    <t>0024683-80.2026.5.24.0072</t>
+  </si>
+  <si>
+    <t>Rio Parana Energia S.A</t>
+  </si>
+  <si>
+    <t>Flavio Rodrigues Valente</t>
+  </si>
+  <si>
+    <t>TRÊS LAGOAS</t>
+  </si>
+  <si>
+    <t>R$             170.573,34</t>
+  </si>
+  <si>
+    <t>ECO</t>
+  </si>
+  <si>
+    <t>https://trt24-jus-br.zoom.us/j/2274633182</t>
+  </si>
+  <si>
+    <t>1000607-04.2022.5.02.0435</t>
+  </si>
+  <si>
+    <t>Marcelo Silva Rodrigues</t>
+  </si>
+  <si>
+    <t>CEJUSC ABC</t>
+  </si>
+  <si>
+    <t>R$             336.223,96</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/82477928530?pwd=WENUNkRGZ1NLbUY4VFZLdjdjOXBxUT09 ID da reunião: 824 7792 8530 Senha de acesso: 391604</t>
+  </si>
+  <si>
+    <t>0011841-62.2025.5.15.0134</t>
+  </si>
+  <si>
+    <t>Tiago Viegas Carvalho</t>
+  </si>
+  <si>
+    <t>LEME</t>
+  </si>
+  <si>
+    <t>R$          1.203.488,64</t>
+  </si>
+  <si>
+    <t>DPR</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/8060729658?pwd=NDNlcU8wVzcxZ09qVjFDRFBGT2ljQT09 ID da reunião: 806 072 9658 Senha de acesso: 868717</t>
+  </si>
+  <si>
+    <t>1001826-18.2023.5.02.0435</t>
+  </si>
+  <si>
+    <t>Rodrigo Fernandes Da Silva</t>
+  </si>
+  <si>
+    <t>R$             204.334,53</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/88297719933?pwd=U3VWVjB2RHh0Vm9VMHZ0ZFd1eUk1dz09 ID da reunião: 882 9771 9933 Senha de acesso: 091850</t>
+  </si>
+  <si>
+    <t>1000899-59.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>Carlos Alberto De Castro</t>
+  </si>
+  <si>
+    <t>Cumprimento de Sentença</t>
+  </si>
+  <si>
+    <t>R$               86.225,68</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/88959116257?pwd=Q09WTmd6SnZibUUrZWxMSFdiRm9tUT09 ID da reunião: 889 5911 6257 Senha de acesso: 136898</t>
+  </si>
+  <si>
+    <t>1001342-80.2021.5.02.0432</t>
+  </si>
+  <si>
+    <t>Natanael Marques Vieira</t>
+  </si>
+  <si>
+    <t>Recurso Parcial de Mérito</t>
+  </si>
+  <si>
+    <t>R$             137.042,10</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/85239557292?pwd=enBMVGxIVlR2bG5uUmk3Sy8yWmR6dz09 ID da reunião: 852 3955 7292 Senha de acesso: 611035</t>
+  </si>
+  <si>
+    <t>1001636-94.2024.5.02.0055</t>
+  </si>
+  <si>
+    <t>Construtora Elias Victor Nigri Ltda.</t>
+  </si>
+  <si>
+    <t>Derivaldo Dos Santos Silva</t>
+  </si>
+  <si>
+    <t>CEJUSC RUY BARBOSA</t>
+  </si>
+  <si>
+    <t>R$             544.507,98</t>
   </si>
   <si>
     <t>CAL</t>
   </si>
   <si>
-    <t>Audiência Inicial -  Telepresencial</t>
-  </si>
-  <si>
-    <t>0011042-44.2026.5.15.0082</t>
-  </si>
-  <si>
-    <t>Moema Bioenergia S.A. - Moema</t>
-  </si>
-  <si>
-    <t>Renan De Azevedo Gomes</t>
-  </si>
-  <si>
-    <t>SÃO JOSÉ DO RIO PRETO</t>
-  </si>
-  <si>
-    <t>R$             200.000,00</t>
-  </si>
-  <si>
-    <t>JNE</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/87100825693?pwd=Ulpt0u9ZPHbqliJGGGKn8D17RPJwW2.1 ID da reunião: 871 0082 5693 Senha: 864984</t>
-  </si>
-  <si>
-    <t>1001057-08.2026.5.02.0434</t>
-  </si>
-  <si>
-    <t>Elizeu Luiz Freire</t>
-  </si>
-  <si>
-    <t>04ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             158.737,00</t>
-  </si>
-  <si>
-    <t>Audiência Inicial - Presencial</t>
-  </si>
-  <si>
-    <t>1000383-33.2026.5.02.0433</t>
-  </si>
-  <si>
-    <t>Wesley Thiago Dos Santos Silva</t>
-  </si>
-  <si>
-    <t>Ação de Consignação em Pagamento</t>
-  </si>
-  <si>
-    <t>R$                 8.821,89</t>
-  </si>
-  <si>
-    <t>JPE</t>
-  </si>
-  <si>
-    <t>Sessão de Julgamento TRT - Presencial</t>
-  </si>
-  <si>
-    <t>1000592-97.2025.5.02.0445</t>
-  </si>
-  <si>
-    <t>Telefonica Brasil S.A.</t>
-  </si>
-  <si>
-    <t>Marisilda Henriques</t>
-  </si>
-  <si>
-    <t>SANTOS</t>
-  </si>
-  <si>
-    <t>06ª TURMA</t>
-  </si>
-  <si>
-    <t>Recursal</t>
-  </si>
-  <si>
-    <t>R$          2.433.235,00</t>
-  </si>
-  <si>
-    <t>Grupo C</t>
-  </si>
-  <si>
-    <t>TFR</t>
-  </si>
-  <si>
-    <t>RCF</t>
-  </si>
-  <si>
-    <t>Audiência Inicial - Telepresencial</t>
-  </si>
-  <si>
-    <t>0001617-53.2025.5.09.0095</t>
-  </si>
-  <si>
-    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
-  </si>
-  <si>
-    <t>Rafael Cordeiro Gripa</t>
-  </si>
-  <si>
-    <t>FOZ DO IGUAÇU</t>
-  </si>
-  <si>
-    <t>PR</t>
-  </si>
-  <si>
-    <t>Inicial</t>
-  </si>
-  <si>
-    <t>R$             326.167,00</t>
-  </si>
-  <si>
-    <t>VSI</t>
-  </si>
-  <si>
-    <t>https://url.trt9.jus.br/hpqcg ID da Reunião: 84656312612 Senha: ws3xteM7dN</t>
-  </si>
-  <si>
-    <t>0001757-47.2025.5.09.0658</t>
-  </si>
-  <si>
-    <t>Arilson Moraes De Almeida</t>
-  </si>
-  <si>
-    <t>R$             188.600,00</t>
-  </si>
-  <si>
-    <t>https://url.trt9.jus.br/j7hoq ID da Reunião: 85022178469 Senha: MnoK8bxzgu</t>
-  </si>
-  <si>
-    <t>Audiência de Conciliação - Telepresencial</t>
-  </si>
-  <si>
-    <t>1000780-92.2026.5.02.0433</t>
-  </si>
-  <si>
-    <t>Flavio Luiz Cossa</t>
-  </si>
-  <si>
-    <t>CEJUSC ABC</t>
-  </si>
-  <si>
-    <t>Recursal com Execução Provisória</t>
-  </si>
-  <si>
-    <t>Cumprimento de Sentença</t>
-  </si>
-  <si>
-    <t>R$             565.498,97</t>
-  </si>
-  <si>
-    <t>https://trt2-jus-br.zoom.us/j/81881873237?pwd=aEs5S29DM2srNHRuRGFVM2ZEYkVUZz09 ID da reunião: 818 8187 3237 Senha de acesso: 459217</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Telepresencial</t>
-  </si>
-  <si>
-    <t>0010215-72.2026.5.03.0080</t>
-  </si>
-  <si>
-    <t>Salitre Fertilizantes Ltda.</t>
-  </si>
-  <si>
-    <t>Ronan Ramos Gregorio Almeida</t>
-  </si>
-  <si>
-    <t>PATROCÍNIO</t>
-  </si>
-  <si>
-    <t>MG</t>
-  </si>
-  <si>
-    <t>R$             112.417,99</t>
-  </si>
-  <si>
-    <t>MBF</t>
-  </si>
-  <si>
-    <t>https://trt3-jus-br.zoom.us/my/vt.patrocinio</t>
-  </si>
-  <si>
-    <t>0010173-80.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>Vinicius Andre Freitas Diniz</t>
-  </si>
-  <si>
-    <t>R$             182.474,98</t>
-  </si>
-  <si>
-    <t>https://trt15-jus.br.zoom.us/j/87527564652?pwd=d3YrZ2diWXk5UjgzbmVkNExteWVMQT09 ID da reunião: 875 2756 4652 Senha de acesso: 246680</t>
-  </si>
-  <si>
-    <t>0010480-06.2026.5.15.0027</t>
-  </si>
-  <si>
-    <t>Guariroba Bioenergia Ltda.</t>
-  </si>
-  <si>
-    <t>Ricardo Mauricio Contel</t>
-  </si>
-  <si>
-    <t>VOTUPORANGA</t>
-  </si>
-  <si>
-    <t>R$             300.000,00</t>
-  </si>
-  <si>
-    <t>https://us02web.zoom.us/j/82212757993?pwd=aSt4Q29rc0JRMnFXSTU0UzdCVVZyQT09</t>
-  </si>
-  <si>
-    <t>0010175-50.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>Valdir Pereira Leal</t>
-  </si>
-  <si>
-    <t>R$             115.000,00</t>
-  </si>
-  <si>
-    <t>RRU</t>
-  </si>
-  <si>
-    <t>0010530-32.2026.5.15.0027</t>
-  </si>
-  <si>
-    <t>Thalia Francisca Ribeiro Da Silva E Silva</t>
-  </si>
-  <si>
-    <t>R$               74.592,48</t>
-  </si>
-  <si>
-    <t>Perícia Técnica</t>
-  </si>
-  <si>
-    <t>1019460-73.2020.8.26.0577</t>
-  </si>
-  <si>
-    <t>Embraer S.A.</t>
-  </si>
-  <si>
-    <t>Daniel Dos Santos Barbosa</t>
-  </si>
-  <si>
-    <t>SAO JOSE DOS CAMPOS</t>
-  </si>
-  <si>
-    <t>08ª VARA CÍVEL</t>
-  </si>
-  <si>
-    <t>Pedido de Benefício - INSS</t>
-  </si>
-  <si>
-    <t>R$               12.540,00</t>
-  </si>
-  <si>
-    <t>Grupo B2</t>
-  </si>
-  <si>
-    <t>VCR</t>
-  </si>
-  <si>
-    <t>NRG</t>
-  </si>
-  <si>
-    <t>Iremos acompanhar</t>
-  </si>
-  <si>
-    <t>0010609-11.2026.5.15.0027</t>
-  </si>
-  <si>
-    <t>Tiago Vieira De Sousa</t>
-  </si>
-  <si>
-    <t>R$             216.000,00</t>
-  </si>
-  <si>
-    <t>0010607-41.2026.5.15.0027</t>
-  </si>
-  <si>
-    <t>Damiao Euflausino Alves</t>
-  </si>
-  <si>
-    <t>R$             187.000,00</t>
-  </si>
-  <si>
-    <t>0010417-72.2026.5.15.0029</t>
-  </si>
-  <si>
-    <t>Daniel Antonio</t>
-  </si>
-  <si>
-    <t>JABOTICABAL</t>
-  </si>
-  <si>
-    <t>R$          1.318.000,00</t>
-  </si>
-  <si>
-    <t>https://zoom.us/j/3072626738 ID da reunião: 3072626738 Senha: 159753</t>
-  </si>
-  <si>
-    <t>0010300-33.2026.5.15.0045</t>
-  </si>
-  <si>
-    <t>Matheus Alberto Silva</t>
-  </si>
-  <si>
-    <t>SÃO JOSÉ DOS CAMPOS</t>
-  </si>
-  <si>
-    <t>R$               96.000,00</t>
-  </si>
-  <si>
-    <t>BCF</t>
-  </si>
-  <si>
-    <t>0012892-87.2025.5.15.0044</t>
-  </si>
-  <si>
-    <t>Marcos Lopes Da Silva</t>
-  </si>
-  <si>
-    <t>02ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             127.204,51</t>
-  </si>
-  <si>
-    <t>https://us02web.zoom.us/j/83908187251?pwd=Ty9tcHNFb0pLZk5WQ0l2Y0V3ZHhhdz09 ID da reunião: 839 0818 7251 e Senha de acesso: 959576</t>
-  </si>
-  <si>
-    <t>0010541-87.2019.5.15.0130</t>
-  </si>
-  <si>
-    <t>Gilson Trindade Gama</t>
-  </si>
-  <si>
-    <t>CAMPINAS</t>
-  </si>
-  <si>
-    <t>CEJUSC</t>
-  </si>
-  <si>
-    <t>Execução</t>
-  </si>
-  <si>
-    <t>R$             326.430,00</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/86385704640?pwd=g1Ig2NoEnHBDvn3uZhXt1tmbVhuO14.1</t>
+    <t>https://trt2-jus-br.zoom.us/j/81872601242?pwd=dmxJTVdoVjBmRGMzSUFKRVoyN0Jndz09</t>
+  </si>
+  <si>
+    <t>L. Sant'Angelo Pinturas Ltda.</t>
+  </si>
+  <si>
+    <t>R$             544.507,98</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -695,14 +731,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -759,14 +787,16 @@
     </border>
     <border>
       <left style="medium">
-        <color indexed="64"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="medium">
-        <color indexed="64"/>
+        <color rgb="FFBFBFBF"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color rgb="FFBFBFBF"/>
+      </top>
       <bottom style="medium">
-        <color indexed="64"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
       <diagonal/>
     </border>
@@ -775,18 +805,19 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -809,12 +840,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1146,29 +1173,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14B93C17-7185-46B4-8EC7-C49F3AE7F90C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B72B31BF-DC39-4A6F-99E4-E27F8E96566B}">
   <dimension ref="A1:R30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="47.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="26.21875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="52.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.77734375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="121" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="111.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1224,15 +1252,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>105072</v>
+        <v>104834</v>
       </c>
       <c r="B2" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C2" s="6">
-        <v>0.35416666666666669</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>18</v>
@@ -1274,45 +1302,45 @@
         <v>30</v>
       </c>
       <c r="Q2" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="R2" s="8" t="s">
         <v>31</v>
       </c>
+      <c r="R2" s="7" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="3" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
-        <v>104495</v>
+        <v>102040</v>
       </c>
       <c r="B3" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C3" s="6">
-        <v>0.35416666666666669</v>
+        <v>0.34722222222222221</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I3" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L3" s="7" t="s">
         <v>26</v>
@@ -1332,43 +1360,43 @@
       <c r="Q3" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="R3" s="8" t="s">
+      <c r="R3" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>103645</v>
+      </c>
+      <c r="B4" s="5">
+        <v>46233</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0.34722222222222221</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="4">
-        <v>105206</v>
-      </c>
-      <c r="B4" s="5">
-        <v>46232</v>
-      </c>
-      <c r="C4" s="6">
-        <v>0.36805555555555558</v>
-      </c>
-      <c r="D4" s="7" t="s">
+      <c r="F4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>47</v>
-      </c>
       <c r="H4" s="7" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="L4" s="7" t="s">
         <v>26</v>
@@ -1377,54 +1405,54 @@
         <v>27</v>
       </c>
       <c r="N4" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q4" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="R4" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>103745</v>
+      </c>
+      <c r="B5" s="5">
+        <v>46233</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="Q4" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="R4" s="8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
-        <v>100523</v>
-      </c>
-      <c r="B5" s="5">
-        <v>46232</v>
-      </c>
-      <c r="C5" s="6">
-        <v>0.375</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>23</v>
-      </c>
       <c r="J5" s="7" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L5" s="7" t="s">
         <v>26</v>
@@ -1433,54 +1461,54 @@
         <v>27</v>
       </c>
       <c r="N5" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="O5" s="7" t="s">
         <v>55</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>40</v>
       </c>
       <c r="P5" s="7" t="s">
         <v>56</v>
       </c>
       <c r="Q5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="R5" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="R5" s="8" t="s">
-        <v>43</v>
-      </c>
     </row>
-    <row r="6" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
-        <v>105065</v>
+        <v>105148</v>
       </c>
       <c r="B6" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C6" s="6">
-        <v>0.38541666666666669</v>
+        <v>0.375</v>
       </c>
       <c r="D6" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="I6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="K6" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>26</v>
@@ -1489,10 +1517,10 @@
         <v>27</v>
       </c>
       <c r="N6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="O6" s="7" t="s">
         <v>65</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>29</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>66</v>
@@ -1500,40 +1528,40 @@
       <c r="Q6" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="R6" s="8" t="s">
+      <c r="R6" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
-        <v>105105</v>
+        <v>105566</v>
       </c>
       <c r="B7" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C7" s="6">
-        <v>0.38541666666666669</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>23</v>
+        <v>73</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>25</v>
@@ -1545,54 +1573,54 @@
         <v>27</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="O7" s="7" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="Q7" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="R7" s="8" t="s">
-        <v>31</v>
+        <v>75</v>
+      </c>
+      <c r="R7" s="7" t="s">
+        <v>76</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
-        <v>102846</v>
+        <v>104499</v>
       </c>
       <c r="B8" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C8" s="6">
-        <v>0.3888888888888889</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I8" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>26</v>
@@ -1601,54 +1629,54 @@
         <v>27</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="O8" s="7" t="s">
         <v>40</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="Q8" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="R8" s="8" t="s">
-        <v>43</v>
+        <v>81</v>
+      </c>
+      <c r="R8" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
-        <v>103333</v>
+        <v>105115</v>
       </c>
       <c r="B9" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C9" s="6">
-        <v>0.40972222222222221</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>26</v>
@@ -1657,54 +1685,54 @@
         <v>27</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="Q9" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="R9" s="8" t="s">
-        <v>43</v>
+        <v>88</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>89</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
-        <v>105455</v>
+        <v>99079</v>
       </c>
       <c r="B10" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C10" s="6">
-        <v>0.41666666666666669</v>
+        <v>0.42569444444444443</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>34</v>
+        <v>92</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>36</v>
+        <v>94</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>64</v>
+        <v>95</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>38</v>
+        <v>96</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>26</v>
@@ -1713,110 +1741,110 @@
         <v>27</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="O10" s="7" t="s">
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>41</v>
+        <v>99</v>
       </c>
       <c r="Q10" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="R10" s="8" t="s">
-        <v>43</v>
+        <v>99</v>
+      </c>
+      <c r="R10" s="7" t="s">
+        <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
-        <v>105327</v>
+        <v>104578</v>
       </c>
       <c r="B11" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C11" s="6">
-        <v>0.4236111111111111</v>
+        <v>0.43055555555555558</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>85</v>
+        <v>35</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>87</v>
+        <v>37</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>88</v>
+        <v>45</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L11" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="O11" s="7" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="P11" s="7" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="Q11" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="R11" s="8" t="s">
-        <v>43</v>
+        <v>105</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
-        <v>104889</v>
+        <v>104380</v>
       </c>
       <c r="B12" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C12" s="6">
-        <v>0.4375</v>
+        <v>0.43055555555555558</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>23</v>
+        <v>111</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L12" s="7" t="s">
         <v>26</v>
@@ -1825,54 +1853,54 @@
         <v>27</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="O12" s="7" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="P12" s="7" t="s">
-        <v>71</v>
+        <v>113</v>
       </c>
       <c r="Q12" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="R12" s="8" t="s">
-        <v>100</v>
+        <v>113</v>
+      </c>
+      <c r="R12" s="7" t="s">
+        <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
-        <v>105230</v>
+        <v>105286</v>
       </c>
       <c r="B13" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C13" s="6">
-        <v>0.47222222222222221</v>
+        <v>0.43055555555555558</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>44</v>
+        <v>115</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>23</v>
+        <v>73</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="L13" s="7" t="s">
         <v>26</v>
@@ -1881,110 +1909,110 @@
         <v>27</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="P13" s="7" t="s">
-        <v>41</v>
+        <v>75</v>
       </c>
       <c r="Q13" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="R13" s="8" t="s">
-        <v>43</v>
+        <v>75</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
-        <v>104323</v>
+        <v>103401</v>
       </c>
       <c r="B14" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C14" s="6">
-        <v>0.49305555555555558</v>
+        <v>0.4375</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>34</v>
+        <v>122</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="I14" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>54</v>
+        <v>125</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>38</v>
+        <v>126</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>108</v>
+        <v>26</v>
       </c>
       <c r="M14" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N14" s="7" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="O14" s="7" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="P14" s="7" t="s">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="Q14" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="R14" s="8" t="s">
-        <v>43</v>
+        <v>87</v>
+      </c>
+      <c r="R14" s="7" t="s">
+        <v>128</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
-        <v>104171</v>
+        <v>103407</v>
       </c>
       <c r="B15" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C15" s="6">
-        <v>0.54166666666666663</v>
+        <v>0.44444444444444442</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>116</v>
+        <v>45</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>117</v>
+        <v>25</v>
       </c>
       <c r="L15" s="7" t="s">
         <v>26</v>
@@ -1993,54 +2021,54 @@
         <v>27</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="O15" s="7" t="s">
-        <v>119</v>
+        <v>65</v>
       </c>
       <c r="P15" s="7" t="s">
-        <v>120</v>
+        <v>87</v>
       </c>
       <c r="Q15" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="R15" s="8" t="s">
-        <v>43</v>
+        <v>87</v>
+      </c>
+      <c r="R15" s="7" t="s">
+        <v>133</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
-        <v>103594</v>
+        <v>102142</v>
       </c>
       <c r="B16" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C16" s="6">
-        <v>0.56041666666666667</v>
+        <v>0.46527777777777779</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>122</v>
+        <v>90</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>126</v>
+        <v>52</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>127</v>
+        <v>53</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>64</v>
+        <v>95</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="L16" s="7" t="s">
         <v>26</v>
@@ -2049,54 +2077,54 @@
         <v>27</v>
       </c>
       <c r="N16" s="7" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="O16" s="7" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="P16" s="7" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="Q16" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="R16" s="8" t="s">
-        <v>131</v>
+        <v>99</v>
+      </c>
+      <c r="R16" s="7" t="s">
+        <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
-        <v>103590</v>
+        <v>105113</v>
       </c>
       <c r="B17" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C17" s="6">
-        <v>0.56527777777777777</v>
+        <v>0.46527777777777779</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>127</v>
+        <v>23</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>64</v>
+        <v>146</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="L17" s="7" t="s">
         <v>26</v>
@@ -2105,110 +2133,110 @@
         <v>27</v>
       </c>
       <c r="N17" s="7" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="O17" s="7" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="P17" s="7" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="Q17" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="R17" s="8" t="s">
-        <v>135</v>
+        <v>149</v>
+      </c>
+      <c r="R17" s="7" t="s">
+        <v>150</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
-        <v>104817</v>
+        <v>103621</v>
       </c>
       <c r="B18" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C18" s="6">
-        <v>0.5708333333333333</v>
+        <v>0.47569444444444442</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>136</v>
+        <v>33</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>139</v>
+        <v>45</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>140</v>
+        <v>25</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>141</v>
+        <v>26</v>
       </c>
       <c r="M18" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N18" s="7" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="O18" s="7" t="s">
         <v>40</v>
       </c>
       <c r="P18" s="7" t="s">
-        <v>110</v>
+        <v>154</v>
       </c>
       <c r="Q18" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="R18" s="8" t="s">
-        <v>143</v>
+        <v>155</v>
+      </c>
+      <c r="R18" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
-        <v>104360</v>
+        <v>104939</v>
       </c>
       <c r="B19" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C19" s="6">
-        <v>0.58333333333333337</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>144</v>
+        <v>101</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>149</v>
+        <v>23</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L19" s="7" t="s">
         <v>26</v>
@@ -2217,54 +2245,54 @@
         <v>27</v>
       </c>
       <c r="N19" s="7" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>29</v>
+        <v>161</v>
       </c>
       <c r="P19" s="7" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="Q19" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="R19" s="8" t="s">
-        <v>152</v>
+        <v>163</v>
+      </c>
+      <c r="R19" s="7" t="s">
+        <v>164</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
-        <v>104030</v>
+        <v>101864</v>
       </c>
       <c r="B20" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C20" s="6">
-        <v>0.58333333333333337</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>144</v>
+        <v>90</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="I20" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>24</v>
+        <v>95</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>38</v>
+        <v>167</v>
       </c>
       <c r="L20" s="7" t="s">
         <v>26</v>
@@ -2273,54 +2301,54 @@
         <v>27</v>
       </c>
       <c r="N20" s="7" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="O20" s="7" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="P20" s="7" t="s">
-        <v>30</v>
+        <v>169</v>
       </c>
       <c r="Q20" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="R20" s="8" t="s">
-        <v>156</v>
+        <v>169</v>
+      </c>
+      <c r="R20" s="7" t="s">
+        <v>170</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="4">
-        <v>105013</v>
+        <v>105465</v>
       </c>
       <c r="B21" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C21" s="6">
-        <v>0.59722222222222221</v>
+        <v>0.4861111111111111</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>93</v>
+        <v>18</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>158</v>
+        <v>35</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>160</v>
+        <v>37</v>
       </c>
       <c r="I21" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L21" s="7" t="s">
         <v>26</v>
@@ -2329,54 +2357,54 @@
         <v>27</v>
       </c>
       <c r="N21" s="7" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="O21" s="7" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="P21" s="7" t="s">
-        <v>92</v>
+        <v>41</v>
       </c>
       <c r="Q21" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="R21" s="8" t="s">
-        <v>162</v>
+        <v>81</v>
+      </c>
+      <c r="R21" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
-        <v>104029</v>
+        <v>102592</v>
       </c>
       <c r="B22" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C22" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.55208333333333337</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>144</v>
+        <v>115</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>20</v>
+        <v>175</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>22</v>
+        <v>177</v>
       </c>
       <c r="I22" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L22" s="7" t="s">
         <v>26</v>
@@ -2385,54 +2413,54 @@
         <v>27</v>
       </c>
       <c r="N22" s="7" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="O22" s="7" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="P22" s="7" t="s">
-        <v>166</v>
+        <v>113</v>
       </c>
       <c r="Q22" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="R22" s="8" t="s">
-        <v>156</v>
+        <v>75</v>
+      </c>
+      <c r="R22" s="7" t="s">
+        <v>179</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
-        <v>105006</v>
+        <v>104799</v>
       </c>
       <c r="B23" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C23" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.57222222222222219</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>93</v>
+        <v>180</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>158</v>
+        <v>182</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>160</v>
+        <v>184</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>23</v>
+        <v>111</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L23" s="7" t="s">
         <v>26</v>
@@ -2441,110 +2469,110 @@
         <v>27</v>
       </c>
       <c r="N23" s="7" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="O23" s="7" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="P23" s="7" t="s">
-        <v>92</v>
+        <v>186</v>
       </c>
       <c r="Q23" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="R23" s="8" t="s">
-        <v>162</v>
+        <v>186</v>
+      </c>
+      <c r="R23" s="7" t="s">
+        <v>187</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
-        <v>93563</v>
+        <v>86787</v>
       </c>
       <c r="B24" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C24" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.57291666666666663</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>170</v>
+        <v>90</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>171</v>
+        <v>188</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>172</v>
+        <v>35</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>174</v>
+        <v>37</v>
       </c>
       <c r="I24" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>176</v>
+        <v>26</v>
       </c>
       <c r="M24" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N24" s="7" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="O24" s="7" t="s">
-        <v>178</v>
+        <v>40</v>
       </c>
       <c r="P24" s="7" t="s">
-        <v>179</v>
+        <v>80</v>
       </c>
       <c r="Q24" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="R24" s="8" t="s">
-        <v>181</v>
+        <v>42</v>
+      </c>
+      <c r="R24" s="7" t="s">
+        <v>192</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
-        <v>105005</v>
+        <v>103154</v>
       </c>
       <c r="B25" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C25" s="6">
-        <v>0.61111111111111116</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>93</v>
+        <v>115</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>158</v>
+        <v>92</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>160</v>
+        <v>195</v>
       </c>
       <c r="I25" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>38</v>
+        <v>137</v>
       </c>
       <c r="L25" s="7" t="s">
         <v>26</v>
@@ -2553,54 +2581,54 @@
         <v>27</v>
       </c>
       <c r="N25" s="7" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="O25" s="7" t="s">
-        <v>29</v>
+        <v>98</v>
       </c>
       <c r="P25" s="7" t="s">
-        <v>92</v>
+        <v>197</v>
       </c>
       <c r="Q25" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="R25" s="8" t="s">
-        <v>162</v>
+        <v>148</v>
+      </c>
+      <c r="R25" s="7" t="s">
+        <v>198</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="4">
-        <v>105009</v>
+        <v>95848</v>
       </c>
       <c r="B26" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C26" s="6">
-        <v>0.61805555555555558</v>
+        <v>0.6</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>158</v>
+        <v>35</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>160</v>
+        <v>37</v>
       </c>
       <c r="I26" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>24</v>
+        <v>190</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>38</v>
+        <v>126</v>
       </c>
       <c r="L26" s="7" t="s">
         <v>26</v>
@@ -2609,166 +2637,166 @@
         <v>27</v>
       </c>
       <c r="N26" s="7" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="O26" s="7" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="P26" s="7" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="Q26" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="R26" s="8" t="s">
-        <v>162</v>
+        <v>81</v>
+      </c>
+      <c r="R26" s="7" t="s">
+        <v>202</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="4">
-        <v>104781</v>
+        <v>105095</v>
       </c>
       <c r="B27" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C27" s="6">
-        <v>0.63194444444444442</v>
+        <v>0.60069444444444442</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>122</v>
+        <v>90</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>190</v>
+        <v>37</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>64</v>
+        <v>190</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>26</v>
+        <v>205</v>
       </c>
       <c r="M27" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N27" s="7" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
       <c r="O27" s="7" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="P27" s="7" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="Q27" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="R27" s="8" t="s">
-        <v>192</v>
+        <v>42</v>
+      </c>
+      <c r="R27" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="4">
-        <v>104065</v>
+        <v>82370</v>
       </c>
       <c r="B28" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C28" s="6">
-        <v>0.63194444444444442</v>
+        <v>0.65625</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>172</v>
+        <v>35</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>195</v>
+        <v>37</v>
       </c>
       <c r="I28" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>54</v>
+        <v>190</v>
       </c>
       <c r="K28" s="7" t="s">
-        <v>38</v>
+        <v>96</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>26</v>
+        <v>210</v>
       </c>
       <c r="M28" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N28" s="7" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="O28" s="7" t="s">
-        <v>178</v>
+        <v>40</v>
       </c>
       <c r="P28" s="7" t="s">
-        <v>197</v>
+        <v>80</v>
       </c>
       <c r="Q28" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="R28" s="8" t="s">
-        <v>43</v>
+        <v>105</v>
+      </c>
+      <c r="R28" s="7" t="s">
+        <v>212</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="4">
-        <v>103414</v>
+        <v>100423</v>
       </c>
       <c r="B29" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C29" s="6">
-        <v>0.63194444444444442</v>
+        <v>0.68055555555555558</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>144</v>
+        <v>90</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>95</v>
+        <v>214</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>199</v>
+        <v>215</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="L29" s="7" t="s">
         <v>26</v>
@@ -2777,54 +2805,54 @@
         <v>27</v>
       </c>
       <c r="N29" s="7" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="O29" s="7" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="P29" s="7" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="Q29" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="R29" s="8" t="s">
-        <v>202</v>
+        <v>218</v>
+      </c>
+      <c r="R29" s="7" t="s">
+        <v>219</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="4">
-        <v>96258</v>
+        <v>99594</v>
       </c>
       <c r="B30" s="5">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C30" s="6">
-        <v>0.65625</v>
+        <v>0.68055555555555558</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>18</v>
+        <v>90</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>34</v>
+        <v>220</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>205</v>
+        <v>145</v>
       </c>
       <c r="I30" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>207</v>
+        <v>25</v>
       </c>
       <c r="L30" s="7" t="s">
         <v>26</v>
@@ -2833,40 +2861,43 @@
         <v>27</v>
       </c>
       <c r="N30" s="7" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="O30" s="7" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="P30" s="7" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="Q30" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="R30" s="8" t="s">
-        <v>209</v>
+        <v>218</v>
+      </c>
+      <c r="R30" s="7" t="s">
+        <v>219</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R2" r:id="rId1" display="https://trt15-jus-br.zoom.us/j/87527564652?pwd=d3YrZ2diWXk5UjgzbmVkNExteWVMQT09%20ID%20da%20reunião:%20875%202756%204652%20Senha%20de%20acesso:%20246680" xr:uid="{94E2FBC1-C2E7-4B74-9E6B-DA5BAAE3929A}"/>
-    <hyperlink ref="R6" r:id="rId2" display="https://trt8-jus-br.zoom.us/j/85053969243?pwd=RVArVU1FbVNNeFhZMVdxd2x0dEpkdz09%20ID:%20850%20%205396%20%209243%20Senha:%201VTAbaete." xr:uid="{7BD1F58B-BB5E-487B-975E-14943DB5FCD3}"/>
-    <hyperlink ref="R7" r:id="rId3" display="https://trt15-jus-br.zoom.us/j/87527564652?pwd=d3YrZ2diWXk5UjgzbmVkNExteWVMQT09%20ID%20da%20reunião:%20875%202756%204652%20Senha%20de%20acesso:%20246680" xr:uid="{1C870E57-7BAE-4003-9CFB-377D4DBBA871}"/>
-    <hyperlink ref="R12" r:id="rId4" display="https://trt15-jus-br.zoom.us/j/87100825693?pwd=Ulpt0u9ZPHbqliJGGGKn8D17RPJwW2.1%20ID%20da%20reunião:%20871%200082%205693%20Senha:%20864984" xr:uid="{47BC48E8-191E-4A1B-9233-B1B5E2FB51D0}"/>
-    <hyperlink ref="R16" r:id="rId5" xr:uid="{08640A5A-8B6B-4EAC-87F5-86BCDF5D1E0E}"/>
-    <hyperlink ref="R17" r:id="rId6" xr:uid="{EF00F63F-74BE-4BD0-848A-0F4C3BD2D6EC}"/>
-    <hyperlink ref="R18" r:id="rId7" display="https://trt2-jus-br.zoom.us/j/81881873237?pwd=aEs5S29DM2srNHRuRGFVM2ZEYkVUZz09%20ID%20da%20reunião:%20818%208187%203237%20Senha%20de%20acesso:%20459217" xr:uid="{B5F8CDFE-F7E6-429A-9945-B7AD869A5935}"/>
-    <hyperlink ref="R19" r:id="rId8" xr:uid="{37E6A29D-3634-42F7-A2BB-428A9895F54C}"/>
-    <hyperlink ref="R20" r:id="rId9" display="https://trt15-jus.br.zoom.us/j/87527564652?pwd=d3YrZ2diWXk5UjgzbmVkNExteWVMQT09%20ID%20da%20reunião:%20875%202756%204652%20Senha%20de%20acesso:%20246680" xr:uid="{1D375665-4441-4541-A698-63F4F964A26C}"/>
-    <hyperlink ref="R21" r:id="rId10" xr:uid="{82EDF4DE-21BA-4D05-B9F8-4E42FA45026C}"/>
-    <hyperlink ref="R22" r:id="rId11" display="https://trt15-jus.br.zoom.us/j/87527564652?pwd=d3YrZ2diWXk5UjgzbmVkNExteWVMQT09%20ID%20da%20reunião:%20875%202756%204652%20Senha%20de%20acesso:%20246680" xr:uid="{7A149931-A36C-45C1-B336-AB52AC373069}"/>
-    <hyperlink ref="R23" r:id="rId12" xr:uid="{E4D1CF2C-D2EA-42D8-82C4-79508ACFED23}"/>
-    <hyperlink ref="R25" r:id="rId13" xr:uid="{6347FD22-0791-4EEB-80AF-63C5C4D5E585}"/>
-    <hyperlink ref="R26" r:id="rId14" xr:uid="{EAF2C722-A498-4115-A4B0-59F6A4F0100D}"/>
-    <hyperlink ref="R27" r:id="rId15" xr:uid="{DF800CF1-A92F-4AC6-A808-3A316822FA8B}"/>
-    <hyperlink ref="R29" r:id="rId16" display="https://us02web.zoom.us/j/83908187251?pwd=Ty9tcHNFb0pLZk5WQ0l2Y0V3ZHhhdz09%20ID%20da%20reunião:%20839%200818%207251%20e%20Senha%20de%20acesso:%20959576" xr:uid="{EC4398F5-76A5-439E-99D1-62C9A2059FDA}"/>
-    <hyperlink ref="R30" r:id="rId17" xr:uid="{3A595EC5-273C-450A-8DD3-51F1C8129426}"/>
+    <hyperlink ref="R5" r:id="rId1" xr:uid="{674EBA33-DB4C-4F65-9DBF-C83992C187BE}"/>
+    <hyperlink ref="R6" r:id="rId2" display="https://trt15-jus-br.zoom.us/j/87527564652?pwd=d3YrZ2diWXk5UjgzbmVkNExteWVMQT09%20ID%20da%20reunião:%20875%202756%204652%20Senha%20de%20acesso:%20246680" xr:uid="{51D7CC3B-7D15-40F8-8886-F87945A63542}"/>
+    <hyperlink ref="R7" r:id="rId3" xr:uid="{BBC7DFE6-02AE-451D-9D6D-D70D606E876D}"/>
+    <hyperlink ref="R9" r:id="rId4" xr:uid="{E4B2D7C5-FB0D-4915-ADA2-AB07515DD4DA}"/>
+    <hyperlink ref="R10" r:id="rId5" display="https://trt15-jus-br.zoom.us/j/7093890373?pwd=eEJTaWhnbTRwVXJrVTR0R0RyMUhkdz09%20Id%20da%20reunião:%207093890373%20Senha%20da%20sala:%20345356" xr:uid="{BA81ED6E-6070-4543-987B-2A91129600AE}"/>
+    <hyperlink ref="R12" r:id="rId6" xr:uid="{744E0CB7-63D1-49F3-BD9D-6F1368D0D705}"/>
+    <hyperlink ref="R13" r:id="rId7" xr:uid="{3E247091-0A76-46DD-BA1D-EA7C1ED52468}"/>
+    <hyperlink ref="R14" r:id="rId8" display="https://trt15-jus-br.zoom.us/j/81390598525?pwd=rdGf0eRPC3KeSMHZlUecdE1edZpE5R.1%20ID%20da%20reunião:%20813%209059%208525%20Senha:%20127812" xr:uid="{116199DB-19CB-4BD3-9E9C-64F81FCF17B6}"/>
+    <hyperlink ref="R15" r:id="rId9" display="https://us02web.zoom.us/j/85763756385?pwd=ZTBCT3ZkZVg1QUVqMFVBNFcxUDdmQT0%20%20ID:%20857%206375%206385%20e%20Senha%20de%20acesso:%20958777" xr:uid="{C6692C79-2C91-4182-A7EF-A7EECCCC3633}"/>
+    <hyperlink ref="R16" r:id="rId10" xr:uid="{AB9E8971-11FC-41B1-82DB-23804E4DB5CF}"/>
+    <hyperlink ref="R20" r:id="rId11" display="https://trt15-jus-br.zoom.us/j/86722354209?pwd=V01VL0NmTFZSZEdhcFhjM0tIczd3dz09%20ID%20da%20reunião:%20867%202235%204209%20Senha%20de%20acesso:%20947812" xr:uid="{71DE643D-5A35-4DCA-92EA-A02CC577F5D6}"/>
+    <hyperlink ref="R22" r:id="rId12" display="https://us02web.zoom.us/j/83352065501?pwd=Lzc2WUJGSVpVWmJyZjB3Y0NvUmJPZz09%20ID%20da%20reunião:%2083352065501%20Senha%20de%20acesso:%20368465" xr:uid="{5C8A79B5-83CE-4DF1-AE4D-1434CA2F9630}"/>
+    <hyperlink ref="R23" r:id="rId13" xr:uid="{81D42F8B-DE70-40B5-BC7E-DD0DAD019305}"/>
+    <hyperlink ref="R24" r:id="rId14" display="https://trt2-jus-br.zoom.us/j/82477928530?pwd=WENUNkRGZ1NLbUY4VFZLdjdjOXBxUT09%20ID%20da%20reunião:%20824%207792%208530%20Senha%20de%20acesso:%20391604" xr:uid="{777747EE-C094-4B75-8081-C54A173801A0}"/>
+    <hyperlink ref="R25" r:id="rId15" display="https://us02web.zoom.us/j/8060729658?pwd=NDNlcU8wVzcxZ09qVjFDRFBGT2ljQT09%20ID%20da%20reunião:%20806%20072%209658%20Senha%20de%20acesso:%20868717" xr:uid="{6EC88838-5C81-409F-8423-DF2EB0405174}"/>
+    <hyperlink ref="R26" r:id="rId16" display="https://trt2-jus-br.zoom.us/j/88297719933?pwd=U3VWVjB2RHh0Vm9VMHZ0ZFd1eUk1dz09%20ID%20da%20reunião:%20882%209771%209933%20Senha%20de%20acesso:%20091850" xr:uid="{4C940D36-102D-4184-95F2-EB8CD6BB9E33}"/>
+    <hyperlink ref="R27" r:id="rId17" display="https://trt2-jus-br.zoom.us/j/88959116257?pwd=Q09WTmd6SnZibUUrZWxMSFdiRm9tUT09%20ID%20da%20reunião:%20889%205911%206257%20Senha%20de%20acesso:%20136898" xr:uid="{3AF64A62-9914-4A16-874E-BB858570944E}"/>
+    <hyperlink ref="R28" r:id="rId18" display="https://trt2-jus-br.zoom.us/j/85239557292?pwd=enBMVGxIVlR2bG5uUmk3Sy8yWmR6dz09%20ID%20da%20reunião:%20852%203955%207292%20Senha%20de%20acesso:%20611035" xr:uid="{182D42C1-7F0E-410E-ACC1-2B66CF202943}"/>
+    <hyperlink ref="R29" r:id="rId19" xr:uid="{E437BA56-71D0-4212-8E39-1C8AE4C59A2C}"/>
+    <hyperlink ref="R30" r:id="rId20" xr:uid="{3B93FBF5-C574-4FA2-B257-92DA549A27A8}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Audiências: sync 2026-07-30 — 29 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="145">
   <si>
     <t>data</t>
   </si>
@@ -49,379 +49,406 @@
     <t>horario</t>
   </si>
   <si>
-    <t>Fatal</t>
+    <t>D-1</t>
+  </si>
+  <si>
+    <t>BCF</t>
+  </si>
+  <si>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>VCR</t>
+  </si>
+  <si>
+    <t>VSI</t>
   </si>
   <si>
     <t>AAP</t>
   </si>
   <si>
-    <t>Correspondente - Hebert</t>
+    <t>RRU</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>JPL</t>
+  </si>
+  <si>
+    <t>GSM</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>JNE</t>
+  </si>
+  <si>
+    <t>TLI</t>
+  </si>
+  <si>
+    <t>JRM</t>
   </si>
   <si>
     <t>LMI</t>
   </si>
   <si>
-    <t>ANB</t>
-  </si>
-  <si>
-    <t>ARC</t>
-  </si>
-  <si>
-    <t>RYL</t>
+    <t>Correspondente - Carlos Florian</t>
   </si>
   <si>
     <t>FCG</t>
   </si>
   <si>
-    <t>TFR</t>
-  </si>
-  <si>
-    <t>VSI</t>
-  </si>
-  <si>
-    <t>JPE</t>
-  </si>
-  <si>
-    <t>MBF</t>
-  </si>
-  <si>
-    <t>CAL</t>
-  </si>
-  <si>
-    <t>RRU</t>
-  </si>
-  <si>
-    <t>VCR</t>
-  </si>
-  <si>
-    <t>BCF</t>
-  </si>
-  <si>
-    <t>JNE</t>
+    <t>ECO</t>
+  </si>
+  <si>
+    <t>DPR</t>
+  </si>
+  <si>
+    <t>RFE</t>
+  </si>
+  <si>
+    <t>Grupo B2</t>
+  </si>
+  <si>
+    <t>Grupo B1</t>
+  </si>
+  <si>
+    <t>Grupo C</t>
   </si>
   <si>
     <t>Grupo E2</t>
   </si>
   <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>Grupo B3</t>
-  </si>
-  <si>
-    <t>Grupo C</t>
-  </si>
-  <si>
-    <t>Grupo B2</t>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>Grupo D1</t>
+  </si>
+  <si>
+    <t>Embraer S.A.</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
   </si>
   <si>
     <t>Viterra Bioenergia S.A.</t>
   </si>
   <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Companhia Brasileira De Cartuchos</t>
-  </si>
-  <si>
-    <t>Fertilizantes Tocantins S.A</t>
-  </si>
-  <si>
-    <t>Panificadora Cepam Ltda.</t>
+    <t>Fertilizantes Heringer S.A</t>
+  </si>
+  <si>
+    <t>Guariroba Bioenergia Ltda. &amp; Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Monteverde</t>
+  </si>
+  <si>
+    <t>Ouroeste Bioenergia Ltda.</t>
   </si>
   <si>
     <t>Moema Bioenergia S.A. - Moema</t>
   </si>
   <si>
-    <t>Telefonica Brasil S.A.</t>
-  </si>
-  <si>
-    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
-  </si>
-  <si>
-    <t>Salitre Fertilizantes Ltda.</t>
-  </si>
-  <si>
-    <t>Guariroba Bioenergia Ltda.</t>
-  </si>
-  <si>
-    <t>Embraer S.A.</t>
-  </si>
-  <si>
-    <t>Audiência de Conciliação - Semipresencial</t>
+    <t>Syngenta Seeds Ltda.</t>
+  </si>
+  <si>
+    <t>Colégio Curumim S/S Ltda</t>
+  </si>
+  <si>
+    <t>Ame Digital Brasil Ltda</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A. - Paulinia - Pln</t>
+  </si>
+  <si>
+    <t>Rio Parana Energia S.A</t>
+  </si>
+  <si>
+    <t>Construtora Elias Victor Nigri Ltda.</t>
+  </si>
+  <si>
+    <t>L. Sant'Angelo Pinturas Ltda.</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Presencial</t>
   </si>
   <si>
     <t>Audiência Instrução - Presencial</t>
   </si>
   <si>
-    <t>Audiência Inicial -  Presencial</t>
+    <t>Audiência Inicial -  Telepresencial</t>
   </si>
   <si>
     <t>Audiência Una - Telepresencial</t>
   </si>
   <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
     <t>Audiência Una - Presencial</t>
   </si>
   <si>
-    <t>Audiência Inicial -  Telepresencial</t>
+    <t>Audiência de Instrução - Semipresencial</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Semipresencial</t>
+  </si>
+  <si>
+    <t>Perícia Técnica</t>
   </si>
   <si>
     <t>Audiência Inicial - Presencial</t>
   </si>
   <si>
-    <t>Sessão de Julgamento TRT - Presencial</t>
-  </si>
-  <si>
-    <t>Audiência Inicial - Telepresencial</t>
-  </si>
-  <si>
-    <t>Audiência de Conciliação - Telepresencial</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Telepresencial</t>
-  </si>
-  <si>
-    <t>Perícia Técnica</t>
-  </si>
-  <si>
-    <t>0010685-63.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>1000527-98.2026.5.02.0435</t>
-  </si>
-  <si>
-    <t>1000832-57.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>1000628-78.2025.5.02.0433</t>
-  </si>
-  <si>
-    <t>0000827-44.2026.5.08.0101</t>
-  </si>
-  <si>
-    <t>0010704-69.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>1001851-66.2025.5.02.0433</t>
-  </si>
-  <si>
-    <t>1002207-61.2025.5.02.0433</t>
-  </si>
-  <si>
-    <t>1001238-18.2026.5.02.0431</t>
-  </si>
-  <si>
-    <t>1001373-05.2026.5.02.0601</t>
-  </si>
-  <si>
-    <t>0011042-44.2026.5.15.0082</t>
-  </si>
-  <si>
-    <t>1001057-08.2026.5.02.0434</t>
-  </si>
-  <si>
-    <t>1000383-33.2026.5.02.0433</t>
-  </si>
-  <si>
-    <t>1000592-97.2025.5.02.0445</t>
-  </si>
-  <si>
-    <t>0001617-53.2025.5.09.0095</t>
-  </si>
-  <si>
-    <t>0001757-47.2025.5.09.0658</t>
-  </si>
-  <si>
-    <t>1000780-92.2026.5.02.0433</t>
-  </si>
-  <si>
-    <t>0010215-72.2026.5.03.0080</t>
-  </si>
-  <si>
-    <t>0010173-80.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>0010480-06.2026.5.15.0027</t>
-  </si>
-  <si>
-    <t>0010175-50.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>0010530-32.2026.5.15.0027</t>
-  </si>
-  <si>
-    <t>1019460-73.2020.8.26.0577</t>
-  </si>
-  <si>
-    <t>0010609-11.2026.5.15.0027</t>
-  </si>
-  <si>
-    <t>0010607-41.2026.5.15.0027</t>
-  </si>
-  <si>
-    <t>0010417-72.2026.5.15.0029</t>
-  </si>
-  <si>
-    <t>0010300-33.2026.5.15.0045</t>
-  </si>
-  <si>
-    <t>0012892-87.2025.5.15.0044</t>
-  </si>
-  <si>
-    <t>0010541-87.2019.5.15.0130</t>
-  </si>
-  <si>
-    <t>Michel Roque Martins Dias</t>
-  </si>
-  <si>
-    <t>Mistoncleso Cruz Da Silva</t>
-  </si>
-  <si>
-    <t>Marli Nogueira Da Silva</t>
-  </si>
-  <si>
-    <t>Adriano Jose Da Silva</t>
-  </si>
-  <si>
-    <t>Rildo Dos Santos Dias</t>
-  </si>
-  <si>
-    <t>Bruno Duque Vanderlei</t>
-  </si>
-  <si>
-    <t>Yago Henrique Almeida Luz</t>
-  </si>
-  <si>
-    <t>Giovani Gustavo Ferreira Da Silva</t>
-  </si>
-  <si>
-    <t>Reinaldo Monteiro</t>
-  </si>
-  <si>
-    <t>Carlos Alberto Arruda Croda</t>
-  </si>
-  <si>
-    <t>Renan De Azevedo Gomes</t>
-  </si>
-  <si>
-    <t>Elizeu Luiz Freire</t>
-  </si>
-  <si>
-    <t>Wesley Thiago Dos Santos Silva</t>
-  </si>
-  <si>
-    <t>Marisilda Henriques</t>
-  </si>
-  <si>
-    <t>Rafael Cordeiro Gripa</t>
-  </si>
-  <si>
-    <t>Arilson Moraes De Almeida</t>
-  </si>
-  <si>
-    <t>Flavio Luiz Cossa</t>
-  </si>
-  <si>
-    <t>Ronan Ramos Gregorio Almeida</t>
-  </si>
-  <si>
-    <t>Vinicius Andre Freitas Diniz</t>
-  </si>
-  <si>
-    <t>Ricardo Mauricio Contel</t>
-  </si>
-  <si>
-    <t>Valdir Pereira Leal</t>
-  </si>
-  <si>
-    <t>Thalia Francisca Ribeiro Da Silva E Silva</t>
-  </si>
-  <si>
-    <t>Daniel Dos Santos Barbosa</t>
-  </si>
-  <si>
-    <t>Tiago Vieira De Sousa</t>
-  </si>
-  <si>
-    <t>Damiao Euflausino Alves</t>
-  </si>
-  <si>
-    <t>Daniel Antonio</t>
-  </si>
-  <si>
-    <t>Matheus Alberto Silva</t>
-  </si>
-  <si>
-    <t>Marcos Lopes Da Silva</t>
-  </si>
-  <si>
-    <t>Gilson Trindade Gama</t>
+    <t>0011446-11.2026.5.15.0013</t>
+  </si>
+  <si>
+    <t>1001605-70.2025.5.02.0433</t>
+  </si>
+  <si>
+    <t>0012525-60.2025.5.15.0045</t>
+  </si>
+  <si>
+    <t>0000008-89.2026.5.09.0195</t>
+  </si>
+  <si>
+    <t>0010718-53.2026.5.15.0050</t>
+  </si>
+  <si>
+    <t>0010598-92.2026.5.03.0066</t>
+  </si>
+  <si>
+    <t>1000510-62.2026.5.02.0435</t>
+  </si>
+  <si>
+    <t>0010657-67.2026.5.15.0027</t>
+  </si>
+  <si>
+    <t>0012012-63.2024.5.15.0066</t>
+  </si>
+  <si>
+    <t>1000584-28.2026.5.02.0432</t>
+  </si>
+  <si>
+    <t>0024058-02.2026.5.24.0022</t>
+  </si>
+  <si>
+    <t>0011078-07.2025.5.03.0066</t>
+  </si>
+  <si>
+    <t>0011770-60.2025.5.15.0037</t>
+  </si>
+  <si>
+    <t>0012741-24.2025.5.15.0044</t>
+  </si>
+  <si>
+    <t>0001208-68.2025.5.09.0195</t>
+  </si>
+  <si>
+    <t>1000639-09.2026.5.02.0034</t>
+  </si>
+  <si>
+    <t>1002378-21.2025.5.02.0432</t>
+  </si>
+  <si>
+    <t>1001149-46.2026.5.02.0511</t>
+  </si>
+  <si>
+    <t>0010921-49.2025.5.15.0050</t>
+  </si>
+  <si>
+    <t>1001275-39.2026.5.02.0433</t>
+  </si>
+  <si>
+    <t>0011437-35.2025.5.15.0126</t>
+  </si>
+  <si>
+    <t>0024683-80.2026.5.24.0072</t>
+  </si>
+  <si>
+    <t>1000607-04.2022.5.02.0435</t>
+  </si>
+  <si>
+    <t>0011841-62.2025.5.15.0134</t>
+  </si>
+  <si>
+    <t>1001826-18.2023.5.02.0435</t>
+  </si>
+  <si>
+    <t>1000899-59.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>1001342-80.2021.5.02.0432</t>
+  </si>
+  <si>
+    <t>1001636-94.2024.5.02.0055</t>
+  </si>
+  <si>
+    <t>Luciano Aparecido Pereira</t>
+  </si>
+  <si>
+    <t>Everton Caldeira Marquesine</t>
+  </si>
+  <si>
+    <t>Reinaldo Aparecido Dos Santos</t>
+  </si>
+  <si>
+    <t>Everaldo Kovalchuk</t>
+  </si>
+  <si>
+    <t>Marco Aurelio Claudio</t>
+  </si>
+  <si>
+    <t>Marcos Paulo Da Silva</t>
+  </si>
+  <si>
+    <t>Cleiton Mendonca De Souza</t>
+  </si>
+  <si>
+    <t>Fernando Henrique Grecco Dos Santos Garcia</t>
+  </si>
+  <si>
+    <t>Edivane Dos Santos</t>
+  </si>
+  <si>
+    <t>Welington Tavian Baptista</t>
+  </si>
+  <si>
+    <t>Taiane Lima Da Silva</t>
+  </si>
+  <si>
+    <t>Walleska Souza Menezes</t>
+  </si>
+  <si>
+    <t>Isabela Carolina Bento Belini Vilela</t>
+  </si>
+  <si>
+    <t>Gilberlandio Cascimiro Barbosa</t>
+  </si>
+  <si>
+    <t>Cerli Coelho Gomes</t>
+  </si>
+  <si>
+    <t>Andre Luiz Da Silva Rocumback</t>
+  </si>
+  <si>
+    <t>Marcilio Alan Ferreira Cavalcanti</t>
+  </si>
+  <si>
+    <t>Daiana Arruda Santos Silva</t>
+  </si>
+  <si>
+    <t>Joao Maria Bonifacio Ribeiro</t>
+  </si>
+  <si>
+    <t>Danilo Oliveira De Lima</t>
+  </si>
+  <si>
+    <t>Jose Maria Pereira</t>
+  </si>
+  <si>
+    <t>Flavio Rodrigues Valente</t>
+  </si>
+  <si>
+    <t>Marcelo Silva Rodrigues</t>
+  </si>
+  <si>
+    <t>Tiago Viegas Carvalho</t>
+  </si>
+  <si>
+    <t>Rodrigo Fernandes Da Silva</t>
+  </si>
+  <si>
+    <t>Carlos Alberto De Castro</t>
+  </si>
+  <si>
+    <t>Natanael Marques Vieira</t>
+  </si>
+  <si>
+    <t>Derivaldo Dos Santos Silva</t>
+  </si>
+  <si>
+    <t>08:00:00</t>
+  </si>
+  <si>
+    <t>08:20:00</t>
   </si>
   <si>
     <t>08:30:00</t>
   </si>
   <si>
-    <t>08:50:00</t>
-  </si>
-  <si>
     <t>09:00:00</t>
   </si>
   <si>
-    <t>09:15:00</t>
-  </si>
-  <si>
     <t>09:20:00</t>
   </si>
   <si>
-    <t>09:50:00</t>
+    <t>09:30:00</t>
   </si>
   <si>
     <t>10:00:00</t>
   </si>
   <si>
-    <t>10:10:00</t>
+    <t>10:13:00</t>
+  </si>
+  <si>
+    <t>10:20:00</t>
   </si>
   <si>
     <t>10:30:00</t>
   </si>
   <si>
-    <t>11:20:00</t>
-  </si>
-  <si>
-    <t>11:50:00</t>
-  </si>
-  <si>
-    <t>13:00:00</t>
-  </si>
-  <si>
-    <t>13:27:00</t>
-  </si>
-  <si>
-    <t>13:34:00</t>
-  </si>
-  <si>
-    <t>13:42:00</t>
+    <t>10:40:00</t>
+  </si>
+  <si>
+    <t>11:10:00</t>
+  </si>
+  <si>
+    <t>11:25:00</t>
+  </si>
+  <si>
+    <t>11:30:00</t>
+  </si>
+  <si>
+    <t>11:40:00</t>
+  </si>
+  <si>
+    <t>13:15:00</t>
+  </si>
+  <si>
+    <t>13:44:00</t>
+  </si>
+  <si>
+    <t>13:45:00</t>
   </si>
   <si>
     <t>14:00:00</t>
   </si>
   <si>
-    <t>14:20:00</t>
-  </si>
-  <si>
-    <t>14:30:00</t>
-  </si>
-  <si>
-    <t>14:40:00</t>
-  </si>
-  <si>
-    <t>14:50:00</t>
-  </si>
-  <si>
-    <t>15:10:00</t>
+    <t>14:24:00</t>
+  </si>
+  <si>
+    <t>14:25:00</t>
   </si>
   <si>
     <t>15:45:00</t>
+  </si>
+  <si>
+    <t>16:20:00</t>
   </si>
 </sst>
 </file>
@@ -797,7 +824,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -806,33 +833,33 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H2" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="I2" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="J2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="K2" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
@@ -841,33 +868,33 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F3" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="G3" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="H3" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="I3" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="J3" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="K3" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
@@ -876,33 +903,33 @@
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="G4" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="H4" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="I4" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="J4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="K4" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
@@ -911,33 +938,33 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="F5" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="G5" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="H5" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="I5" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="J5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="K5" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
@@ -946,313 +973,313 @@
         <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F6" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="G6" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="H6" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="I6" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="J6" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="K6" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="F7" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="H7" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="I7" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="J7" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="K7" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F8" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="G8" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="H8" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="I8" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="J8" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="K8" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="F9" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="H9" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="I9" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="J9" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="K9" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="E10" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="F10" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="G10" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I10" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="J10" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="K10" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F11" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="G11" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="H11" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="I11" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="J11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K11" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B12" t="s">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="E12" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="F12" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="G12" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="H12" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="I12" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="J12" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="K12" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E13" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="F13" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="G13" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="H13" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="I13" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="J13" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="K13" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D14" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="F14" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="G14" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="H14" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="I14" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="J14" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="K14" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B15" t="s">
         <v>11</v>
@@ -1261,418 +1288,418 @@
         <v>19</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E15" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="F15" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="G15" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="H15" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="I15" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="J15" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="K15" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B16" t="s">
         <v>11</v>
       </c>
       <c r="C16" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D16" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E16" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F16" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="G16" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="H16" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="I16" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="J16" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="K16" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B17" t="s">
         <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D17" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E17" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="F17" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="G17" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="H17" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="I17" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J17" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="K17" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B18" t="s">
         <v>11</v>
       </c>
       <c r="C18" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D18" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E18" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F18" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G18" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="H18" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="I18" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="J18" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="K18" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B19" t="s">
         <v>11</v>
       </c>
       <c r="C19" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D19" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="E19" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="F19" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="G19" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="H19" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="I19" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="J19" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="K19" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B20" t="s">
         <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F20" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G20" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="H20" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="I20" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="J20" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="K20" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B21" t="s">
         <v>11</v>
       </c>
       <c r="C21" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="D21" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E21" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F21" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="G21" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="H21" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I21" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="J21" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K21" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B22" t="s">
         <v>11</v>
       </c>
       <c r="C22" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D22" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="E22" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="F22" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="G22" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="H22" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="I22" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="J22" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="K22" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B23" t="s">
         <v>11</v>
       </c>
       <c r="C23" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="D23" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E23" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="F23" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="G23" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="H23" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="I23" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="J23" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="K23" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B24" t="s">
         <v>11</v>
       </c>
       <c r="C24" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D24" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E24" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F24" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G24" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="H24" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="I24" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="J24" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="K24" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B25" t="s">
         <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D25" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="E25" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F25" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="G25" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="H25" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="I25" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="J25" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K25" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B26" t="s">
         <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D26" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E26" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F26" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="G26" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="H26" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="I26" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="J26" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K26" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B27" t="s">
         <v>11</v>
@@ -1681,133 +1708,133 @@
         <v>18</v>
       </c>
       <c r="D27" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E27" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F27" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="G27" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="H27" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="I27" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="J27" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="K27" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B28" t="s">
         <v>11</v>
       </c>
       <c r="C28" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D28" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E28" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F28" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="G28" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="H28" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="I28" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="J28" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="K28" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B29" t="s">
         <v>11</v>
       </c>
       <c r="C29" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="E29" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="F29" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G29" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="H29" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="I29" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="J29" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="K29" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B30" t="s">
         <v>11</v>
       </c>
       <c r="C30" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E30" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="F30" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="G30" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="H30" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="I30" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="J30" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="K30" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Audiências: sync 2026-08-03 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DEDD9EB7-52E2-42D9-8E49-8A48D449AD11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B141AB2-1407-4168-AE07-1B4FAA8B790F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0E2B891C-2E1B-4231-B07B-EF8302005628}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0E2B891C-2E1B-4231-B07B-EF8302005628}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="155">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,18 +95,9 @@
     <t>Link/Observações</t>
   </si>
   <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>1000058-52.2026.5.02.0435</t>
-  </si>
-  <si>
     <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
   </si>
   <si>
-    <t>Anilton De Sa Silva</t>
-  </si>
-  <si>
     <t>SANTO ANDRÉ</t>
   </si>
   <si>
@@ -125,116 +116,401 @@
     <t>CENTRAL</t>
   </si>
   <si>
-    <t>R$             334.173,52</t>
-  </si>
-  <si>
     <t>Grupo B1</t>
   </si>
   <si>
     <t>JPE</t>
   </si>
   <si>
-    <t>GSM</t>
-  </si>
-  <si>
     <t>Presencial</t>
   </si>
   <si>
     <t>Audiência Una - Telepresencial</t>
   </si>
   <si>
-    <t>0000074-09.2026.5.21.0010</t>
-  </si>
-  <si>
-    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
-  </si>
-  <si>
-    <t>Everton Muller Da Costa Maia</t>
-  </si>
-  <si>
-    <t>NATAL</t>
-  </si>
-  <si>
-    <t>RN</t>
-  </si>
-  <si>
-    <t>10ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$               52.315,43</t>
-  </si>
-  <si>
     <t>Grupo C</t>
   </si>
   <si>
-    <t>VSI</t>
-  </si>
-  <si>
-    <t>https://trt21-jus-br.zoom.us/my/natal10vt</t>
-  </si>
-  <si>
     <t>Audiência Una - Presencial</t>
   </si>
   <si>
-    <t>1000586-95.2026.5.02.0432</t>
-  </si>
-  <si>
-    <t>Vagner Aparecido Da Silva</t>
-  </si>
-  <si>
     <t>02ª VARA DO TRABALHO</t>
   </si>
   <si>
-    <t>R$             196.932,24</t>
-  </si>
-  <si>
     <t>Correspondente - Hebert</t>
   </si>
   <si>
     <t>RFE</t>
   </si>
   <si>
-    <t>1000303-38.2026.5.02.0411</t>
-  </si>
-  <si>
     <t>Cbc - Companhia Brasileira De Cartuchos</t>
   </si>
   <si>
-    <t>Mariane Paulino Dos Santos Alves</t>
-  </si>
-  <si>
     <t>RIBEIRÃO PIRES</t>
   </si>
   <si>
     <t>VARA DO TRABALHO</t>
   </si>
   <si>
-    <t>R$             348.205,41</t>
-  </si>
-  <si>
     <t>Grupo B3</t>
   </si>
   <si>
     <t>LMI</t>
   </si>
   <si>
-    <t>1000859-40.2026.5.02.0411</t>
-  </si>
-  <si>
     <t>Companhia Brasileira De Cartuchos</t>
   </si>
   <si>
-    <t>Elismar Pereira De Jesus Brito</t>
-  </si>
-  <si>
-    <t>R$               50.170,61</t>
+    <t>Audiência Inicial -  Telepresencial</t>
+  </si>
+  <si>
+    <t>0011284-81.2026.5.03.0164</t>
+  </si>
+  <si>
+    <t>Sistenge Construcoes E Comercio Ltda</t>
+  </si>
+  <si>
+    <t>Marionsergio Campos Cabral</t>
+  </si>
+  <si>
+    <t>CONTAGEM</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>06ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               31.127,22</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>JNE</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/j/81126952316</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Telepresencial</t>
+  </si>
+  <si>
+    <t>0011650-59.2026.5.15.0044</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Antonio Carlos Espejo</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DO RIO PRETO</t>
+  </si>
+  <si>
+    <t>R$             315.485,31</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/87555371032?pwd=ckVSVmpnMHBpcnhHQUZzd0VtT0JBUT09   ID DA REUNIÃO: 875 5537 1032 SENHA DE ACESSO: 772981</t>
+  </si>
+  <si>
+    <t>1001261-61.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>Potira Brunhera</t>
+  </si>
+  <si>
+    <t>01ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               28.968,13</t>
+  </si>
+  <si>
+    <t>TAM</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>1001249-53.2025.5.02.0020</t>
+  </si>
+  <si>
+    <t>Cleivan Oliveira Amorim</t>
+  </si>
+  <si>
+    <t>SÃO PAULO</t>
+  </si>
+  <si>
+    <t>20ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             254.352,14</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/87319779344?pwd=XGh65AWoaNQktqbDH9bXKlU0RqZckb.1 ID da reunião: 873 1977 9344 Senha de acesso: 863962</t>
+  </si>
+  <si>
+    <t>1000659-67.2026.5.02.0432</t>
+  </si>
+  <si>
+    <t>Jose Roberto Lopes Da Silva</t>
+  </si>
+  <si>
+    <t>R$             280.302,24</t>
+  </si>
+  <si>
+    <t>0000031-87.2026.5.18.0129</t>
+  </si>
+  <si>
+    <t>Uhe São Simão Energia S.A.</t>
+  </si>
+  <si>
+    <t>Wigor Paulo Saturno Fernandes</t>
+  </si>
+  <si>
+    <t>QUIRINÓPOLIS</t>
+  </si>
+  <si>
+    <t>GO</t>
+  </si>
+  <si>
+    <t>R$             204.522,65</t>
+  </si>
+  <si>
+    <t>ECO</t>
+  </si>
+  <si>
+    <t>https://trt18-jus-br.zoom.us/j/89772670047</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>0020030-93.2024.5.04.0029</t>
+  </si>
+  <si>
+    <t>Francisco Boaventura Teixeira Moreira</t>
+  </si>
+  <si>
+    <t>PORTO ALEGRE</t>
+  </si>
+  <si>
+    <t>RS</t>
+  </si>
+  <si>
+    <t>CEJUSC 2º GRAU</t>
+  </si>
+  <si>
+    <t>R$             100.000,00</t>
+  </si>
+  <si>
+    <t>Correspondente - Jaeger</t>
+  </si>
+  <si>
+    <t>https://trt4-jus-br.zoom.us/my/cejusc.revista.sala3 ID da reunião:  286 582 7324</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Presencial</t>
+  </si>
+  <si>
+    <t>1001341-13.2026.5.02.0435</t>
+  </si>
+  <si>
+    <t>Nilson Ignacio</t>
+  </si>
+  <si>
+    <t>R$               76.540,57</t>
+  </si>
+  <si>
+    <t>1000939-53.2026.5.02.0039</t>
+  </si>
+  <si>
+    <t>Mitre Realty Empreendimentos E Participacoes Ltda.</t>
+  </si>
+  <si>
+    <t>Aparecida Ferreira Da Silva Mendes</t>
+  </si>
+  <si>
+    <t>39ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             345.284,94</t>
+  </si>
+  <si>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>1000858-55.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>Marco Antonio Ferreira De Moura</t>
+  </si>
+  <si>
+    <t>R$               60.000,00</t>
+  </si>
+  <si>
+    <t>1000815-21.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>Maikon Flavio Gomes Dos Santos</t>
+  </si>
+  <si>
+    <t>R$               54.319,65</t>
+  </si>
+  <si>
+    <t>1000864-62.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>Silene Antonia Silva De Lima</t>
+  </si>
+  <si>
+    <t>R$               67.618,05</t>
+  </si>
+  <si>
+    <t>0010612-97.2026.5.03.0156</t>
+  </si>
+  <si>
+    <t>Frutal Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Fernanda De Jesus Martins</t>
+  </si>
+  <si>
+    <t>FRUTAL</t>
+  </si>
+  <si>
+    <t>Ação de Consignação em Pagamento</t>
+  </si>
+  <si>
+    <t>R$                 5.463,72</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vtfrutal</t>
+  </si>
+  <si>
+    <t>0012826-11.2024.5.15.0152</t>
+  </si>
+  <si>
+    <t>Dell Computadores Do Brasil Ltda</t>
+  </si>
+  <si>
+    <t>Rafael Reboucas Dos Santos</t>
+  </si>
+  <si>
+    <t>HORTOLÂNDIA</t>
+  </si>
+  <si>
+    <t>CEJUSC</t>
+  </si>
+  <si>
+    <t>R$                 4.116,31</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>ALF</t>
+  </si>
+  <si>
+    <t>https://bit.ly/cejusclimeirasala1</t>
+  </si>
+  <si>
+    <t>0024175-55.2026.5.24.0066</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Monteverde</t>
+  </si>
+  <si>
+    <t>Dionaty Sousa Dos Santos</t>
+  </si>
+  <si>
+    <t>PONTA PORÃ</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>R$               55.756,42</t>
+  </si>
+  <si>
+    <t>FCG</t>
+  </si>
+  <si>
+    <t>https://trt24-jus-br.zoom.us/j/88062331360</t>
+  </si>
+  <si>
+    <t>1001486-47.2025.5.02.0001</t>
+  </si>
+  <si>
+    <t>Telefonica Brasil S.A.</t>
+  </si>
+  <si>
+    <t>Luciene Vicentina Pereira Barros</t>
+  </si>
+  <si>
+    <t>Recursal</t>
+  </si>
+  <si>
+    <t>Cumprimento de Sentença</t>
+  </si>
+  <si>
+    <t>R$             360.084,51</t>
+  </si>
+  <si>
+    <t>TFR</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/81939223002?pwd=VbNbYIp6i5iFsvbFRWAbpt9hdRmaMd.1 ID da reunião: 819 3922 3002 Senha de acesso: 958620</t>
+  </si>
+  <si>
+    <t>0010653-93.2026.5.15.0103</t>
+  </si>
+  <si>
+    <t>Viterra Bioenergia S.A</t>
+  </si>
+  <si>
+    <t>Marcelo Aparecido Da Silva</t>
+  </si>
+  <si>
+    <t>ARAÇATUBA</t>
+  </si>
+  <si>
+    <t>03ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               99.314,26</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/81582489033?pwd=WFBLcGVJNkJMaWQ2Y3JqZ3d6YjIydz09 ID da reunião: 815 824 9033 Senha: 1234</t>
+  </si>
+  <si>
+    <t>1001114-58.2026.5.02.0003</t>
+  </si>
+  <si>
+    <t>T4F Entretenimento S.A.</t>
+  </si>
+  <si>
+    <t>Luiz Carlos Vieira De Jesus</t>
+  </si>
+  <si>
+    <t>R$               25.644,85</t>
+  </si>
+  <si>
+    <t>ANB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -254,6 +530,14 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -276,7 +560,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -332,11 +616,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -359,8 +672,27 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -693,7 +1025,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{459E5191-63A4-4A99-A31D-30E5C65929BB}">
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
@@ -715,7 +1047,7 @@
     <col min="18" max="18" width="32.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -772,288 +1104,1025 @@
       </c>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
-        <v>103781</v>
-      </c>
-      <c r="B2" s="5">
-        <v>46234</v>
-      </c>
-      <c r="C2" s="6">
-        <v>0.3611111111111111</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="7" t="s">
+      <c r="A2" s="8">
+        <v>105542</v>
+      </c>
+      <c r="B2" s="9">
+        <v>46237</v>
+      </c>
+      <c r="C2" s="10">
+        <v>0.34027777777777779</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="K2" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="L2" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="M2" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="K2" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q2" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="R2" s="7" t="s">
-        <v>32</v>
+      <c r="N2" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="R2" s="12" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
-        <v>103864</v>
+        <v>105498</v>
       </c>
       <c r="B3" s="5">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="C3" s="6">
-        <v>0.375</v>
+        <v>0.3576388888888889</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="P3" s="7" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="Q3" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="R3" s="7" t="s">
-        <v>43</v>
+        <v>49</v>
+      </c>
+      <c r="R3" s="13" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
-        <v>104570</v>
+        <v>105456</v>
       </c>
       <c r="B4" s="5">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="C4" s="6">
-        <v>0.4201388888888889</v>
+        <v>0.375</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="F4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4" s="7" t="s">
+      <c r="J4" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="K4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="L4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="K4" s="7" t="s">
+      <c r="M4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="O4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="L4" s="7" t="s">
+      <c r="P4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="M4" s="7" t="s">
+      <c r="Q4" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="R4" s="7" t="s">
         <v>27</v>
-      </c>
-      <c r="N4" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="O4" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="P4" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q4" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="R4" s="7" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
-        <v>104333</v>
+        <v>101846</v>
       </c>
       <c r="B5" s="5">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="C5" s="6">
-        <v>0.44444444444444442</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>26</v>
-      </c>
       <c r="M5" s="7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="O5" s="7" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="Q5" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="R5" s="7" t="s">
-        <v>32</v>
+        <v>38</v>
+      </c>
+      <c r="R5" s="13" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
-        <v>105245</v>
+        <v>104679</v>
       </c>
       <c r="B6" s="5">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="C6" s="6">
+        <v>0.39930555555555558</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="R6" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>103777</v>
+      </c>
+      <c r="B7" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C7" s="6">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="R7" s="13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>97099</v>
+      </c>
+      <c r="B8" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0.44791666666666669</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="P8" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="R8" s="13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>105532</v>
+      </c>
+      <c r="B9" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N9" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="O9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="P9" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>105224</v>
+      </c>
+      <c r="B10" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="O10" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="P10" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q10" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="R10" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>105244</v>
+      </c>
+      <c r="B11" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.4826388888888889</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N11" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="O11" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="P11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>105210</v>
+      </c>
+      <c r="B12" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C12" s="6">
         <v>0.50347222222222221</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="I6" s="7" t="s">
+      <c r="D12" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L12" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="J6" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="M6" s="7" t="s">
+      <c r="M12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N12" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="O12" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="P12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="R12" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N6" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="P6" s="7" t="s">
+    </row>
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>105288</v>
+      </c>
+      <c r="B13" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.51388888888888884</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N13" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="O13" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="P13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>105433</v>
+      </c>
+      <c r="B14" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.57986111111111116</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N14" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="O14" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="P14" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="Q6" s="7" t="s">
+      <c r="Q14" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="R6" s="7" t="s">
-        <v>32</v>
+      <c r="R14" s="13" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>99562</v>
+      </c>
+      <c r="B15" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.59444444444444444</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N15" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="O15" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="P15" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="Q15" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="R15" s="13" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
+        <v>104492</v>
+      </c>
+      <c r="B16" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N16" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="O16" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="P16" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q16" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="R16" s="13" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>104395</v>
+      </c>
+      <c r="B17" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.625</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N17" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="O17" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P17" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="R17" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>105073</v>
+      </c>
+      <c r="B18" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.62847222222222221</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="O18" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="R18" s="13" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>105595</v>
+      </c>
+      <c r="B19" s="5">
+        <v>46237</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M19" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N19" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="O19" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="P19" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q19" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="R19" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R3" r:id="rId1" xr:uid="{059A838D-B7D5-4590-915D-C34822A16248}"/>
+    <hyperlink ref="R2" r:id="rId1" xr:uid="{76CF7C19-890C-4BFC-B161-BE23385ACD87}"/>
+    <hyperlink ref="R3" r:id="rId2" display="https://trt15-jus-br.zoom.us/j/87555371032?pwd=ckVSVmpnMHBpcnhHQUZzd0VtT0JBUT09%20%20%20ID%20DA%20REUNIÃO:%20875%205537%201032%20SENHA%20DE%20ACESSO:%20772981" xr:uid="{C113F32D-984C-4AD8-84D8-4732C3D4F859}"/>
+    <hyperlink ref="R5" r:id="rId3" display="https://trt2-jus-br.zoom.us/j/87319779344?pwd=XGh65AWoaNQktqbDH9bXKlU0RqZckb.1%20ID%20da%20reunião:%20873%201977%209344%20Senha%20de%20acesso:%20863962" xr:uid="{7B009CB1-FD0F-413D-AE50-F30846EBF341}"/>
+    <hyperlink ref="R7" r:id="rId4" xr:uid="{F5F85478-D20B-42D0-ADC0-19E0770A71E9}"/>
+    <hyperlink ref="R8" r:id="rId5" display="https://trt4-jus-br.zoom.us/my/cejusc.revista.sala3 ID da reunião:  286 582 7324" xr:uid="{34A7DEC5-B07C-4753-A27D-D57801DC4C6F}"/>
+    <hyperlink ref="R14" r:id="rId6" xr:uid="{598873CA-A701-4F81-8CB6-BA99895D67A0}"/>
+    <hyperlink ref="R15" r:id="rId7" xr:uid="{111EEB3A-AF07-45FB-B1B7-3653CDEB97B1}"/>
+    <hyperlink ref="R16" r:id="rId8" xr:uid="{35FA42D5-58FB-4F76-A032-4F8C4510EDE0}"/>
+    <hyperlink ref="R17" r:id="rId9" display="https://trt2-jus-br.zoom.us/j/81939223002?pwd=VbNbYIp6i5iFsvbFRWAbpt9hdRmaMd.1%20ID%20da%20reunião:%20819%203922%203002%20Senha%20de%20acesso:%20958620" xr:uid="{D753409F-7EB8-48B7-A0CF-9BD9EF444450}"/>
+    <hyperlink ref="R18" r:id="rId10" display="https://trt15-jus-br.zoom.us/j/81582489033?pwd=WFBLcGVJNkJMaWQ2Y3JqZ3d6YjIydz09%20ID%20da%20reunião:%20815%20824%209033%20Senha:%201234" xr:uid="{C6402A31-C826-4F2D-B6E5-DFC37CB77D80}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Audiências: sync 2026-08-03 — 18 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="103">
   <si>
     <t>data</t>
   </si>
@@ -49,94 +49,280 @@
     <t>horario</t>
   </si>
   <si>
-    <t>Fatal</t>
+    <t>D-1</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>MBF</t>
   </si>
   <si>
     <t>JPE</t>
   </si>
   <si>
-    <t>VSI</t>
+    <t>LMI</t>
+  </si>
+  <si>
+    <t>RFE</t>
+  </si>
+  <si>
+    <t>ECO</t>
+  </si>
+  <si>
+    <t>Correspondente - Jaeger</t>
   </si>
   <si>
     <t>Correspondente - Hebert</t>
   </si>
   <si>
-    <t>LMI</t>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>ALF</t>
+  </si>
+  <si>
+    <t>TFR</t>
+  </si>
+  <si>
+    <t>JNE</t>
+  </si>
+  <si>
+    <t>ANB</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
   </si>
   <si>
     <t>Grupo B1</t>
   </si>
   <si>
+    <t>Grupo B3</t>
+  </si>
+  <si>
     <t>Grupo C</t>
   </si>
   <si>
-    <t>Grupo B3</t>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>Sistenge Construcoes E Comercio Ltda</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
   </si>
   <si>
     <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
   </si>
   <si>
-    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
+    <t>Companhia Brasileira De Cartuchos</t>
+  </si>
+  <si>
+    <t>Uhe São Simão Energia S.A.</t>
+  </si>
+  <si>
+    <t>Mitre Realty Empreendimentos E Participacoes Ltda.</t>
   </si>
   <si>
     <t>Cbc - Companhia Brasileira De Cartuchos</t>
   </si>
   <si>
-    <t>Companhia Brasileira De Cartuchos</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Presencial</t>
+    <t>Frutal Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Dell Computadores Do Brasil Ltda</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Monteverde</t>
+  </si>
+  <si>
+    <t>Telefonica Brasil S.A.</t>
+  </si>
+  <si>
+    <t>Viterra Bioenergia S.A</t>
+  </si>
+  <si>
+    <t>T4F Entretenimento S.A.</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Presencial</t>
   </si>
   <si>
     <t>Audiência Una - Telepresencial</t>
   </si>
   <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>1000058-52.2026.5.02.0435</t>
-  </si>
-  <si>
-    <t>0000074-09.2026.5.21.0010</t>
-  </si>
-  <si>
-    <t>1000586-95.2026.5.02.0432</t>
-  </si>
-  <si>
-    <t>1000303-38.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>1000859-40.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Anilton De Sa Silva</t>
-  </si>
-  <si>
-    <t>Everton Muller Da Costa Maia</t>
-  </si>
-  <si>
-    <t>Vagner Aparecido Da Silva</t>
-  </si>
-  <si>
-    <t>Mariane Paulino Dos Santos Alves</t>
-  </si>
-  <si>
-    <t>Elismar Pereira De Jesus Brito</t>
-  </si>
-  <si>
-    <t>08:40:00</t>
+    <t>0011284-81.2026.5.03.0164</t>
+  </si>
+  <si>
+    <t>0011650-59.2026.5.15.0044</t>
+  </si>
+  <si>
+    <t>1001261-61.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>1001249-53.2025.5.02.0020</t>
+  </si>
+  <si>
+    <t>1000659-67.2026.5.02.0432</t>
+  </si>
+  <si>
+    <t>0000031-87.2026.5.18.0129</t>
+  </si>
+  <si>
+    <t>0020030-93.2024.5.04.0029</t>
+  </si>
+  <si>
+    <t>1001341-13.2026.5.02.0435</t>
+  </si>
+  <si>
+    <t>1000939-53.2026.5.02.0039</t>
+  </si>
+  <si>
+    <t>1000858-55.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>1000815-21.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>1000864-62.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>0010612-97.2026.5.03.0156</t>
+  </si>
+  <si>
+    <t>0012826-11.2024.5.15.0152</t>
+  </si>
+  <si>
+    <t>0024175-55.2026.5.24.0066</t>
+  </si>
+  <si>
+    <t>1001486-47.2025.5.02.0001</t>
+  </si>
+  <si>
+    <t>0010653-93.2026.5.15.0103</t>
+  </si>
+  <si>
+    <t>1001114-58.2026.5.02.0003</t>
+  </si>
+  <si>
+    <t>Marionsergio Campos Cabral</t>
+  </si>
+  <si>
+    <t>Antonio Carlos Espejo</t>
+  </si>
+  <si>
+    <t>Potira Brunhera</t>
+  </si>
+  <si>
+    <t>Cleivan Oliveira Amorim</t>
+  </si>
+  <si>
+    <t>Jose Roberto Lopes Da Silva</t>
+  </si>
+  <si>
+    <t>Wigor Paulo Saturno Fernandes</t>
+  </si>
+  <si>
+    <t>Francisco Boaventura Teixeira Moreira</t>
+  </si>
+  <si>
+    <t>Nilson Ignacio</t>
+  </si>
+  <si>
+    <t>Aparecida Ferreira Da Silva Mendes</t>
+  </si>
+  <si>
+    <t>Marco Antonio Ferreira De Moura</t>
+  </si>
+  <si>
+    <t>Maikon Flavio Gomes Dos Santos</t>
+  </si>
+  <si>
+    <t>Silene Antonia Silva De Lima</t>
+  </si>
+  <si>
+    <t>Fernanda De Jesus Martins</t>
+  </si>
+  <si>
+    <t>Rafael Reboucas Dos Santos</t>
+  </si>
+  <si>
+    <t>Dionaty Sousa Dos Santos</t>
+  </si>
+  <si>
+    <t>Luciene Vicentina Pereira Barros</t>
+  </si>
+  <si>
+    <t>Marcelo Aparecido Da Silva</t>
+  </si>
+  <si>
+    <t>Luiz Carlos Vieira De Jesus</t>
+  </si>
+  <si>
+    <t>08:10:00</t>
+  </si>
+  <si>
+    <t>08:35:00</t>
   </si>
   <si>
     <t>09:00:00</t>
   </si>
   <si>
-    <t>10:05:00</t>
-  </si>
-  <si>
-    <t>10:40:00</t>
+    <t>09:30:00</t>
+  </si>
+  <si>
+    <t>09:35:00</t>
+  </si>
+  <si>
+    <t>10:00:00</t>
+  </si>
+  <si>
+    <t>10:45:00</t>
+  </si>
+  <si>
+    <t>11:00:00</t>
+  </si>
+  <si>
+    <t>11:35:00</t>
   </si>
   <si>
     <t>12:05:00</t>
+  </si>
+  <si>
+    <t>12:20:00</t>
+  </si>
+  <si>
+    <t>13:55:00</t>
+  </si>
+  <si>
+    <t>14:16:00</t>
+  </si>
+  <si>
+    <t>14:45:00</t>
+  </si>
+  <si>
+    <t>15:00:00</t>
+  </si>
+  <si>
+    <t>15:05:00</t>
+  </si>
+  <si>
+    <t>16:00:00</t>
   </si>
 </sst>
 </file>
@@ -472,7 +658,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -512,7 +698,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="1">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -521,33 +707,33 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="H2" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="I2" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="K2" t="s">
-        <v>36</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="1">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
@@ -556,33 +742,33 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="G3" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="H3" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="I3" t="s">
-        <v>32</v>
+        <v>69</v>
       </c>
       <c r="J3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="K3" t="s">
-        <v>37</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="1">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
@@ -591,33 +777,33 @@
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G4" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="I4" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="K4" t="s">
-        <v>38</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="1">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
@@ -626,63 +812,518 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="G5" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="H5" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="I5" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="J5" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="K5" t="s">
-        <v>39</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
       <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" t="s">
+        <v>45</v>
+      </c>
+      <c r="H6" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" t="s">
+        <v>72</v>
+      </c>
+      <c r="J6" t="s">
+        <v>32</v>
+      </c>
+      <c r="K6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I7" t="s">
+        <v>73</v>
+      </c>
+      <c r="J7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H8" t="s">
+        <v>56</v>
+      </c>
+      <c r="I8" t="s">
+        <v>74</v>
+      </c>
+      <c r="J8" t="s">
+        <v>33</v>
+      </c>
+      <c r="K8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" t="s">
+        <v>48</v>
+      </c>
+      <c r="H9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I9" t="s">
+        <v>75</v>
+      </c>
+      <c r="J9" t="s">
+        <v>32</v>
+      </c>
+      <c r="K9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" t="s">
+        <v>45</v>
+      </c>
+      <c r="H10" t="s">
+        <v>58</v>
+      </c>
+      <c r="I10" t="s">
+        <v>76</v>
+      </c>
+      <c r="J10" t="s">
+        <v>35</v>
+      </c>
+      <c r="K10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
         <v>15</v>
       </c>
-      <c r="D6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="D11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" t="s">
+        <v>45</v>
+      </c>
+      <c r="H11" t="s">
+        <v>59</v>
+      </c>
+      <c r="I11" t="s">
+        <v>77</v>
+      </c>
+      <c r="J11" t="s">
+        <v>36</v>
+      </c>
+      <c r="K11" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" t="s">
+        <v>45</v>
+      </c>
+      <c r="H12" t="s">
+        <v>60</v>
+      </c>
+      <c r="I12" t="s">
+        <v>78</v>
+      </c>
+      <c r="J12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K12" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" t="s">
+        <v>48</v>
+      </c>
+      <c r="G13" t="s">
+        <v>48</v>
+      </c>
+      <c r="H13" t="s">
+        <v>61</v>
+      </c>
+      <c r="I13" t="s">
+        <v>79</v>
+      </c>
+      <c r="J13" t="s">
+        <v>33</v>
+      </c>
+      <c r="K13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" t="s">
+        <v>43</v>
+      </c>
+      <c r="H14" t="s">
+        <v>62</v>
+      </c>
+      <c r="I14" t="s">
+        <v>80</v>
+      </c>
+      <c r="J14" t="s">
+        <v>37</v>
+      </c>
+      <c r="K14" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" t="s">
+        <v>47</v>
+      </c>
+      <c r="G15" t="s">
+        <v>47</v>
+      </c>
+      <c r="H15" t="s">
+        <v>63</v>
+      </c>
+      <c r="I15" t="s">
+        <v>81</v>
+      </c>
+      <c r="J15" t="s">
+        <v>38</v>
+      </c>
+      <c r="K15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" t="s">
+        <v>39</v>
+      </c>
+      <c r="F16" t="s">
+        <v>49</v>
+      </c>
+      <c r="G16" t="s">
+        <v>49</v>
+      </c>
+      <c r="H16" t="s">
+        <v>64</v>
+      </c>
+      <c r="I16" t="s">
+        <v>82</v>
+      </c>
+      <c r="J16" t="s">
+        <v>39</v>
+      </c>
+      <c r="K16" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s">
         <v>22</v>
       </c>
-      <c r="F6" t="s">
+      <c r="D17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17" t="s">
+        <v>47</v>
+      </c>
+      <c r="H17" t="s">
+        <v>65</v>
+      </c>
+      <c r="I17" t="s">
+        <v>83</v>
+      </c>
+      <c r="J17" t="s">
+        <v>40</v>
+      </c>
+      <c r="K17" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" t="s">
         <v>25</v>
       </c>
-      <c r="G6" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6" t="s">
-        <v>30</v>
-      </c>
-      <c r="I6" t="s">
-        <v>35</v>
-      </c>
-      <c r="J6" t="s">
-        <v>22</v>
-      </c>
-      <c r="K6" t="s">
-        <v>40</v>
+      <c r="E18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" t="s">
+        <v>44</v>
+      </c>
+      <c r="G18" t="s">
+        <v>44</v>
+      </c>
+      <c r="H18" t="s">
+        <v>66</v>
+      </c>
+      <c r="I18" t="s">
+        <v>84</v>
+      </c>
+      <c r="J18" t="s">
+        <v>41</v>
+      </c>
+      <c r="K18" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" t="s">
+        <v>42</v>
+      </c>
+      <c r="F19" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19" t="s">
+        <v>45</v>
+      </c>
+      <c r="H19" t="s">
+        <v>67</v>
+      </c>
+      <c r="I19" t="s">
+        <v>85</v>
+      </c>
+      <c r="J19" t="s">
+        <v>42</v>
+      </c>
+      <c r="K19" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Audiências: sync 2026-08-04 — 32 registros
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="160">
   <si>
     <t>data</t>
   </si>
@@ -52,277 +52,448 @@
     <t>D-1</t>
   </si>
   <si>
+    <t>TAM</t>
+  </si>
+  <si>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>JNE</t>
+  </si>
+  <si>
+    <t>ACA</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>JPL</t>
+  </si>
+  <si>
+    <t>ANB</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>DPR</t>
+  </si>
+  <si>
+    <t>RRU</t>
+  </si>
+  <si>
+    <t>CAL</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>Correspondente - Ana</t>
+  </si>
+  <si>
+    <t>VCR</t>
+  </si>
+  <si>
+    <t>TFR</t>
+  </si>
+  <si>
+    <t>BSO</t>
+  </si>
+  <si>
+    <t>VRO</t>
+  </si>
+  <si>
+    <t>ECO</t>
+  </si>
+  <si>
+    <t>JQS</t>
+  </si>
+  <si>
     <t>RYL</t>
   </si>
   <si>
-    <t>MBF</t>
-  </si>
-  <si>
-    <t>JPE</t>
-  </si>
-  <si>
-    <t>LMI</t>
-  </si>
-  <si>
-    <t>RFE</t>
-  </si>
-  <si>
-    <t>ECO</t>
-  </si>
-  <si>
-    <t>Correspondente - Jaeger</t>
-  </si>
-  <si>
-    <t>Correspondente - Hebert</t>
-  </si>
-  <si>
-    <t>ARC</t>
-  </si>
-  <si>
-    <t>ALF</t>
-  </si>
-  <si>
-    <t>TFR</t>
-  </si>
-  <si>
-    <t>JNE</t>
-  </si>
-  <si>
-    <t>ANB</t>
+    <t>RCF</t>
+  </si>
+  <si>
+    <t>BCF</t>
+  </si>
+  <si>
+    <t>Grupo B1</t>
   </si>
   <si>
     <t>Grupo E2</t>
   </si>
   <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>Grupo B3</t>
-  </si>
-  <si>
     <t>Grupo C</t>
   </si>
   <si>
     <t>Grupo E1</t>
   </si>
   <si>
-    <t>Sistenge Construcoes E Comercio Ltda</t>
+    <t>Grupo D1</t>
+  </si>
+  <si>
+    <t>Grupo B2</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
   </si>
   <si>
     <t>Moema Bioenergia S.A. - Moema</t>
   </si>
   <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Companhia Brasileira De Cartuchos</t>
-  </si>
-  <si>
-    <t>Uhe São Simão Energia S.A.</t>
-  </si>
-  <si>
-    <t>Mitre Realty Empreendimentos E Participacoes Ltda.</t>
-  </si>
-  <si>
-    <t>Cbc - Companhia Brasileira De Cartuchos</t>
-  </si>
-  <si>
-    <t>Frutal Bioenergia Ltda.</t>
-  </si>
-  <si>
-    <t>Dell Computadores Do Brasil Ltda</t>
-  </si>
-  <si>
-    <t>Moema Bioenergia S.A. - Monteverde</t>
+    <t>Sistenge Construções E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Rio Paranapanema Energia S.A.</t>
+  </si>
+  <si>
+    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
+  </si>
+  <si>
+    <t>Syngenta Seeds Ltda.</t>
+  </si>
+  <si>
+    <t>Bit Services Inovação E Tecnologia Ltda.</t>
+  </si>
+  <si>
+    <t>Syngenta Seeds Ltda</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda.</t>
+  </si>
+  <si>
+    <t>Salitre Fertilzantes Ltda</t>
+  </si>
+  <si>
+    <t>Mahle Metal Leve S.A.</t>
+  </si>
+  <si>
+    <t>Embraer S.A.</t>
+  </si>
+  <si>
+    <t>Joanilson Nunes De Oliveira</t>
   </si>
   <si>
     <t>Telefonica Brasil S.A.</t>
   </si>
   <si>
-    <t>Viterra Bioenergia S.A</t>
-  </si>
-  <si>
-    <t>T4F Entretenimento S.A.</t>
+    <t>Eurochem Comercio De Produtos Quimicos Ltda.</t>
+  </si>
+  <si>
+    <t>Direct Express Logística Integrada S.A.</t>
+  </si>
+  <si>
+    <t>Viterra Bioenergia S.A.</t>
+  </si>
+  <si>
+    <t>International Paper Do Brasil Ltda.</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
   </si>
   <si>
     <t>Audiência Inicial -  Telepresencial</t>
   </si>
   <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Una- Telepresencial</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TST - Presencial</t>
+  </si>
+  <si>
     <t>Audiência Inicial - Telepresencial</t>
   </si>
   <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
     <t>Audiência Una - Presencial</t>
   </si>
   <si>
     <t>Audiência Instrução - Telepresencial</t>
   </si>
   <si>
-    <t>Audiência de Conciliação - Telepresencial</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Presencial</t>
+    <t>Audiência de Instrução - Semipresencial</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Presencial</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Semipresencial</t>
   </si>
   <si>
     <t>Audiência Una - Telepresencial</t>
   </si>
   <si>
-    <t>0011284-81.2026.5.03.0164</t>
-  </si>
-  <si>
-    <t>0011650-59.2026.5.15.0044</t>
-  </si>
-  <si>
-    <t>1001261-61.2026.5.02.0431</t>
-  </si>
-  <si>
-    <t>1001249-53.2025.5.02.0020</t>
-  </si>
-  <si>
-    <t>1000659-67.2026.5.02.0432</t>
-  </si>
-  <si>
-    <t>0000031-87.2026.5.18.0129</t>
-  </si>
-  <si>
-    <t>0020030-93.2024.5.04.0029</t>
-  </si>
-  <si>
-    <t>1001341-13.2026.5.02.0435</t>
-  </si>
-  <si>
-    <t>1000939-53.2026.5.02.0039</t>
-  </si>
-  <si>
-    <t>1000858-55.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>1000815-21.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>1000864-62.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>0010612-97.2026.5.03.0156</t>
-  </si>
-  <si>
-    <t>0012826-11.2024.5.15.0152</t>
-  </si>
-  <si>
-    <t>0024175-55.2026.5.24.0066</t>
-  </si>
-  <si>
-    <t>1001486-47.2025.5.02.0001</t>
-  </si>
-  <si>
-    <t>0010653-93.2026.5.15.0103</t>
-  </si>
-  <si>
-    <t>1001114-58.2026.5.02.0003</t>
-  </si>
-  <si>
-    <t>Marionsergio Campos Cabral</t>
-  </si>
-  <si>
-    <t>Antonio Carlos Espejo</t>
-  </si>
-  <si>
-    <t>Potira Brunhera</t>
-  </si>
-  <si>
-    <t>Cleivan Oliveira Amorim</t>
-  </si>
-  <si>
-    <t>Jose Roberto Lopes Da Silva</t>
-  </si>
-  <si>
-    <t>Wigor Paulo Saturno Fernandes</t>
-  </si>
-  <si>
-    <t>Francisco Boaventura Teixeira Moreira</t>
-  </si>
-  <si>
-    <t>Nilson Ignacio</t>
-  </si>
-  <si>
-    <t>Aparecida Ferreira Da Silva Mendes</t>
-  </si>
-  <si>
-    <t>Marco Antonio Ferreira De Moura</t>
-  </si>
-  <si>
-    <t>Maikon Flavio Gomes Dos Santos</t>
-  </si>
-  <si>
-    <t>Silene Antonia Silva De Lima</t>
-  </si>
-  <si>
-    <t>Fernanda De Jesus Martins</t>
-  </si>
-  <si>
-    <t>Rafael Reboucas Dos Santos</t>
-  </si>
-  <si>
-    <t>Dionaty Sousa Dos Santos</t>
-  </si>
-  <si>
-    <t>Luciene Vicentina Pereira Barros</t>
-  </si>
-  <si>
-    <t>Marcelo Aparecido Da Silva</t>
-  </si>
-  <si>
-    <t>Luiz Carlos Vieira De Jesus</t>
-  </si>
-  <si>
-    <t>08:10:00</t>
-  </si>
-  <si>
-    <t>08:35:00</t>
+    <t>0012545-86.2025.5.15.0001</t>
+  </si>
+  <si>
+    <t>1001866-53.2025.5.02.0039</t>
+  </si>
+  <si>
+    <t>0010484-64.2026.5.03.0031</t>
+  </si>
+  <si>
+    <t>0011099-48.2016.5.15.0103</t>
+  </si>
+  <si>
+    <t>0000167-80.2026.5.09.0567</t>
+  </si>
+  <si>
+    <t>0010782-28.2024.5.03.0063</t>
+  </si>
+  <si>
+    <t>1000297-47.2026.5.02.0050</t>
+  </si>
+  <si>
+    <t>0011509-40.2026.5.15.0044</t>
+  </si>
+  <si>
+    <t>0010703-78.2026.5.03.0063</t>
+  </si>
+  <si>
+    <t>0000355-16.2025.5.05.0019</t>
+  </si>
+  <si>
+    <t>0010751-83.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>1000773-09.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>0012465-43.2024.5.15.0071</t>
+  </si>
+  <si>
+    <t>0011744-39.2023.5.15.0132</t>
+  </si>
+  <si>
+    <t>1002067-85.2025.5.02.0058</t>
+  </si>
+  <si>
+    <t>1000911-89.2026.5.02.0361</t>
+  </si>
+  <si>
+    <t>0001705-27.2025.5.09.0084</t>
+  </si>
+  <si>
+    <t>0010290-14.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>1000623-26.2026.5.02.0464</t>
+  </si>
+  <si>
+    <t>1000152-53.2023.5.02.0613</t>
+  </si>
+  <si>
+    <t>0010226-04.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>0001578-56.2025.5.09.0095</t>
+  </si>
+  <si>
+    <t>0011022-49.2025.5.15.0030</t>
+  </si>
+  <si>
+    <t>1001126-80.2017.5.02.0361</t>
+  </si>
+  <si>
+    <t>0010416-24.2026.5.15.0050</t>
+  </si>
+  <si>
+    <t>0107600-10.2009.5.15.0071</t>
+  </si>
+  <si>
+    <t>0010376-28.2024.5.15.0045</t>
+  </si>
+  <si>
+    <t>1000407-97.2022.5.02.0434</t>
+  </si>
+  <si>
+    <t>0010054-22.2026.5.15.0050</t>
+  </si>
+  <si>
+    <t>0012301-55.2025.5.15.0132</t>
+  </si>
+  <si>
+    <t>0010344-23.2026.5.15.0087</t>
+  </si>
+  <si>
+    <t>Marcos De Faria Paes</t>
+  </si>
+  <si>
+    <t>Cleber Donizeti Da Trindade</t>
+  </si>
+  <si>
+    <t>Kaio Rodrigo Goncalves Da Cruz</t>
+  </si>
+  <si>
+    <t>Luiz Antonio Goncalves</t>
+  </si>
+  <si>
+    <t>Claudemir Mendonca</t>
+  </si>
+  <si>
+    <t>Carlos Fernando Santos Silva</t>
+  </si>
+  <si>
+    <t>Marcelo Bertossi Barbosa</t>
+  </si>
+  <si>
+    <t>Moises De Aguiar Caires</t>
+  </si>
+  <si>
+    <t>Robert Da Silva Vilela</t>
+  </si>
+  <si>
+    <t>Denilson Dos Santos</t>
+  </si>
+  <si>
+    <t>Wellinthon Dos Reis Garajau</t>
+  </si>
+  <si>
+    <t>Jonathan Wanus Batista Santos</t>
+  </si>
+  <si>
+    <t>Horlando Cicero Da Silva</t>
+  </si>
+  <si>
+    <t>Lucas Moreira Fabricio</t>
+  </si>
+  <si>
+    <t>Rafael Vinicius Campioto</t>
+  </si>
+  <si>
+    <t>Jose Leite De Sousa</t>
+  </si>
+  <si>
+    <t>Pedro Lopes Barboza</t>
+  </si>
+  <si>
+    <t>Joao Marcos Pereira De Souza</t>
+  </si>
+  <si>
+    <t>Darcisio Campos Da Cruz</t>
+  </si>
+  <si>
+    <t>Edson De Lima Solla</t>
+  </si>
+  <si>
+    <t>Wesley Fernando Araujo</t>
+  </si>
+  <si>
+    <t>Allan Ferreira Silva</t>
+  </si>
+  <si>
+    <t>Sara Beatriz Correa De Andrade</t>
+  </si>
+  <si>
+    <t>Thiago Rodrigues Da Silva</t>
+  </si>
+  <si>
+    <t>Luis Antonio Pedro</t>
+  </si>
+  <si>
+    <t>Ministério Público Do Trabalho</t>
+  </si>
+  <si>
+    <t>Anderson Rodrigo Da Costa</t>
+  </si>
+  <si>
+    <t>Cleiton Goncalves Ferreira</t>
+  </si>
+  <si>
+    <t>Edson Aparecido Arf</t>
+  </si>
+  <si>
+    <t>Anderson Izidoro Dos Santos</t>
+  </si>
+  <si>
+    <t>Reginaldo Rodrigues Da Silva</t>
+  </si>
+  <si>
+    <t>08:40:00</t>
+  </si>
+  <si>
+    <t>08:50:00</t>
+  </si>
+  <si>
+    <t>08:55:00</t>
   </si>
   <si>
     <t>09:00:00</t>
   </si>
   <si>
+    <t>09:10:00</t>
+  </si>
+  <si>
+    <t>09:20:00</t>
+  </si>
+  <si>
     <t>09:30:00</t>
   </si>
   <si>
-    <t>09:35:00</t>
+    <t>09:31:00</t>
   </si>
   <si>
     <t>10:00:00</t>
   </si>
   <si>
-    <t>10:45:00</t>
+    <t>10:05:00</t>
+  </si>
+  <si>
+    <t>10:20:00</t>
+  </si>
+  <si>
+    <t>10:30:00</t>
+  </si>
+  <si>
+    <t>10:40:00</t>
   </si>
   <si>
     <t>11:00:00</t>
   </si>
   <si>
-    <t>11:35:00</t>
-  </si>
-  <si>
-    <t>12:05:00</t>
-  </si>
-  <si>
-    <t>12:20:00</t>
-  </si>
-  <si>
-    <t>13:55:00</t>
-  </si>
-  <si>
-    <t>14:16:00</t>
+    <t>11:10:00</t>
+  </si>
+  <si>
+    <t>11:30:00</t>
+  </si>
+  <si>
+    <t>11:55:00</t>
+  </si>
+  <si>
+    <t>13:00:00</t>
+  </si>
+  <si>
+    <t>13:30:00</t>
+  </si>
+  <si>
+    <t>13:44:00</t>
+  </si>
+  <si>
+    <t>14:00:00</t>
+  </si>
+  <si>
+    <t>14:09:00</t>
+  </si>
+  <si>
+    <t>14:22:00</t>
+  </si>
+  <si>
+    <t>14:30:00</t>
   </si>
   <si>
     <t>14:45:00</t>
   </si>
   <si>
-    <t>15:00:00</t>
-  </si>
-  <si>
-    <t>15:05:00</t>
-  </si>
-  <si>
-    <t>16:00:00</t>
+    <t>14:50:00</t>
   </si>
 </sst>
 </file>
@@ -658,7 +829,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -698,7 +869,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -707,33 +878,33 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F2" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="G2" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="H2" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="I2" t="s">
-        <v>68</v>
+        <v>103</v>
       </c>
       <c r="J2" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K2" t="s">
-        <v>86</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
@@ -742,33 +913,33 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E3" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="F3" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="H3" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="J3" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="K3" t="s">
-        <v>87</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
@@ -777,33 +948,33 @@
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="F4" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="G4" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="H4" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="I4" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="J4" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="K4" t="s">
-        <v>88</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
@@ -812,33 +983,33 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F5" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="G5" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="H5" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="I5" t="s">
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="J5" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="K5" t="s">
-        <v>89</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
@@ -847,33 +1018,33 @@
         <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="G6" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="H6" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="I6" t="s">
-        <v>72</v>
+        <v>107</v>
       </c>
       <c r="J6" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="K6" t="s">
-        <v>90</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
@@ -882,33 +1053,33 @@
         <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="G7" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="I7" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="J7" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="K7" t="s">
-        <v>91</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B8" t="s">
         <v>11</v>
@@ -917,33 +1088,33 @@
         <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="E8" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="F8" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="H8" t="s">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="I8" t="s">
-        <v>74</v>
+        <v>109</v>
       </c>
       <c r="J8" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="K8" t="s">
-        <v>92</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
@@ -952,33 +1123,33 @@
         <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="F9" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="G9" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="I9" t="s">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="J9" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="K9" t="s">
-        <v>93</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
@@ -987,343 +1158,833 @@
         <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="F10" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="G10" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="H10" t="s">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="I10" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="J10" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="K10" t="s">
-        <v>93</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F11" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="G11" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="H11" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="I11" t="s">
-        <v>77</v>
+        <v>112</v>
       </c>
       <c r="J11" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="K11" t="s">
-        <v>94</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B12" t="s">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E12" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="F12" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="G12" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="H12" t="s">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="I12" t="s">
-        <v>78</v>
+        <v>113</v>
       </c>
       <c r="J12" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="K12" t="s">
-        <v>95</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="E13" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="F13" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="G13" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="H13" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="I13" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="J13" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="K13" t="s">
-        <v>96</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="D14" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="E14" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="F14" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="G14" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="H14" t="s">
-        <v>62</v>
+        <v>84</v>
       </c>
       <c r="I14" t="s">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="J14" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="K14" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B15" t="s">
         <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D15" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F15" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="G15" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="H15" t="s">
-        <v>63</v>
+        <v>85</v>
       </c>
       <c r="I15" t="s">
-        <v>81</v>
+        <v>116</v>
       </c>
       <c r="J15" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="K15" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B16" t="s">
         <v>11</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="D16" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="E16" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="F16" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="G16" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="H16" t="s">
-        <v>64</v>
+        <v>85</v>
       </c>
       <c r="I16" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="J16" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="K16" t="s">
-        <v>99</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B17" t="s">
         <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="E17" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="F17" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="G17" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="H17" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="I17" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="J17" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="K17" t="s">
-        <v>100</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B18" t="s">
         <v>11</v>
       </c>
       <c r="C18" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D18" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F18" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="G18" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="H18" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="I18" t="s">
-        <v>84</v>
+        <v>118</v>
       </c>
       <c r="J18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K18" t="s">
-        <v>101</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B19" t="s">
         <v>11</v>
       </c>
       <c r="C19" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D19" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="E19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F19" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="G19" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="H19" t="s">
+        <v>88</v>
+      </c>
+      <c r="I19" t="s">
+        <v>119</v>
+      </c>
+      <c r="J19" t="s">
+        <v>44</v>
+      </c>
+      <c r="K19" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" t="s">
+        <v>66</v>
+      </c>
+      <c r="G20" t="s">
+        <v>66</v>
+      </c>
+      <c r="H20" t="s">
+        <v>89</v>
+      </c>
+      <c r="I20" t="s">
+        <v>120</v>
+      </c>
+      <c r="J20" t="s">
+        <v>48</v>
+      </c>
+      <c r="K20" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" t="s">
+        <v>37</v>
+      </c>
+      <c r="E21" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" t="s">
+        <v>65</v>
+      </c>
+      <c r="G21" t="s">
+        <v>65</v>
+      </c>
+      <c r="H21" t="s">
+        <v>90</v>
+      </c>
+      <c r="I21" t="s">
+        <v>121</v>
+      </c>
+      <c r="J21" t="s">
+        <v>50</v>
+      </c>
+      <c r="K21" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" t="s">
+        <v>68</v>
+      </c>
+      <c r="G22" t="s">
+        <v>68</v>
+      </c>
+      <c r="H22" t="s">
+        <v>91</v>
+      </c>
+      <c r="I22" t="s">
+        <v>122</v>
+      </c>
+      <c r="J22" t="s">
+        <v>53</v>
+      </c>
+      <c r="K22" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B23" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" t="s">
+        <v>35</v>
+      </c>
+      <c r="E23" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" t="s">
+        <v>66</v>
+      </c>
+      <c r="G23" t="s">
+        <v>66</v>
+      </c>
+      <c r="H23" t="s">
+        <v>92</v>
+      </c>
+      <c r="I23" t="s">
+        <v>123</v>
+      </c>
+      <c r="J23" t="s">
+        <v>48</v>
+      </c>
+      <c r="K23" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24" t="s">
+        <v>44</v>
+      </c>
+      <c r="F24" t="s">
         <v>67</v>
       </c>
-      <c r="I19" t="s">
-        <v>85</v>
-      </c>
-      <c r="J19" t="s">
-        <v>42</v>
-      </c>
-      <c r="K19" t="s">
+      <c r="G24" t="s">
+        <v>67</v>
+      </c>
+      <c r="H24" t="s">
+        <v>93</v>
+      </c>
+      <c r="I24" t="s">
+        <v>124</v>
+      </c>
+      <c r="J24" t="s">
+        <v>44</v>
+      </c>
+      <c r="K24" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" t="s">
+        <v>21</v>
+      </c>
+      <c r="D25" t="s">
+        <v>35</v>
+      </c>
+      <c r="E25" t="s">
+        <v>54</v>
+      </c>
+      <c r="F25" t="s">
+        <v>69</v>
+      </c>
+      <c r="G25" t="s">
+        <v>69</v>
+      </c>
+      <c r="H25" t="s">
+        <v>94</v>
+      </c>
+      <c r="I25" t="s">
+        <v>125</v>
+      </c>
+      <c r="J25" t="s">
+        <v>54</v>
+      </c>
+      <c r="K25" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
+      <c r="A26" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B26" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" t="s">
+        <v>30</v>
+      </c>
+      <c r="D26" t="s">
+        <v>38</v>
+      </c>
+      <c r="E26" t="s">
+        <v>55</v>
+      </c>
+      <c r="F26" t="s">
+        <v>64</v>
+      </c>
+      <c r="G26" t="s">
+        <v>64</v>
+      </c>
+      <c r="H26" t="s">
+        <v>95</v>
+      </c>
+      <c r="I26" t="s">
+        <v>126</v>
+      </c>
+      <c r="J26" t="s">
+        <v>55</v>
+      </c>
+      <c r="K26" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B27" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" t="s">
+        <v>31</v>
+      </c>
+      <c r="D27" t="s">
+        <v>35</v>
+      </c>
+      <c r="E27" t="s">
+        <v>56</v>
+      </c>
+      <c r="F27" t="s">
+        <v>61</v>
+      </c>
+      <c r="G27" t="s">
+        <v>61</v>
+      </c>
+      <c r="H27" t="s">
+        <v>96</v>
+      </c>
+      <c r="I27" t="s">
+        <v>127</v>
+      </c>
+      <c r="J27" t="s">
+        <v>56</v>
+      </c>
+      <c r="K27" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
+      <c r="A28" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B28" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" t="s">
+        <v>32</v>
+      </c>
+      <c r="D28" t="s">
+        <v>35</v>
+      </c>
+      <c r="E28" t="s">
+        <v>57</v>
+      </c>
+      <c r="F28" t="s">
+        <v>62</v>
+      </c>
+      <c r="G28" t="s">
+        <v>62</v>
+      </c>
+      <c r="H28" t="s">
+        <v>97</v>
+      </c>
+      <c r="I28" t="s">
+        <v>128</v>
+      </c>
+      <c r="J28" t="s">
+        <v>57</v>
+      </c>
+      <c r="K28" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
+      <c r="A29" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B29" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" t="s">
+        <v>39</v>
+      </c>
+      <c r="E29" t="s">
+        <v>51</v>
+      </c>
+      <c r="F29" t="s">
+        <v>70</v>
+      </c>
+      <c r="G29" t="s">
+        <v>70</v>
+      </c>
+      <c r="H29" t="s">
+        <v>98</v>
+      </c>
+      <c r="I29" t="s">
+        <v>129</v>
+      </c>
+      <c r="J29" t="s">
+        <v>51</v>
+      </c>
+      <c r="K29" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
+      <c r="A30" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B30" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" t="s">
+        <v>23</v>
+      </c>
+      <c r="D30" t="s">
+        <v>34</v>
+      </c>
+      <c r="E30" t="s">
+        <v>40</v>
+      </c>
+      <c r="F30" t="s">
+        <v>64</v>
+      </c>
+      <c r="G30" t="s">
+        <v>64</v>
+      </c>
+      <c r="H30" t="s">
+        <v>99</v>
+      </c>
+      <c r="I30" t="s">
+        <v>130</v>
+      </c>
+      <c r="J30" t="s">
+        <v>40</v>
+      </c>
+      <c r="K30" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
+      <c r="A31" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B31" t="s">
+        <v>11</v>
+      </c>
+      <c r="C31" t="s">
+        <v>31</v>
+      </c>
+      <c r="D31" t="s">
+        <v>35</v>
+      </c>
+      <c r="E31" t="s">
+        <v>56</v>
+      </c>
+      <c r="F31" t="s">
+        <v>71</v>
+      </c>
+      <c r="G31" t="s">
+        <v>71</v>
+      </c>
+      <c r="H31" t="s">
+        <v>100</v>
+      </c>
+      <c r="I31" t="s">
+        <v>131</v>
+      </c>
+      <c r="J31" t="s">
+        <v>56</v>
+      </c>
+      <c r="K31" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11">
+      <c r="A32" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B32" t="s">
+        <v>11</v>
+      </c>
+      <c r="C32" t="s">
+        <v>33</v>
+      </c>
+      <c r="D32" t="s">
+        <v>39</v>
+      </c>
+      <c r="E32" t="s">
+        <v>51</v>
+      </c>
+      <c r="F32" t="s">
+        <v>65</v>
+      </c>
+      <c r="G32" t="s">
+        <v>65</v>
+      </c>
+      <c r="H32" t="s">
+        <v>101</v>
+      </c>
+      <c r="I32" t="s">
+        <v>132</v>
+      </c>
+      <c r="J32" t="s">
+        <v>51</v>
+      </c>
+      <c r="K32" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11">
+      <c r="A33" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B33" t="s">
+        <v>11</v>
+      </c>
+      <c r="C33" t="s">
+        <v>17</v>
+      </c>
+      <c r="D33" t="s">
+        <v>37</v>
+      </c>
+      <c r="E33" t="s">
+        <v>58</v>
+      </c>
+      <c r="F33" t="s">
+        <v>59</v>
+      </c>
+      <c r="G33" t="s">
+        <v>59</v>
+      </c>
+      <c r="H33" t="s">
         <v>102</v>
+      </c>
+      <c r="I33" t="s">
+        <v>133</v>
+      </c>
+      <c r="J33" t="s">
+        <v>58</v>
+      </c>
+      <c r="K33" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Audiências: sync 2026-08-11 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB90DA08-74CA-4237-AA12-6AF6B1CC556C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B05DDE9D-E5F1-4496-AD32-0CE32A04B1CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5887CEB3-535E-43A1-8951-4C0AB082E04F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{ECACBBAE-0407-4536-883E-0345D98247B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,25 +95,25 @@
     <t>Link/Observações</t>
   </si>
   <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>1000593-90.2026.5.02.0431</t>
-  </si>
-  <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Jurandir Pereira Da Silva</t>
-  </si>
-  <si>
-    <t>SANTO ANDRÉ</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>05ª VARA DO TRABALHO</t>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>0010610-42.2026.5.03.0152</t>
+  </si>
+  <si>
+    <t>Santa Juliana Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Everton De Menezes Santos</t>
+  </si>
+  <si>
+    <t>UBERABA</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>03ª VARA DO TRABALHO</t>
   </si>
   <si>
     <t>Instrução</t>
@@ -125,110 +125,26 @@
     <t>CENTRAL</t>
   </si>
   <si>
-    <t>R$             893.529,55</t>
-  </si>
-  <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>JPE</t>
-  </si>
-  <si>
-    <t>GSM</t>
-  </si>
-  <si>
-    <t>Presencial</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>1000759-22.2026.5.02.0432</t>
-  </si>
-  <si>
-    <t>Samuel Sousa Salgado</t>
-  </si>
-  <si>
-    <t>02ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             271.985,81</t>
-  </si>
-  <si>
-    <t>RFE</t>
-  </si>
-  <si>
-    <t>Audiência de Encerramento de Instrução</t>
-  </si>
-  <si>
-    <t>c</t>
-  </si>
-  <si>
-    <t>Itumbiara Bioenergia S.A.</t>
-  </si>
-  <si>
-    <t>Isadora Moscardini Roschel</t>
-  </si>
-  <si>
-    <t>SÃO PAULO</t>
-  </si>
-  <si>
-    <t>22ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$          1.198.073,17</t>
+    <t>R$               83.122,87</t>
   </si>
   <si>
     <t>Grupo E2</t>
   </si>
   <si>
-    <t>ARC</t>
-  </si>
-  <si>
-    <t>Dispensado o comparecimento das partes</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Telepresencial</t>
-  </si>
-  <si>
-    <t>0000916-95.2026.5.10.0009</t>
-  </si>
-  <si>
-    <t>Ferrero Do Brasil Industria Doceira E Alimentar Ltda</t>
-  </si>
-  <si>
-    <t>Jose Carlos Dos Santos Ramos</t>
-  </si>
-  <si>
-    <t>BRASÍLIA</t>
-  </si>
-  <si>
-    <t>DF</t>
-  </si>
-  <si>
-    <t>09ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>1ª Instância</t>
-  </si>
-  <si>
-    <t>R$             630.017,05</t>
-  </si>
-  <si>
-    <t>Grupo B3</t>
-  </si>
-  <si>
-    <t>ANB</t>
-  </si>
-  <si>
-    <t>https://trt10-jus-br.zoom.us/j/2748578818</t>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>JNE</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt3uberaba</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -248,6 +164,14 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -327,10 +251,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -353,8 +278,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -686,30 +615,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C3838E7-10E4-4CBA-967B-D9FFCBE8CB54}">
-  <dimension ref="A1:R5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8489D535-48A6-45C0-9211-4EB3308F96FB}">
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.21875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.88671875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.88671875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="35.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -765,15 +694,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>104579</v>
+        <v>105324</v>
       </c>
       <c r="B2" s="5">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="C2" s="6">
-        <v>0.35416666666666669</v>
+        <v>0.34375</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>18</v>
@@ -817,181 +746,13 @@
       <c r="Q2" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="R2" s="8" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4">
-        <v>104772</v>
-      </c>
-      <c r="B3" s="5">
-        <v>46241</v>
-      </c>
-      <c r="C3" s="6">
-        <v>0.4513888888888889</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="L3" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="M3" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="N3" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="O3" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="P3" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q3" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="R3" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="4">
-        <v>102861</v>
-      </c>
-      <c r="B4" s="5">
-        <v>46241</v>
-      </c>
-      <c r="C4" s="6">
-        <v>0.59027777777777779</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="L4" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="M4" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="N4" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="O4" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="P4" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q4" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="R4" s="7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
-        <v>105612</v>
-      </c>
-      <c r="B5" s="5">
-        <v>46241</v>
-      </c>
-      <c r="C5" s="6">
-        <v>0.66111111111111109</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="P5" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q5" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="R5" s="7" t="s">
-        <v>60</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R5" r:id="rId1" xr:uid="{6BAA673C-60B3-4830-B9B2-BFA693A810EA}"/>
+    <hyperlink ref="R2" r:id="rId1" xr:uid="{E47E0F5C-03E4-4A63-A1AC-7B1AC9FF3CEE}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Audiências: sync 2026-09-01 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://peixotoecuryadv-my.sharepoint.com/personal/blu_peixotoecury_com_br/Documents/Área de Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{83F675F7-239A-4454-8121-5D9A8386F7E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9DDC202D-505B-4DB3-9CC0-97F21ADC752E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{882225A2-E4F3-4ADF-913D-09EB867047ED}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A1CC5714-94CC-4D0C-AD10-3598BE313F79}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="195">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,337 +95,535 @@
     <t>Link/Observações</t>
   </si>
   <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>0010940-21.2025.5.15.0126</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
+  </si>
+  <si>
+    <t>Edvanio Dos Santos Silva</t>
+  </si>
+  <si>
+    <t>PAULÍNIA</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>02ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>1ª Instância</t>
+  </si>
+  <si>
+    <t>Reclamação Trabalhista</t>
+  </si>
+  <si>
+    <t>CENTRAL</t>
+  </si>
+  <si>
+    <t>R$               72.310,02</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>JRM</t>
+  </si>
+  <si>
+    <t>GVM</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/9973700634?pwd=dENDekhCNjFLekRnSExiTzhmK1VLdz09 ID da reunião: 997 370 0634 Senha: 592209</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Semipresencial</t>
+  </si>
+  <si>
+    <t>0012114-81.2024.5.15.0132</t>
+  </si>
+  <si>
+    <t>Embraer S.A.</t>
+  </si>
+  <si>
+    <t>Ronnie Anderson Benedito</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DOS CAMPOS</t>
+  </si>
+  <si>
+    <t>04ª TURMA</t>
+  </si>
+  <si>
+    <t>Recursal TRT</t>
+  </si>
+  <si>
+    <t>R$             671.139,88</t>
+  </si>
+  <si>
+    <t>Grupo B2</t>
+  </si>
+  <si>
+    <t>GSM</t>
+  </si>
+  <si>
+    <t>BCF</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/82717131621?pwd=pODkGMMik6OAPMNpdT855vizOcYdKQ.1 iD da reunião: 827 1713 1621 Senha: 761332</t>
+  </si>
+  <si>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>1000658-10.2026.5.02.0262</t>
+  </si>
+  <si>
+    <t>Msa Do Brasil Equip E Instrumentos De Seguranca Ltda.</t>
+  </si>
+  <si>
+    <t>Sara Francisca Dos Santos</t>
+  </si>
+  <si>
+    <t>SÃO PAULO</t>
+  </si>
+  <si>
+    <t>14ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Instrução</t>
+  </si>
+  <si>
+    <t>R$               42.898,20</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/87449545935?pwd=wCgGe2V8ntb7v8A97BI4itvBX6i0Ya.1 ID da reunião: 874 4954 5935 Senha de acesso: 047941</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>1000978-35.2026.5.02.0432</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Lucas Figueiredo Saturnino</t>
+  </si>
+  <si>
+    <t>SANTO ANDRÉ</t>
+  </si>
+  <si>
+    <t>R$             863.640,00</t>
+  </si>
+  <si>
+    <t>Grupo B1</t>
+  </si>
+  <si>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>Presencial</t>
+  </si>
+  <si>
+    <t>1001287-79.2026.5.02.0004</t>
+  </si>
+  <si>
+    <t>Telefonica Brasil S.A.</t>
+  </si>
+  <si>
+    <t>Marcia Valeria Brandao De Mello Cucco Pereira</t>
+  </si>
+  <si>
+    <t>04ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$          1.958.789,00</t>
+  </si>
+  <si>
+    <t>Grupo C</t>
+  </si>
+  <si>
+    <t>TFR</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/83934068085?pwd=vsilyvu3m7bMldNPplkinUYQRGR2Xz.1 ID da reunião: 839 3406 8085 Senha de acesso: 359721</t>
+  </si>
+  <si>
+    <t>0010417-48.2026.5.03.0048</t>
+  </si>
+  <si>
+    <t>Santa Juliana Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Samuel Henrique Saturnino</t>
+  </si>
+  <si>
+    <t>ITURAMA</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             556.517,03</t>
+  </si>
+  <si>
+    <t>CAL</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt.iturama</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>0011252-18.2025.5.15.0022</t>
+  </si>
+  <si>
+    <t>Mahle Metal Leve S.A.</t>
+  </si>
+  <si>
+    <t>Jailton Aparecido De Souza Senne</t>
+  </si>
+  <si>
+    <t>MOGI MIRIM</t>
+  </si>
+  <si>
+    <t>R$             212.312,95</t>
+  </si>
+  <si>
+    <t>Correspondente - Ana</t>
+  </si>
+  <si>
+    <t>TLI</t>
+  </si>
+  <si>
+    <t>0011298-88.2025.5.15.0092</t>
+  </si>
+  <si>
+    <t>Waldemar Da Silva Filho</t>
+  </si>
+  <si>
+    <t>CAMPINAS</t>
+  </si>
+  <si>
+    <t>05ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             210.000,00</t>
+  </si>
+  <si>
+    <t>Correspondente - Daniela Prandi</t>
+  </si>
+  <si>
+    <t>BSO</t>
+  </si>
+  <si>
     <t>Audiência Inicial -  Telepresencial</t>
   </si>
   <si>
-    <t>0000949-91.2026.5.18.0129</t>
-  </si>
-  <si>
-    <t>Spic Brasil Energia Participacoes S.A.</t>
-  </si>
-  <si>
-    <t>Cosmo Alves Da Silva</t>
-  </si>
-  <si>
-    <t>QUIRINÓPOLIS</t>
-  </si>
-  <si>
-    <t>GO</t>
-  </si>
-  <si>
-    <t>VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Instrução</t>
-  </si>
-  <si>
-    <t>Reclamação Trabalhista</t>
-  </si>
-  <si>
-    <t>CENTRAL</t>
-  </si>
-  <si>
-    <t>R$                       38.688,52</t>
-  </si>
-  <si>
-    <t>Grupo C</t>
+    <t>0000309-08.2026.5.09.0657</t>
+  </si>
+  <si>
+    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
+  </si>
+  <si>
+    <t>Jean Gilbert Dos Santos</t>
+  </si>
+  <si>
+    <t>COLOMBO</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>01ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               73.000,00</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>https://url.trt9.jus.br/xx0w9 ID da reunião: 82127329940 Senha de acesso: W0FBQYvT0q</t>
+  </si>
+  <si>
+    <t>0011763-13.2026.5.15.0044</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Matheus Felipe Januario Domingues</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DO RIO PRETO</t>
+  </si>
+  <si>
+    <t>R$             356.093,25</t>
+  </si>
+  <si>
+    <t>RRU</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/81757243738?pwd=UXAvdEpveHlrNU05M2ZsZnRrYy9Vdz09 ID DA REUNIÃO: 817 5724 3738 SENHA: 954332</t>
+  </si>
+  <si>
+    <t>0010974-59.2026.5.15.0126</t>
+  </si>
+  <si>
+    <t>Ronilson Rodrigues De Souza</t>
+  </si>
+  <si>
+    <t>R$             135.668,67</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/83352065501?pwd=Lzc2WUJGSVpVWmJyZjB3Y0NvUmJPZz09 ID da reunião: 833 5206 5501 Senha de acesso: 368465</t>
+  </si>
+  <si>
+    <t>0010719-78.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda</t>
+  </si>
+  <si>
+    <t>Gleydson Freitas Sousa</t>
+  </si>
+  <si>
+    <t>PATROCÍNIO</t>
+  </si>
+  <si>
+    <t>Conhecimento</t>
+  </si>
+  <si>
+    <t>R$             117.254,25</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt.patrocinio</t>
+  </si>
+  <si>
+    <t>0010708-49.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>Gustavo Martins Montandon</t>
+  </si>
+  <si>
+    <t>R$               70.920,29</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>1000249-72.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>Companhia Brasileira De Cartuchos</t>
+  </si>
+  <si>
+    <t>Eraldo Joao Pimentel</t>
+  </si>
+  <si>
+    <t>RIBEIRÃO PIRES</t>
+  </si>
+  <si>
+    <t>R$             137.570,07</t>
+  </si>
+  <si>
+    <t>Grupo B3</t>
+  </si>
+  <si>
+    <t>LMI</t>
+  </si>
+  <si>
+    <t>1001385-17.2023.5.02.0086</t>
+  </si>
+  <si>
+    <t>Rodrigo Da Silva Pareschi</t>
+  </si>
+  <si>
+    <t>10ª TURMA</t>
+  </si>
+  <si>
+    <t>Recursal</t>
+  </si>
+  <si>
+    <t>R$             240.242,94</t>
   </si>
   <si>
     <t>RCF</t>
   </si>
   <si>
-    <t>ECO</t>
-  </si>
-  <si>
-    <t>https://trt18-jus-br.zoom.us/my/cejuscdigital.manha</t>
-  </si>
-  <si>
-    <t>0000943-84.2026.5.18.0129</t>
-  </si>
-  <si>
-    <t>Jose Carlos Do Nascimento</t>
-  </si>
-  <si>
-    <t>R$                       40.220,45</t>
+    <t>Presencial | https://trt2-jus-br.zoom.us/j/89651014670?pwd=FW0AFzyGa5XXc5LOiaXNalueDYjcGW.1 ID da reunião: 896 5101 4670 Senha de acesso: 729254</t>
+  </si>
+  <si>
+    <t>0011639-51.2026.5.03.0048</t>
+  </si>
+  <si>
+    <t>Santa Juliana Bioenergia Ltda</t>
+  </si>
+  <si>
+    <t>Julio Cesar Mulina</t>
+  </si>
+  <si>
+    <t>ARAXÁ</t>
+  </si>
+  <si>
+    <t>R$             144.023,89</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt.araxa</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Presencial</t>
+  </si>
+  <si>
+    <t>1001792-72.2025.5.02.0435</t>
+  </si>
+  <si>
+    <t>Ricardo Aparecido De Lima</t>
+  </si>
+  <si>
+    <t>11ª TURMA</t>
+  </si>
+  <si>
+    <t>R$             242.576,46</t>
+  </si>
+  <si>
+    <t>TAM</t>
+  </si>
+  <si>
+    <t>RFE</t>
+  </si>
+  <si>
+    <t>0010227-28.2025.5.15.0132</t>
+  </si>
+  <si>
+    <t>Alexandre Leite Da Silva</t>
+  </si>
+  <si>
+    <t>Inicial</t>
+  </si>
+  <si>
+    <t>R$             253.000,00</t>
+  </si>
+  <si>
+    <t>0010641-40.2026.5.15.0019</t>
+  </si>
+  <si>
+    <t>Viterra Bioenergia S.A.</t>
+  </si>
+  <si>
+    <t>Ricardo Francisco De Almeida</t>
+  </si>
+  <si>
+    <t>ARAÇATUBA</t>
+  </si>
+  <si>
+    <t>R$             227.571,64</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/83908076312?pwd=VnVGRnpYWFZmZjFwN3k4eVpnYTNSZz09 ID da reunião: 839 0807 6312 Senha de acesso: 248026</t>
+  </si>
+  <si>
+    <t>0010218-66.2025.5.15.0132</t>
+  </si>
+  <si>
+    <t>R$             140.841,42</t>
+  </si>
+  <si>
+    <t>ANB</t>
+  </si>
+  <si>
+    <t>0010555-69.2026.5.15.0019</t>
+  </si>
+  <si>
+    <t>Marcos Lima Moreira</t>
+  </si>
+  <si>
+    <t>R$             187.618,69</t>
+  </si>
+  <si>
+    <t>0001510-51.2025.5.12.0054</t>
+  </si>
+  <si>
+    <t>Pilkington Brasil Ltda.</t>
+  </si>
+  <si>
+    <t>Leonardo Jose Vivas Castillejo</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ</t>
+  </si>
+  <si>
+    <t>SC</t>
+  </si>
+  <si>
+    <t>03ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               42.832,25</t>
+  </si>
+  <si>
+    <t>https://trt12-jus-br.zoom.us/j/86949386199</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Telepresencial</t>
+  </si>
+  <si>
+    <t>0010813-79.2026.5.15.0019</t>
+  </si>
+  <si>
+    <t>Valdeir David De Souza</t>
+  </si>
+  <si>
+    <t>R$             144.381,80</t>
+  </si>
+  <si>
+    <t>0012756-50.2025.5.15.0025</t>
+  </si>
+  <si>
+    <t>Silmara Campos De Oliveira</t>
+  </si>
+  <si>
+    <t>BOTUCATU</t>
+  </si>
+  <si>
+    <t>R$             222.776,26</t>
   </si>
   <si>
     <t>Audiência Inicial -  Presencial</t>
   </si>
   <si>
-    <t>1001266-74.2026.5.02.0434</t>
-  </si>
-  <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Douglas Bernardo Santos</t>
-  </si>
-  <si>
-    <t>SANTO ANDRÉ</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>04ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$                     128.884,72</t>
-  </si>
-  <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>JPE</t>
-  </si>
-  <si>
-    <t>TAM</t>
-  </si>
-  <si>
-    <t>Presencial</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Telepresencial</t>
-  </si>
-  <si>
-    <t>0010455-22.2026.5.15.0082</t>
-  </si>
-  <si>
-    <t>Moema Bioenergia S.A. - Moema</t>
-  </si>
-  <si>
-    <t>Doralice Da Silva Ferreira</t>
-  </si>
-  <si>
-    <t>SÃO JOSÉ DO RIO PRETO</t>
-  </si>
-  <si>
-    <t>03ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$                     650.000,00</t>
-  </si>
-  <si>
-    <t>Grupo E2</t>
-  </si>
-  <si>
-    <t>MBF</t>
-  </si>
-  <si>
-    <t>CAL</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/81869084210?pwd=V0EwalRCY0V5ZFhUY0lCMEU1QVBJQT09 ID da reunião: 818 6908 4210 Senha de acesso: 306523</t>
-  </si>
-  <si>
-    <t>0010095-88.2026.5.15.0017</t>
-  </si>
-  <si>
-    <t>Tiago Firmino Dos Santos</t>
-  </si>
-  <si>
-    <t>01ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$                     238.000,00</t>
-  </si>
-  <si>
-    <t>RYL</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/81715388288?pwd=UFAwUGVFQkN1bGNXcStQUEovR2VZUT09</t>
-  </si>
-  <si>
-    <t>0010810-37.2026.5.03.0156</t>
-  </si>
-  <si>
-    <t>Itapagipe Bioenergia Ltda.</t>
-  </si>
-  <si>
-    <t>Miguel Oliveira Braz</t>
-  </si>
-  <si>
-    <t>FRUTAL</t>
-  </si>
-  <si>
-    <t>MG</t>
-  </si>
-  <si>
-    <t>Ação de Consignação em Pagamento</t>
-  </si>
-  <si>
-    <t>R$                       10.795,94</t>
-  </si>
-  <si>
-    <t> MBF</t>
-  </si>
-  <si>
-    <t>https://trt3-jus-br.zoom.us/my/vtfrutal</t>
-  </si>
-  <si>
-    <t>Audiência Inicial - Telepresencial</t>
-  </si>
-  <si>
-    <t>0010592-67.2026.5.15.0061</t>
-  </si>
-  <si>
-    <t>Viterra Bioenergia S.A.</t>
-  </si>
-  <si>
-    <t>Tiago Gomes Dos Santos</t>
-  </si>
-  <si>
-    <t>ARAÇATUBA</t>
-  </si>
-  <si>
-    <t>02ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$                     232.079,12</t>
-  </si>
-  <si>
-    <t>RRU</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/85968854254?pwd=UkYxemkvazd5bU94Y2MrQWRZTFVJdz09 ID da reunião: 859 6885 4254 Senha de Acesso: 1234</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>1001761-88.2025.5.02.0035</t>
-  </si>
-  <si>
-    <t>Willian Marcelino</t>
-  </si>
-  <si>
-    <t>SÃO PAULO</t>
-  </si>
-  <si>
-    <t>35ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$                     573.120,80</t>
-  </si>
-  <si>
-    <t>GSM</t>
-  </si>
-  <si>
-    <t>BSO</t>
-  </si>
-  <si>
-    <t>0012042-69.2025.5.15.0032</t>
-  </si>
-  <si>
-    <t>Itw Ppf Brasil Adesivos Ltda.</t>
-  </si>
-  <si>
-    <t>Jose Victor Da Silva Pereira</t>
-  </si>
-  <si>
-    <t>CAMPINAS</t>
-  </si>
-  <si>
-    <t>R$                       13.880,81</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/89978823106?pwd=TlFNRkViSE1yUjJyWjUvY2hSd2lVUT09 ID da reunião: 899 7882 3106 Senha: 112233</t>
-  </si>
-  <si>
-    <t>Audiência Una - Telepresencial</t>
-  </si>
-  <si>
-    <t>0010690-03.2026.5.15.0045</t>
-  </si>
-  <si>
-    <t>Embraer S.A.</t>
-  </si>
-  <si>
-    <t>Carlos Ulisses De Almeida</t>
-  </si>
-  <si>
-    <t>SÃO JOSÉ DOS CAMPOS</t>
-  </si>
-  <si>
-    <t>R$                     111.462,89</t>
-  </si>
-  <si>
-    <t>Grupo B2</t>
-  </si>
-  <si>
-    <t>ANB</t>
-  </si>
-  <si>
-    <t>https://us02web.zoom.us/j/81965031150?pwd=OG5KcVh3WVFncjA5SWhDTDRrb3E2QT09 ID: 819 6503 1150 Senha: 351446 - Preposto: Correspondente - Hebert</t>
-  </si>
-  <si>
-    <t>Audiência de Conciliação - Telepresencial</t>
-  </si>
-  <si>
-    <t>0000469-73.2026.5.10.0861</t>
-  </si>
-  <si>
-    <t>Pedro Afonso Bioenergia Ltda.</t>
-  </si>
-  <si>
-    <t>Marizete Rodrigues Torres</t>
-  </si>
-  <si>
-    <t>GUARAÍ</t>
-  </si>
-  <si>
-    <t>TO</t>
-  </si>
-  <si>
-    <t>Conciliação</t>
-  </si>
-  <si>
-    <t>R$                         6.001,59</t>
-  </si>
-  <si>
-    <t>https://trt10-jus-br.zoom.us/j/6334644559</t>
-  </si>
-  <si>
-    <t>1001034-62.2026.5.02.0434</t>
-  </si>
-  <si>
-    <t>Guilherme Arenghi</t>
-  </si>
-  <si>
-    <t>R$                       31.203,97</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>1001188-78.2026.5.02.0467</t>
-  </si>
-  <si>
-    <t>Mahle Metal Leve S.A.</t>
-  </si>
-  <si>
-    <t>Rita De Cassia Da Silva</t>
-  </si>
-  <si>
-    <t>SÃO BERNARDO DO CAMPO</t>
-  </si>
-  <si>
-    <t>07ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Inicial</t>
-  </si>
-  <si>
-    <t>R$                       39.364,65</t>
-  </si>
-  <si>
-    <t>Grupo E1</t>
-  </si>
-  <si>
-    <t>Correspondente - Carlos Florian</t>
-  </si>
-  <si>
-    <t>TLI</t>
+    <t>0010992-15.2026.5.15.0083</t>
+  </si>
+  <si>
+    <t>Fabiano Benedito Ribeiro</t>
+  </si>
+  <si>
+    <t>R$             157.090,00</t>
+  </si>
+  <si>
+    <t>VCR</t>
   </si>
 </sst>
 </file>
@@ -903,11 +1101,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20669F14-8D00-4D50-8AA2-3B7681DDCFEF}">
-  <dimension ref="A1:R14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{196F33B3-08C0-41F4-8779-9AF243AC5467}">
+  <dimension ref="A1:R26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="130" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -963,15 +1180,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>105814</v>
+        <v>101561</v>
       </c>
       <c r="B2" s="5">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="C2" s="6">
-        <v>0.34722222222222221</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>18</v>
@@ -1019,39 +1236,39 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
-        <v>105813</v>
+        <v>99373</v>
       </c>
       <c r="B3" s="5">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="C3" s="6">
-        <v>0.375</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="I3" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="L3" s="7" t="s">
         <v>26</v>
@@ -1060,54 +1277,54 @@
         <v>27</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="P3" s="7" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="Q3" s="7" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="R3" s="8" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
-        <v>105500</v>
+        <v>105315</v>
       </c>
       <c r="B4" s="5">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="C4" s="6">
-        <v>0.3888888888888889</v>
+        <v>0.40972222222222221</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="L4" s="7" t="s">
         <v>26</v>
@@ -1116,54 +1333,54 @@
         <v>27</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="Q4" s="7" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
-        <v>104283</v>
+        <v>105046</v>
       </c>
       <c r="B5" s="5">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="C5" s="6">
-        <v>0.39583333333333331</v>
+        <v>0.40972222222222221</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="G5" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="7" t="s">
         <v>51</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="L5" s="7" t="s">
         <v>26</v>
@@ -1172,54 +1389,54 @@
         <v>27</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="O5" s="7" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="P5" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="R5" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>105811</v>
+      </c>
+      <c r="B6" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="Q5" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="R5" s="8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="4">
-        <v>104054</v>
-      </c>
-      <c r="B6" s="5">
-        <v>46265</v>
-      </c>
-      <c r="C6" s="6">
-        <v>0.40972222222222221</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>48</v>
-      </c>
       <c r="E6" s="7" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>26</v>
@@ -1228,110 +1445,110 @@
         <v>27</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="R6" s="8" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
-        <v>105877</v>
+        <v>104382</v>
       </c>
       <c r="B7" s="5">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="C7" s="6">
-        <v>0.54513888888888884</v>
+        <v>0.4236111111111111</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>18</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>24</v>
+        <v>78</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="M7" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="O7" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="Q7" s="7" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="R7" s="8" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
-        <v>104931</v>
+        <v>101611</v>
       </c>
       <c r="B8" s="5">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="C8" s="6">
-        <v>0.54861111111111116</v>
+        <v>0.43194444444444446</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="H8" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>79</v>
-      </c>
       <c r="K8" s="7" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>26</v>
@@ -1340,54 +1557,54 @@
         <v>27</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="O8" s="7" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="Q8" s="7" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="R8" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>101555</v>
+      </c>
+      <c r="B9" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0.4375</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="4">
-        <v>103266</v>
-      </c>
-      <c r="B9" s="5">
-        <v>46265</v>
-      </c>
-      <c r="C9" s="6">
-        <v>0.55555555555555558</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>83</v>
-      </c>
       <c r="E9" s="7" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>26</v>
@@ -1396,54 +1613,54 @@
         <v>27</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="Q9" s="7" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="R9" s="8" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
-        <v>103794</v>
+        <v>104422</v>
       </c>
       <c r="B10" s="5">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="C10" s="6">
-        <v>0.55555555555555558</v>
+        <v>0.45277777777777778</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>41</v>
+        <v>102</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>26</v>
@@ -1452,54 +1669,54 @@
         <v>27</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="O10" s="7" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>63</v>
+        <v>105</v>
       </c>
       <c r="Q10" s="7" t="s">
-        <v>63</v>
+        <v>105</v>
       </c>
       <c r="R10" s="8" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
-        <v>104623</v>
+        <v>105365</v>
       </c>
       <c r="B11" s="5">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="C11" s="6">
-        <v>0.5625</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>97</v>
+        <v>18</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>79</v>
+        <v>24</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="L11" s="7" t="s">
         <v>26</v>
@@ -1508,110 +1725,110 @@
         <v>27</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="O11" s="7" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="P11" s="7" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="Q11" s="7" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="R11" s="8" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
-        <v>105574</v>
+        <v>105375</v>
       </c>
       <c r="B12" s="5">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="C12" s="6">
-        <v>0.59722222222222221</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>106</v>
+        <v>45</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>108</v>
+        <v>20</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>110</v>
+        <v>22</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>111</v>
+        <v>23</v>
       </c>
       <c r="J12" s="7" t="s">
         <v>24</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>112</v>
+        <v>25</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="O12" s="7" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="P12" s="7" t="s">
-        <v>57</v>
+        <v>89</v>
       </c>
       <c r="Q12" s="7" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="R12" s="8" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
-        <v>105186</v>
+        <v>105389</v>
       </c>
       <c r="B13" s="5">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="C13" s="6">
-        <v>0.61111111111111116</v>
+        <v>0.46527777777777779</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>83</v>
+        <v>18</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>40</v>
+        <v>122</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>41</v>
+        <v>77</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="L13" s="7" t="s">
         <v>26</v>
@@ -1620,54 +1837,54 @@
         <v>27</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="P13" s="7" t="s">
-        <v>45</v>
+        <v>125</v>
       </c>
       <c r="Q13" s="7" t="s">
-        <v>46</v>
+        <v>80</v>
       </c>
       <c r="R13" s="8" t="s">
-        <v>47</v>
+        <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
-        <v>105634</v>
+        <v>105331</v>
       </c>
       <c r="B14" s="5">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="C14" s="6">
-        <v>0.68055555555555558</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>118</v>
+        <v>18</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>120</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>122</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>41</v>
+        <v>77</v>
       </c>
       <c r="J14" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="K14" s="7" t="s">
         <v>123</v>
-      </c>
-      <c r="K14" s="7" t="s">
-        <v>124</v>
       </c>
       <c r="L14" s="7" t="s">
         <v>26</v>
@@ -1676,32 +1893,711 @@
         <v>27</v>
       </c>
       <c r="N14" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="O14" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="P14" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="O14" s="7" t="s">
+      <c r="Q14" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="R14" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="P14" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="Q14" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="R14" s="8" t="s">
-        <v>47</v>
+    </row>
+    <row r="15" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>104242</v>
+      </c>
+      <c r="B15" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.49305555555555558</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="O15" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="P15" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q15" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="R15" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
+        <v>101265</v>
+      </c>
+      <c r="B16" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N16" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="O16" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="P16" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q16" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="R16" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>105778</v>
+      </c>
+      <c r="B17" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.5625</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N17" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="O17" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="P17" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="R17" s="8" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>102783</v>
+      </c>
+      <c r="B18" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.5625</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="O18" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="R18" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>99942</v>
+      </c>
+      <c r="B19" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M19" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N19" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="O19" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P19" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q19" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="R19" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>105069</v>
+      </c>
+      <c r="B20" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0.60069444444444442</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N20" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="O20" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="P20" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q20" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="R20" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="4">
+        <v>99870</v>
+      </c>
+      <c r="B21" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J21" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N21" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="O21" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P21" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q21" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="R21" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="4">
+        <v>105173</v>
+      </c>
+      <c r="B22" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N22" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="O22" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="P22" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q22" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="R22" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="4">
+        <v>102767</v>
+      </c>
+      <c r="B23" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N23" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="O23" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="P23" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q23" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="R23" s="8" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="4">
+        <v>105441</v>
+      </c>
+      <c r="B24" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C24" s="6">
+        <v>0.60555555555555551</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N24" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="O24" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="P24" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q24" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="R24" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="4">
+        <v>105847</v>
+      </c>
+      <c r="B25" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C25" s="6">
+        <v>0.625</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N25" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="O25" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P25" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="Q25" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="R25" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
+        <v>104977</v>
+      </c>
+      <c r="B26" s="5">
+        <v>46266</v>
+      </c>
+      <c r="C26" s="6">
+        <v>0.65277777777777779</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L26" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M26" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N26" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="O26" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P26" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q26" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="R26" s="8" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R2" r:id="rId1" xr:uid="{C9190C39-CA9A-4ABB-9C1C-AD98FA321DD5}"/>
-    <hyperlink ref="R3" r:id="rId2" xr:uid="{4F6A4EEF-8A6F-4ABE-94F7-BF81531B5040}"/>
-    <hyperlink ref="R5" r:id="rId3" display="https://trt15-jus-br.zoom.us/j/81869084210?pwd=V0EwalRCY0V5ZFhUY0lCMEU1QVBJQT09%20ID%20da%20reunião:%20818%206908%204210%20Senha%20de%20acesso:%20306523" xr:uid="{D27B1D90-2F74-4FD0-816F-6D7266A3F711}"/>
-    <hyperlink ref="R6" r:id="rId4" xr:uid="{834CC90E-942F-4E41-9C64-E740868A639C}"/>
-    <hyperlink ref="R7" r:id="rId5" xr:uid="{7796BE1C-FE79-41A2-9DD3-0810F9DFE1D0}"/>
-    <hyperlink ref="R8" r:id="rId6" display="https://trt15-jus-br.zoom.us/j/85968854254?pwd=UkYxemkvazd5bU94Y2MrQWRZTFVJdz09%20ID%20da%20reunião:%20859%206885%204254%20Senha%20de%20Acesso:%201234" xr:uid="{BB1C6E94-B4E6-47A8-BD57-424D8A4B9F57}"/>
-    <hyperlink ref="R10" r:id="rId7" display="https://trt15-jus-br.zoom.us/j/89978823106?pwd=TlFNRkViSE1yUjJyWjUvY2hSd2lVUT09%20ID%20da%20reunião:%20899%207882%203106%20Senha:%20112233" xr:uid="{F48BAFCE-0E97-4ADD-B998-EAF7F5138387}"/>
-    <hyperlink ref="R11" r:id="rId8" display="https://us02web.zoom.us/j/81965031150?pwd=OG5KcVh3WVFncjA5SWhDTDRrb3E2QT09%20ID:%20819%206503%201150%20Senha:%20351446%20-%20Preposto:%20Correspondente%20-%20Hebert" xr:uid="{341F6CF5-2499-4125-85AA-86BCB476064D}"/>
-    <hyperlink ref="R12" r:id="rId9" xr:uid="{EF469F9B-93A4-4F57-A5BB-A01CB60FCF84}"/>
+    <hyperlink ref="R2" r:id="rId1" display="https://trt15-jus-br.zoom.us/j/9973700634?pwd=dENDekhCNjFLekRnSExiTzhmK1VLdz09%20ID%20da%20reunião:%20997%20370%200634%20Senha:%20592209" xr:uid="{8D689261-A6BE-494D-9C3C-A54ACE6B562B}"/>
+    <hyperlink ref="R3" r:id="rId2" display="https://trt15-jus-br.zoom.us/j/82717131621?pwd=pODkGMMik6OAPMNpdT855vizOcYdKQ.1%20iD%20da%20reunião:%20827%201713%201621%20Senha:%20761332" xr:uid="{70B921AB-E3D1-4594-9320-9F10D6B32A82}"/>
+    <hyperlink ref="R4" r:id="rId3" display="https://trt2-jus-br.zoom.us/j/87449545935?pwd=wCgGe2V8ntb7v8A97BI4itvBX6i0Ya.1%20ID%20da%20reunião:%20874%204954%205935%20Senha%20de%20acesso:%20047941" xr:uid="{730BBD45-D7BD-4EC9-8257-F4BA3663EBFA}"/>
+    <hyperlink ref="R6" r:id="rId4" display="https://trt2-jus-br.zoom.us/j/83934068085?pwd=vsilyvu3m7bMldNPplkinUYQRGR2Xz.1%20ID%20da%20reunião:%20839%203406%208085%20Senha%20de%20acesso:%20359721" xr:uid="{C2EC9EAD-6678-4EF6-90BE-AEFBE0085A0D}"/>
+    <hyperlink ref="R7" r:id="rId5" xr:uid="{43731B18-E42F-46D2-8A68-CF18DB233278}"/>
+    <hyperlink ref="R10" r:id="rId6" xr:uid="{F12C266A-23D0-4642-8C4C-28A921164996}"/>
+    <hyperlink ref="R11" r:id="rId7" display="https://us02web.zoom.us/j/81757243738?pwd=UXAvdEpveHlrNU05M2ZsZnRrYy9Vdz09%20ID%20DA%20REUNIÃO:%20817%205724%203738%20SENHA:%20954332" xr:uid="{C4E791E1-5919-48B1-9A63-6CF826D68207}"/>
+    <hyperlink ref="R12" r:id="rId8" display="https://us02web.zoom.us/j/83352065501?pwd=Lzc2WUJGSVpVWmJyZjB3Y0NvUmJPZz09%20ID%20da%20reunião:%20833%205206%205501%20Senha%20de%20acesso:%20368465" xr:uid="{12460121-9F59-4D5B-A10A-07D590EC3A5E}"/>
+    <hyperlink ref="R13" r:id="rId9" xr:uid="{4DD08ADD-D135-4263-979E-6D8C2089F4FE}"/>
+    <hyperlink ref="R14" r:id="rId10" xr:uid="{CD24E493-B451-4B64-A644-902CDE18A4EB}"/>
+    <hyperlink ref="R16" r:id="rId11" display="https://trt2-jus-br.zoom.us/j/89651014670?pwd=FW0AFzyGa5XXc5LOiaXNalueDYjcGW.1" xr:uid="{2C9F0EDD-D834-4CB9-8061-0E56DF462839}"/>
+    <hyperlink ref="R17" r:id="rId12" xr:uid="{F3FB26E2-B13C-4E77-9C9F-08B878B92941}"/>
+    <hyperlink ref="R20" r:id="rId13" display="https://trt15-jus-br.zoom.us/j/83908076312?pwd=VnVGRnpYWFZmZjFwN3k4eVpnYTNSZz09%20ID%20da%20reunião:%20839%200807%206312%20Senha%20de%20acesso:%20248026" xr:uid="{6FD5EE01-87B2-4E0E-815B-1933C9C47DA8}"/>
+    <hyperlink ref="R22" r:id="rId14" display="https://trt15-jus-br.zoom.us/j/83908076312?pwd=VnVGRnpYWFZmZjFwN3k4eVpnYTNSZz09%20ID%20da%20reunião:%20839%200807%206312%20Senha%20de%20acesso:%20248026" xr:uid="{6BD86EEA-E27E-4433-9555-67EB5F2DEC2B}"/>
+    <hyperlink ref="R23" r:id="rId15" xr:uid="{7879208E-C822-4031-AE76-6F815C47568B}"/>
+    <hyperlink ref="R24" r:id="rId16" display="https://trt15-jus-br.zoom.us/j/83908076312?pwd=VnVGRnpYWFZmZjFwN3k4eVpnYTNSZz09%20ID%20da%20reunião:%20839%200807%206312%20Senha%20de%20acesso:%20248026" xr:uid="{AD29B6A5-5445-43F1-80DD-59DA7ECE936C}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>